<commit_message>
Map Data: Amended market plaza
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -13753,40 +13753,305 @@
       <c r="A318" s="5" t="n">
         <v>316</v>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Lingering-effect timing (neo1-4 audit): every retreat lock (Jaw Clamp, Sticky Nectar, Magma Ring, Spider Web, Mean Look, Scary Face, Clutch/Corner/Bear Hug/Spook...) placed by EITHER side was wiped at the end of the attacker's own turn, as were Screech/Crunch, Pursuit, Triggered Poison and Dark Tentacle; Lock-on and High-Speed Charge/Leek Jab/Rock Tackle locks expired before the owner's next turn; lowercased disabled-attack keys never matched; Freeze and Scary Face only stopped attacks aimed at the attacker (Leer-style); Spider Web/Mean Look had no lasting lock; Giant Wave/Crushing Earth disabled only one attack.</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>[03/10/2026] clear_neo1/2/3_flags_end_of_turn rewritten (protections expire on the owner's side, defender-held effects on the side whose turn ended, Screech by set turn); retreat_disabled left to Main; is_attack_disabled case-insensitive; skip_one_turn for 'can't use this attack next turn'; all attacks skip_one_turn for 'can't attack next turn'; until_benched effects retreat_locked / cant_attack_until_benched (cleared in clear_all_statuses); Scary Face/Leer/Tickling Vines use cant_attack_next_turn; attack_unusable_reason disables the attack row; Dark Tentacle enforced in get_valid_evolution_targets; Lock-on via boost_set_turn.</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="5" t="n">
         <v>317</v>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Engine gaps found in the neo/ecard audit: card_ops.discard_energy_from_pokemon left the card attached (Searing Flames, Dark Flame, Mega Flame, Twister, Lava Flow... put it in two places); text-parsed Special Conditions ignored every immunity Body (Immunity, Poison Resistance, Thick Skin, Clear Body...); card_ops.apply_status ignored Agility/Transparency; Pollen Shield, Light Wave, Charm, Armor Up and Dodge did nothing or the wrong thing; Growl/Negative Ion reduced any attacker after W/R; Sputter's power lock had no owner/end; Jaw Clamp-style 'can't be switched' never applied.</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>[03/10/2026] Energy is detached inside discard_energy_from_pokemon; apply_status_effect applies through card_ops.apply_status (reports 'unaffected'); apply_status checks status_immune + is_protected_from_effects during an attack and records Mirror Move statuses; effects status_immune / neo4_light_wave / neo_charm / neo_growl (calculate_final_damage, before W/R, source-tied) / neo4_armor_up (flip at KO time, until owner's next turn) / neo4_dodge (owner flips); goop_gas_expire_turn for Sputter; active_switch_locked() checked by force switch, self switch, gusts and switch attacks.</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Live: 6</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="5" t="n">
         <v>318</v>
       </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>neo1/neo2 attack audit: Flower Dance counted the opponent's Bellossom; Zzzap/Shockwave/Dust Devil were raw HP cuts; Sweet Scent healed by absolute side (CPU heads healed the player, player prompted on CPU's attack); Fin Slap/Sketch read the side-level last attack (any Pokemon, any turn); Sweep Away milled the bottom of the deck; False Swipe ignored W/R/PlusPower; Shockwave skipped its switch on tails; Belly Drum counters took PlusPower/Defender; Hyper Reverse/Poison Bite healed by computed not dealt damage; Pilfer/Magic Dust/Baton Pass/Energy Cycle CPU picks random or first; Sputter missing its 10 damage.</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>[03/10/2026] All rewritten per card text; Sketch copies the Defending Pokemon's last-turn attack via the per-attack record (new attacker_id) and execute_copied_attack; helpers r3_evolve_with, r3_choose_count, r3_cpu_best_condition, r3_pick_defender_energy; CPU uses benefit / dump / need pickers; Magic Dust via choose_special_condition.</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>Live: 10</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="5" t="n">
         <v>319</v>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>neo3/neo4 attack audit: Evolutionary Spore put evolutions in the HAND; Psychic Damage did damage not counters; Dark Flame/Devastate/Burning Flame went ahead without their Fire cost; Outrage (tails did 30, heads +30) and Raging Headbutt (+10) wrong; Explosive Evolution skipped its evolution on tails; Max Burst counted only the Defender's Energy; Call Back stole the card onto the attacker's Bench; Evolution Song and Light Wave unimplemented; Tusk Toss/Bubble Jump left an empty Active; Aerowing, Lightning Strike, Lava Flow, Rushing Flames, Ball of Flame, Sweet Kiss, Provoke, Searchlight, Fish Out, Mysterious Wing gave the player no choice or forced it; many CPU picks were first/lowest-HP; Water Slash hacked the card metadata; Perish Song ignored 'last turn'; Nap always healed 3.</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>[03/10/2026] Each handler follows the card text: real evolution path, counters, cost gates, coin tables; optional effects prompt the player and the CPU decides on KO / Energy surplus / value; snipe/gust/energy-removal/benefit pickers for CPU targets; Water Slash cost-aware with the ignore_resistance flag; Night Eyes turn stamp; Nap count from text.</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>Live: 26</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="5" t="n">
         <v>320</v>
       </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>ecard1/ecard2 attack audit: Charge Up never flipped and only found basic Energy; Stamp (ecard1) did nothing on tails; Super Psywave was damage not counters and always hit the Active; Earth Rift hit the Active for 30 and skipped the Bench; Skedaddle, Gigacrush, Shuffle Attack, Miracle Tail and Energy Kick dropped their printed damage; Energy Kick had attacker/owner choices swapped and damaged with no Bench; Energy Punch did damage on tails; Sleep Inducer (Drowzee) never flipped; Growth Spurt routed to ex5's Grass-only handler; Spore Evolution dropped Tools; Copy ignored its Energy requirement; many CPU picks were first-in-list.</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>[03/10/2026] Fixed per text; Copy routed to the ex10 energy-checked copy; Shuffle Attack reorders (r3_reorder_top); Miracle Tail offers all 5 conditions; Fire Blow 'any number' choice; Destructive Roar/Dual Burn/Energy Punch choices; CPU uses need/heal/snipe/gust/removal pickers.</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>Live: 11</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="5" t="n">
         <v>321</v>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>ecard3 audit: 15 attacks had no implementation at all (Bounce Off, Sudden Growth, Star Back, Warp Hole, Gift of Spite, Water of Evolution, Surprise Slash, Energy Recycle, Limited Delivery, Energy Heal, Assist, Sudden Swipe, Evil Eye, Blindside, Energy Plant); Retro Cave put the card on TOP of the deck and kept HP instead of damage; Electric Blast/Thunder Force used damage not counters, CPU always discarded; Energy Splash missing its 70; cards routed to later sets' handlers: Triple Smash (+20 not +10), Energy Burst (no coin), Signs of Evolution (searched Silcoon...), Collect Fire (attached 2), Eruption (any Energy), Aqua Trick/Freeze Solid (no coin), Foresight (5 cards), Kick Away (no damage), Drag Off (did nothing with no Bench / not optional), Discharge (30 not 40/heads), Murkrow's Call for Family (any Basic), Telekinesis (30 not 20), Roar (no coin), Metal Reversal (defender chose), Knock Over (forced).</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>[03/10/2026] New _register_r3_fixes() registered LAST: text-gated _r3_wrap wrappers (other cards with the same name fall through to the previous handler) with full handlers for every listed attack; Retro Cave / Electric Blast / Stone Crush / Energy Splash fixed in place; _ex6_call_for_family parses 'named X or Y'; execute_discharge per-heads parameter; execute_ex5_metal_reversal attacker chooses; ex6 Knock Over optional.</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="5" t="n">
         <v>322</v>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Text-parser / resolver gaps (neo/ecard): Curve Attack &amp; Burrow ('prevent all damage done BY ATTACKS to'), neo4 Leer &amp; Tickling Vines (no named target), Sudden Charge &amp; Shake (opponent switches), Attract (choose &amp; switch), Draining Cut ('a damage counter'), Rolling Thunder tails half, Spinning Head coin gate, Karate Chop ('reduced by'), Energy Cannon ('plus 10 damage for each'), Claw (no comma) all parsed nothing; ~35 coin-table / choice attacks (Mislead, Double Cross, Poison Needle Rush, Spinning Blow, Scatterbomb, Ice Cyclone, Needle Rush, Continuous Bite, Crushing Lava, Lightning Sphere, Metal Tail, Shadow Hand, Iron Fist, Dogpile, Super Eggsplosion, Charm, Burning Fang...) were mis-applied.</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>[03/10/2026] Parser rules added (no_damage wording, attack_block_any, extra force_switch wordings, self_switch coin context, 'a damage counter', Rolling Thunder); _normalise_damage_text for the resolver/estimator; the rest got dedicated _r3_wrap handlers.</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="5" t="n">
         <v>323</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>CPU attack valuation for neo1-4 / ecard1-3: the damage estimator misread board-scaled / table / conditional attacks (Black Fang, Max Burst, Rushing Flames, Burning Flame, Gentle Flames, Syncroblast, Dream Eater...) and ~90 utility attacks scored 0, so they were only used when nothing else was usable; per-set Flower Dance counted both sides, Sketch used the side-level record, Pilfer got a flat bonus.</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>[03/10/2026] _r3_estimate() in estimate_attack_damage_range (min/max/expected per formula); cpu_utility_attack_value extended with board-aware values for the neo/ecard utility attacks (heals, searches, evolutions, locks, prize-gated Mystery Plates, Perish Song KO...); per-set entries corrected.</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
       </c>
     </row>
     <row r="326">

</xml_diff>

<commit_message>
Debug: Made sure all Neo and EX cards were implemented and working to a basic level
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -14058,200 +14058,1400 @@
       <c r="A326" s="5" t="n">
         <v>324</v>
       </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>ex1/ex2 attack audit: choices the card offers were forced or decided by fixed CPU picks (Lizard Poison, Critical Move, Fire Stream, Dark Slash, Lure Poison, Metal Hook, Energy Call, Drizzle, Influence/Team Assembly, Haunt, Split Blast, Sniff Out...); Stockpile never expired; Rest/Signs of Evolution wrong; devolve could leave 1 HP; CPU deck searches took the first card in deck order.</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Round-4 shared helpers added at the end of Attack_Effects.gd (r4_pick_own_energy, r4_cpu_spend_energy, r4_would_ko, r4_energy_amount, r4_optional_gust, r4_cpu_wants_self_switch, _r4_copy_rank, r4_num...) and _register_r4_fixes (runs LAST). Player choices now prompt; CPU decides from KO / need / value. Card_Ops.search_deck_to_hand CPU ranks by keep value. Debug: ISSUE #324 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="5" t="n">
         <v>325</v>
       </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Cross-set attack-name collisions: a later set's handler for the same attack name used another card's numbers/effect (Gigashock, Plus Energy, Energy Catch, Flame Pillar, Kerzap, Leaf Poison, Slashing Strike, Recharge, Shock Bolt, Energy Bomb, Shakedown, Dark Fire, Brick Smash, Energy Draw, Explosive Evolution, Volcanic Ash, Black Magic, Sweet Scent, Flames of Rage, Fury Cutter, Cry for Help, Self Charge, Kindle, Hyper Whirlpool, Call for Friends/Family, Attract Current).</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Text-gated overrides in _register_r4_fixes (r3_wrap / r4_wrap_if) read each card's own text; other printings fall through to the previous handler. Debug: ISSUE #325 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="5" t="n">
         <v>326</v>
       </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>'You may switch' self-switch attacks always switched (player) or never switched (CPU).</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>apply_self_switch(..., optional) — player is asked; CPU uses r4_cpu_wants_self_switch (KO danger / badly hurt / Special Condition and a better Bench option). Parser adds 'optional' for 'you may switch'. Debug: ISSUE #326 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="5" t="n">
         <v>327</v>
       </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>ex3 attack audit: Energy Shower, Pick On, Dragon Dew, circuit snipes, Damage Curse/Double Metal Ball (damage not counters), Power Generation, Quick Charge, Energy Stream, Spiral Growth, Backspin, Quick Touch, Dragon Crush, Quick Dive, Dragon Wave, Mist Ball, Dragon Burst, Lava Flow — forced choices / naive CPU picks.</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Player choices + KO-aware CPU picks; counters use gym1_place_counters; 'Energy amount' uses r4_energy_amount. Debug: ISSUE #327 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="5" t="n">
         <v>328</v>
       </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>ex4 attack audit: Miracle, Crushing Magma, Knock Over, Hydro/Aqua Reverse, Land Stream, Magma Burn, Hot Air, Dark Poison, Flame Ball, place-counter attacks, Energy Flip, Crushing Wave, Miracle Powder/Essence, Pick and Choose — forced choices / fixed CPU picks / damage instead of counters.</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Choices prompt; CPU picks smart (r3_cpu_best_condition etc.); _ex4_put_counter places counters. Debug: ISSUE #328 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="5" t="n">
         <v>329</v>
       </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>ex5 attack audit: Darkness Chant, Flutter Trick, Mass Destruction (ignored protection), Make a Wish/Ascension, Push Aside, Chime, Sunshine, Forecast, Silver Wind (bonus never expired), Scattered Shower, Coral Glow, Sweet Temptation, Intense Glare, Minus Energy, Heavy Blizzard, Crushing Mantle, Super Tidal Wave, Tonnage, Ice/Steel Generator.</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Silver Wind data {bonus,turn} applied only on turn+2; all choices prompt / CPU smart. Debug: ISSUE #329 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="5" t="n">
         <v>330</v>
       </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>ex6 attack audit: Salt Water, Psychic Exchange ('up to'), Signs of Evolution, Thunder Reflection &amp; Crush and Burn (CPU stubs), Hoard, Speed Shot, Toss, Vine Tease, Energy Powder, Pickup, Burn Down, Breakdown.</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Implemented CPU logic for the stubs; choices prompt; counters placed as counters. Debug: ISSUE #330 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="5" t="n">
         <v>331</v>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>ex7 attack audit: Dark Link/Rainbow Moves/Mimicry/Skill Hack copy picks, Hard Bone, Spread Poison, Litter, Souvenir, Quick Change, Quick Tail Smash, Aqua Trick, Dump and Draw, Friend Search, Dark Aid, Darkness Switch (protection), Fire Dance, Rotating Claws, Raging Thunder, Snatch and Run.</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>_r4_copy_rank for copy attacks (payable, damage, KO); rest smart CPU / player choice. Debug: ISSUE #331 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="5" t="n">
         <v>332</v>
       </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>ex8 attack audit: Luring Antenna (forced gust), Hustle Punch duration, Back Burner, multi-snipe, Powerful Hand, Healing Steps, Foresight (stub), Magnetic Tackle, Reflected Beam, Mid-air Crush (no W/R on Active, wrong chooser), Psyburst, Darkness Blast.</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Optional gust via r4_optional_gust; Foresight uses r3_reorder_top; choices fixed. Debug: ISSUE #332 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="5" t="n">
         <v>333</v>
       </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>ex9 attacks + Swift-type attacks: Power Short, Shadow Beam (Energy amount); Dragon Mist/Fastwave/ex5 Brick Smash/Speed Shot/Burn Down ignored Weakness rules.</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>execute_swift(..., apply_weakness) — 'isn't affected by Resistance...' attacks keep Weakness. Debug: ISSUE #333 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="5" t="n">
         <v>334</v>
       </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>ex10 attack audit incl. Unown Hidden Powers (B, C, D, E, G, H, I, J, K, L, M, Q, S, U, W, !), Elemental Blast, Bouncy Move, Derail, Healing Milk, Night Song, Pop, Push Away, Time Trap (stub), Miraculous Thunder, Spider Trap, Standing By (never expired), Upward Lick, Aqua Supply.</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>All choices player/CPU-smart; Standing By expiry added to the boost list in Trainer_Effects. Debug: ISSUE #334 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="5" t="n">
         <v>335</v>
       </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>ex11 attack audit: Holon searches, multi-snipe, Recover, Psychic Rage, Energy Bone, Delta Crush, Return Burn/Spark/Wave, Type Match, Delta Fang ('can't attack' only blocked attacks on the attacker), Psychic Option, Glide (never expired), Disable, Pickup Power.</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>cant_attack_next_turn effect; CPU decisions spend Energy only when it pays; Glide expiry. Debug: ISSUE #335 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="5" t="n">
         <v>336</v>
       </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>ex12 attack audit: target choice CPU, Stretch Claws, Reactive Blast ('any number'), Devolution Wave (cards went to hand not deck), Entangling Vines, Flame Swirl, Flick Poison, Power Move &amp; Tripping Turn (CPU never switched), Return Trance.</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Fixed per card text; optional switches use the shared helper. Debug: ISSUE #336 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="5" t="n">
         <v>337</v>
       </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>ex13 attack audit: Fossil Charge/Metallic Thunder/Devo Crush (CPU always paid the cost), Spiral Growth, Paste, Deceive (raw HP cut), Delta Draw ('up to'), Mind Play &amp; Brush Aside (random instead of the player's blind pick; Brush Aside flipped a coin it doesn't have).</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>CPU pays costs only for a KO / spare Energy; blind picks via _pick_blind_from_hand; Deceive places counters. Debug: ISSUE #337 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="5" t="n">
         <v>338</v>
       </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>ex14 attack audit: Mining (CPU never attached the Tool), Ultra Pump (CPU always discarded), Leaf Shade, Skill Copy (first card), Drag Off (always gusted), Tail Whip (only blocked attacks on Wartortle), Even Game ('up to' ignored cancel), Call-for-Pokemon CPU picked highest HP; Shield Beam also shut off Poke-Bodies and missed newly benched Pokemon.</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Shield Beam is now a side-wide Powers-only lock (main.shield_beam_lock_*), cleared at end of that side's turn. ULTRA_PUMP_CPU_JUNK_VALUE = 35. Debug: ISSUE #338 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="5" t="n">
         <v>339</v>
       </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>ex15 attack audit: Grind (Energy amount), Dig Deep, Dark Horn (CPU always discarded), Trick Tail, Delta Mind &amp; Dragon Roar (raw HP instead of counters), Power Crush, Dual Stream (CPU always split), Electromark, Shock-wave.</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Counters via gym1_place_counters; CPU choices KO/threat aware. Debug: ISSUE #339 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="5" t="n">
         <v>340</v>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>ex16 attacks: Rock Blast and Hydro Wave left discarded Energy still attached (in discard AND on the Pokemon); Dark Swirl milled the BOTTOM of the deck; Mix-Up refreshed the wrong deck icon; Electabuzz Power of Evolution drew from the top (should be bottom); Mantine Power Circulation put the card on the bottom; Rock Blast CPU dumped all Fighting Energy.</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>discard_energy_from_pokemon used; deck top = array FRONT throughout. Debug: ISSUE #340 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="5" t="n">
         <v>341</v>
       </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>pop attacks: Critical Crush/Fire Spin discarded the first 2 basics (no choice), Power/Body Bolt CPU lowest HP, Extra Draw CPU took first 2 Energy.</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Owner picks the Energy; CPU smart. Debug: ISSUE #341 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="5" t="n">
         <v>342</v>
       </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Generic-parser gaps: Star Pokemon names never matched their text ('Torchic Star'); Strike and Run, Pollen Hazard, Headache (ex7), Extra Curse, Shatter, String Pull, Metal Burn, Speedy Uppercut, Power Heal, Delta Reduction (ex13/ex15) parsed nothing or the wrong thing; extra-Energy resolver missed Metal/Darkness; Hyper Pump counted Special Energy.</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Name normalisation ★-&gt;star; wrappers in _register_r4_fixes; pre-W/R self-reduction effect r4_pre_wr_reduction in calculate_final_damage. Debug: ISSUE #342 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="5" t="n">
         <v>343</v>
       </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>ex1 powers: Firestarter/Water Call/Psy Shadow CPU targets naive (Psy Shadow always the Active); Energy Draw always drew 3 ('up to') and left the discarded Energy in the hand; Drive Off used every turn (even to cure the player's Active).</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Fixed; PSY_SHADOW_CPU_HP_MARGIN = 30. Debug: ISSUE #343 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="5" t="n">
         <v>344</v>
       </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>'Prevent all effects of attacks' Bodies/effects (Safeguard, Wonder Guard, Holy Shield, Fast Protection, Beacon/Extra/Reactive Shield, Solid Shell, Psychic Shield, Advanced Armor, ex Shield, Mysterious Shard, Protective Dust, Crystal Body, Darkness Veil, Dragon Aura, Jynx Stages of Evolution, Reactive Barrier, Holon Energy WP) only stopped damage / Special Conditions — gusts, Energy removal, counters, can't-attack still landed.</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Attack_Effects.r4_attack_effect_shield() folded into is_protected_from_effects (judged against the attack in progress). Base Drag Off still damages when only the switch is prevented. Debug: ISSUE #344 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="5" t="n">
         <v>345</v>
       </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>ex2/ex3 powers: Baby Evolution never matched Tyrogue's 3 names or δ evolutions; Fan Away CPU took the first Energy; Chaos Flash used on Confused targets; Energy Protection/Jagged Stone gates; Power Pinchers applied after W/R; Dragon Wind gusted every turn; Magnetic Field left the discarded card in hand; Call for Power stripped every Energy on the board onto Dragonite ex; Loose Shell bench limit.</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>r4_cpu_gust_choice shared gust decision; Call for Power moves only what Dragonite needs. Debug: ISSUE #345 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="5" t="n">
         <v>346</v>
       </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>ex4 powers: Power Shift moved ALL basic Energy ('any number'); CPU never used Power Shift / Magma Switch; Overheat/Auxiliary Light used every turn regardless of need.</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>New shared CPU Energy-move planner r4_cpu_plan_energy_moves (only moves that reduce an attack's unmet cost). Debug: ISSUE #346 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="5" t="n">
         <v>347</v>
       </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>ex5 powers: Metal Juncture &amp; Temperamental Weather never used by CPU; Crush Draw always onto Walrein; Heal Dance first target; Energy Grounding auto-picked/no decline; Healing Shower CPU used it even when it only healed the player; Castform/Form Change HP floored at 1 instead of KO.</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Fixed; form-switch powers use _r4_cpu_best_castform / _r4_cpu_best_form. Debug: ISSUE #347 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="5" t="n">
         <v>348</v>
       </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>ex6 powers: Form Variation CPU picked highest HP (even ones the damage KOs); Strange Behavior &amp; Energy Rain never used by CPU; Assistance removed ALL Special Conditions (text: 1); Extra Energy Bomb CPU fired freely (gives 2 Prizes) and dumped all Energy on the Active; Legendary Ascent auto-switched and pulled every matching Energy.</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Fixed; STRANGE_BEHAVIOR_CPU_HP_FLOOR = 30. Debug: ISSUE #348 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="5" t="n">
         <v>349</v>
       </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>ex7 powers: Dark Trance never used by CPU and player couldn't pick which Darkness card; Dark Spell/Ripples CPU picks naive.</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Planner + smart targets. Debug: ISSUE #349 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="5" t="n">
         <v>350</v>
       </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>~18 Bodies/Tools printed '(before applying Weakness and Resistance)' were applied after W/R (Intimidating Fang, Hunch, Lazy Aura, Intimidating Pattern, Vigorous Aura, Blaze, Hitmonlee Stages, Danger Perception, Reversal Aura +20, Ancient Fang, Paranoid, Delta Reactor, Water Pressure, Battle Aura, Extra Feather, Extra Smoke, Solid Rage).</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Powers_And_Bodies.run_pre_wr_hooks called from calculate_final_damage before W/R; those hooks are no-ops outside the pass. Intimidating Fang / Reversal Aura read their own wording (Granbull is 'after'). Debug: ISSUE #350 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="5" t="n">
         <v>351</v>
       </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>ex8 powers: Magnetic Reversal let the OPPONENT pick the Benched Pokemon; Wishing Star CPU took the top card; Super Connectivity CPU fed the Active every turn; Form Change CPU never used / first card; Smooth Over, Fan Action, Magnetic Reversal, Wishing Star never used by CPU; Distortion lowest HP; Lightning Burst always switched; Dragon Boost ignored need; Sunbeam floored HP at 1.</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Fixed. Debug: ISSUE #351 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="5" t="n">
         <v>352</v>
       </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>ex9 powers: the ex9 Heal Dance handler replaced ex5's and dropped the once-per-turn-across-Heal-Dance rule (Bellossom + Gardevoir both fired); Water Cyclone never used by CPU.</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Shared heal-dance flag; Water Cyclone rescues Energy off a doomed Active. Debug: ISSUE #352 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="5" t="n">
         <v>353</v>
       </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>ex10 powers: Darker Ring let the opponent pick the Benched Pokemon; Silver Sparkle/Golden Wing took the first Energy/target; Makeover &amp; Snappy Move never used by CPU; Snappy Move/Shuffle ignored Power shutdowns; Nurture and Heal/Bursting Up CPU targets.</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Fixed. Debug: ISSUE #353 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="5" t="n">
         <v>354</v>
       </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>ex11 powers: Power-ready helper ignored Toxic Gas-style locks; Delta Charge/Crush Draw CPU fewest-Energy target; Energy Jump, Duplicate, Delta Switch never used by CPU; Delta Control first Pokemon; Duplicate floored HP at 1; Evolutionary Swirl always fired and forced 4 draws ('up to').</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>EVOLUTIONARY_SWIRL_CPU_MIN_HAND = 5. Debug: ISSUE #354 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="5" t="n">
         <v>355</v>
       </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Abilities vs Special Conditions: every Poke-BODY switched off while its holder was Asleep/Confused/Paralyzed (ex-era Bodies keep working); 'can't be used if affected by a Special Condition' Poke-Powers ignored Poisoned/Burned; Powers-only locks (Lazy, Stench, Wise Aura, Rear Sensor, Sol/Luna Shade, Dark Gaze, Delta Reserve, Black Cry, Holon Legacy, Extra Liquid, Intimidating Ring, Dark Impact) also shut off Bodies.</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>r4_ability_is_body_only / r4_status_blocks_ability in is_power_blocked(_by_status); [P] locks skip body-only Pokemon. Debug: ISSUE #355 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="5" t="n">
         <v>356</v>
       </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>ex12 powers: Reactive Shift never used by CPU; Nectar Pod gusted every time; Shady Move CPU always own-most-damaged -&gt; player Active; Emerge Charge first Energy / no decline; Shadow Curse lowest HP; Reactive Recharge fewest Energy; ex12 phase announced Baby Evolution with nothing in hand; Reactive Protection/Ancient Shell/Pattern Distraction ignored Body locks.</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Fixed. Debug: ISSUE #356 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="5" t="n">
         <v>357</v>
       </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>ex13 powers: Delta Supply CPU first Energy -&gt; Active; Dragon Curse lowest HP; Splash Back most-Energy only; Driving Howl used every turn.</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Fixed. Debug: ISSUE #357 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="5" t="n">
         <v>358</v>
       </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>ex14 powers + deck ends: Excavate looked at the BOTTOM card; Peal of Thunder looked at the bottom 5; Time Travel put Celebi Star on TOP; PokeNav looked at the bottom 3 and never let you order the rest; Spike Storm lowest HP; Delta Transport CPU rule; Hard Rock counted cards not Energy.</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Deck top = array front everywhere. EXCAVATE_CPU_DISCARD_BELOW = 40. Debug: ISSUE #358 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="5" t="n">
         <v>359</v>
       </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>ex15 powers: Dig Up CPU first Tool / no decline on first pick; Tropical Heal fired with nothing to remove; Dozing never used by CPU; Mantine Power Circulation HP margin.</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Fixed. Debug: ISSUE #359 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="5" t="n">
         <v>360</v>
       </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>ex16/pop powers: Crimson/Yellow/Blue/Purple Ray ('you may', hit BOTH Actives) always fired; Dark Ray was random for the player; Time Reversal CPU first Pokemon; Cursed Eyes CPU moved counters off the most-damaged Pokemon; Magnetic Redraw only on small CPU hand.</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>_r4_ray_wanted: player asked, CPU only when it comes out ahead. Debug: ISSUE #360 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="5" t="n">
         <v>361</v>
       </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Trainer Effect</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>ex/pop Trainers: POW! Hand Extension CPU could never choose 'move Energy' and moved the first Energy; Surprise! Time Machine / Swoop! Teleporter / Holon Transceiver / Holon Fossil / Pokemon Retriever / Rocket's Mission / Venture Bomb / Life Herb / Great Ball / team-bench Trainers used first-in-list or highest-HP CPU picks.</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>_r4_cpu_best_basic + keep-value / gust-choice decisions. Debug: ISSUE #361 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="5" t="n">
         <v>362</v>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Special Energy damage never applied: Darkness Energy (+10), R Energy (+10), Double Rainbow Energy (-10), Metal Energy (-10 taken / -10 dealt by non-Metal on old printings) — the modifier functions had no callers. ex8/ex15 Strength Charm also applied after W/R.</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Special_Energy_Effects.r4_energy_damage_mod called pre- and post-W/R per each printing's text and type condition. Debug: ISSUE #362 prints/comments.</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="5" t="n">
         <v>363</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Enervating Pollen (ecard2-49 Gloom): Resistance should only reduce damage by 10; it reused the Resistance Gym math (-20 Resistance became 0).</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Resistance capped at -10 while any Gloom with Enervating Pollen is in play. Found by the full-game coverage sweep. Debug: ISSUE #363.</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
       </c>
     </row>
     <row r="366">

</xml_diff>

<commit_message>
Debug: Fixed over 100 incorrect attack/trainer/power effects
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J372"/>
+  <dimension ref="A1:J376"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -1662,11 +1662,7 @@
       <c r="H22" s="8" t="n">
         <v>46221</v>
       </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>Live: 2</t>
-        </is>
-      </c>
+      <c r="J22" s="7" t="n"/>
     </row>
     <row r="23" ht="43.35" customHeight="1">
       <c r="A23" s="5" t="n">
@@ -7312,11 +7308,6 @@
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr">
-        <is>
-          <t>Live: 1</t>
-        </is>
-      </c>
     </row>
     <row r="160" ht="30" customHeight="1">
       <c r="A160" s="5" t="n">
@@ -12453,11 +12444,6 @@
           <t>03/09/2026</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr">
-        <is>
-          <t>Live: 1 (REMOVE)</t>
-        </is>
-      </c>
     </row>
     <row r="285" ht="43.2" customHeight="1">
       <c r="A285" s="5" t="n">
@@ -14088,6 +14074,11 @@
           <t>04/10/2026</t>
         </is>
       </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>Live: 5</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="5" t="n">
@@ -14123,6 +14114,11 @@
           <t>04/10/2026</t>
         </is>
       </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="5" t="n">
@@ -14158,6 +14154,11 @@
           <t>04/10/2026</t>
         </is>
       </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="5" t="n">
@@ -14263,6 +14264,11 @@
           <t>04/10/2026</t>
         </is>
       </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="5" t="n">
@@ -14578,6 +14584,11 @@
           <t>04/10/2026</t>
         </is>
       </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="5" t="n">
@@ -14858,6 +14869,11 @@
           <t>04/10/2026</t>
         </is>
       </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="5" t="n">
@@ -15458,35 +15474,440 @@
       <c r="A366" s="5" t="n">
         <v>364</v>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Card text says CHOOSE but the game picked at random (or auto-picked): Texture Magic, Paint, Shakedown / Knock Off ("without looking"), Bad News (several cards without looking), Prize Shift (face-down Prize), Card-Flip Game (opponent's Prize), Unown [Search], Unown [Tell].</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Blind picks now go through _pick_blind / new _pick_blind_many_from_hand (the chooser picks face-down cards on one screen); Prize Shift uses _choose_face_down_prize; Card-Flip Game shows the chosen Prize face up; [Search]/[Tell] use show_cards. Debug: ISSUE #364 prints.</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>Live: 7</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="5" t="n">
         <v>365</v>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>"You may" effects forced, and mandatory effects made optional: Warp/Cyclone Energy, Froth, Evolutionary Flame/Thunder/Swirl, Chilling Breath, Energy Recharge, Flame Vapor, Cunning, Unown [Give]/[Help]/[Want], Impostor Oak's Invention, Thought Wave Machine, Personality Test, Evil Deeds, Engage, Gold Scale, Conversion 1, Buzzap / Shift type lists, Fossil Egg.</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Warp/Cyclone Energy mandatory + Active only (both sides). New _r4_power_may(holder, opp, title, question, cpu_wants) asks the player / lets the CPU decide. Unown words check the Bench requirement; [Give] lets the player pick the Energy. Conversion/Buzzap gained Darkness + Metal; Buzzap/Shift show an Energy image per type. Fossil Egg asks deck or hand. Debug: ISSUE #365 prints.</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>Live: 11</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="5" t="n">
         <v>366</v>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Trainer Effect</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>"Up to" / exact counts wrong in prompts and draw counts: Energy Conversion, Growth, Energy Absorption, Energy Retrieval, Steel Generator, Double Attack, Hidden Power, Critical Collection, Devolution Wave, Sonic Signal, Computer Error, Rocket's Trap, Energy Charge, Desert Shaman, Steven's Advice, Rocket's Admin., Psychic Exchange, Super Energy Removal, Town Volunteers, Fisherman, Speed Growth, Extra Draw, Reflected Sunlight, Water Plant, Magnetic Field, Wildfire.</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Prompt minimums fixed (min 0 for "up to", exact where the text is exact); draw counts use choose_up_to_draw_count; Super Energy Removal no longer auto-picks with 2 attached; Wildfire is one screen and checks Confusion. Debug: ISSUE #366 prints.</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>Live: 5</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="5" t="n">
         <v>367</v>
       </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>"Look at" effects never showed the cards: the opponent's hand (Bursting Hand, Rob, Threaten, Push Away, Eerie Howl, Scam, Supernatural, Flutter Trick, Push Aside, Poltergeist, Psyscan, Glaring Gaze, Carry Off, Sharing, Sneak Attack, Unown E, Skill Hack, Provoke) and looked-at deck/prize cards (Master Ball family, PokéGear, Friend Search, Arcade Game, Seer, Spy, Baby Outing, Forest Guardian, Radio Tower, Vine Tease, Look for Friends, Fast Ball, Flipper Stroke, [Observe], Investigate, Peal of Thunder, Holon Lass). Reorder prompts missing: Underground Expedition, PokéNav, Delta Control.</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>New helpers: Attack_Effects._reveal_opp_hand, Card_Ops.pick_from_looked_at (all looked-at cards shown, eligible ones selectable) and Card_Ops.show_cards. Flutter Trick also now removes the card from hand. Reorders use prompt_reorder_cards. Debug: ISSUE #367 prints.</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>Live: 7</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="5" t="n">
         <v>368</v>
       </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Energy discarded/moved by an attack was auto-picked instead of the owner choosing: Continuous Fireball, Flames of Rage, Scavenge, Flame Wheel, Devastate, Burning Flame, Fire Blow, Elemental Blast (neo1), Plasma, Afternoon Nap, Energy Control, Jet Stream, Magnetic Flow, Streaming Mantle, Burning Sludge.</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Owner picks through pick_own_energies / r4_pick_own_energy (CPU uses cpu_own_energy_discard_order). Continuous Fireball also checks Confusion; Energy Control is basic-only with a choice; Burning Sludge goes through apply_status. Debug: ISSUE #368 prints.</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="5" t="n">
         <v>369</v>
       </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Evolve/devolve effects bypassed the real evolution path (no evolution triggers, wrong card stacking): Energy Evolution, Hatch, Evolution Helper, Star Piece, Hyper Devolution Spray.</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Routed through r3_evolve_with / _ex2_devolve_pokemon. Star Piece is mandatory per its text. Debug: ISSUE #369 prints.</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>Live: 5</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="5" t="n">
         <v>370</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Attack Effect</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Attack text mismatches: Delta Draw / Paste / Delta Call had no Confusion check; Metal Pincer; Comet Punch neo1-63 damage; Tentacle Wrap tails (+1 retreat) missing; Poison Bind lock; Cat Punch target chooser; Super Metronome could only copy the Defending Pokémon; Strange Scent counters; Squirt / Tongue Stretch / Sharpshooter applied Weakness/Resistance to Benched targets.</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Metal Pincer uses r3_flip_until_tails_plus; neo1-63 JSON damage "10×"; Tentacle Wrap sets neo4_tentacle_wrap (read in get_retreat_cost); Poison Bind sets jaw_clamp_locked; Cat Punch: defender chooses; Super Metronome copies any opposing Pokémon via execute_copied_attack; Strange Scent: player places each counter; bench snipes use hit_no_wr + CPU snipe targeting. Debug: ISSUE #370 prints.</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>371</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Trainer Effect</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Trainer/Energy/attack text not implemented as written: EXP.ALL, Magnifier, Old Darkness Energy counter, Rainbow Energy types, Multi Energy, Breeder Fields, Energy Ark, Island Hermit, ex Pokémon Reversal (who chooses), Lava Flow, Belly Drum, Type Change, Legendary Body, Hard Cocoon / Sand Guard result, Even Game, Octazooka, Pull In, Flame Pillar, Super Energy Retrieval, Tropical Tidal Wave.</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>EXP.ALL is a pre-KO hook; Magnifier skips Resistance and is discarded at end of turn; Old Darkness Energy counter between turns; Rainbow = all 8 types; Multi Energy goes Colorless with another Special attached; Island Hermit turns Prizes face up (prize_face_up); new effect_ex_pokemon_reversal(opp, opponent_chooses); Octazooka persistent until benched; Legendary Body blocks removal + discards attached Trainers. Debug: ISSUE #371 prints.</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>Live: 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>372</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Hidden-card selection screens hid face-up copies (Array == compares contents); Night Vision / Psychic Vision / [Tell] didn't show the hand; Back Burner minimum; Bounce / Retro / Miracle / Crystal Energy provided nothing (never implemented); Power Gene applied after Weakness/Resistance.</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>should_hide uses is_same() for the opponent hand / Prize piles. Special Energies implemented in Special_Energy_Effects (types, can_attach_to, on-attach; Miracle discarded end of turn; Crystal resolved per holder in Main). _ex2_devolve_pokemon gained a "discard" destination. Power Gene: the existing hook now runs in the pre-W/R pass (duplicate hook removed). Debug: ISSUE #372 prints.</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>Live: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>373</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Prioritisation</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Opponent turn should play like a person: Bill before Professor Oak, hand-replacing draws only after everything else, draw Supporters valued on real cards drawn, Stage 2 lines kept, spare Energy discarded before needed Energy, smart retreats (not back-and-forth, shed Confusion, retreat into a KO), take KOs (game-winning / 2-Prize), status attacks timed to the board without endless stalling, Damage Swap + Pokémon Center stall, Scoop Up on big-HP Pokémon at low HP, synergy pieces held, activated Powers the CPU never used.</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>New HUMAN-PLAY LAYER in CPU_AI: CPU_DRAW_CARDS model + _cpu_score_draw_card; cpu_score_trainer_for_play holds Oak/Elm/Gambler/Copycat/etc. by phase (early/mid/late) unless the hand is stuck; after a late draw the CPU evolves/benches/attaches again. Discard priority uses cpu_evolution_line_state + cpu_hand_energy_keep. cpu_scoop_value / cpu_pick_scoop_target drive Scoop Up, Super Scoop Up, Mr. Briney, [Undo]. _cpu_attack_context_adjust (win/2-Prize KO bonus, Paralysis/Sleep when their attack would KO us, Poison on big HP, stall guard via cpu_no_damage_streak, defensive "prevent all damage" attacks). Retreat: status-escape reason, no consecutive offensive retreats, retreat into a bench Pokémon that KOs. Switch valued for Paralysis/Sleep. Gust stall target, Energy Removal via cpu_removal_delays_attack, heal items only when they rescue (_cpu_score_heal_item), Pokémon Center vs Energy lost, Damage Swap parks counters on safe Energy-free sponges. cpu_decision_override filled (Rare Candy/Breeder with a live Stage 2, DCE, Pokémon Center + Damage Swap, Rain Dance Water...). Energy Search / Lady Outing / Mr. Stone scored on need; Fossils scored on their evolution; TM 01s scored. cpu_phase_human_powers uses Type Shift / Eclipses / Submerge (Weakness), Energy Converter, Cunning, [Join], [Give], [Want], [Help], [Quicken], [Undo], Spatial Distortion, Prize Shift, Final Sting, Energy Recycle + Fellow Boost (final check only, end the turn). Face-up Prizes taken on purpose. Bench cap respected (Narrow Gym / Giant Stump). Rules fixes found on the way: Super Scoop Up returns ALL attached cards to hand (was discarding them), [Join] only Pokémon, [Undo] side-aware + new Active, Energy Recycle/Fellow Boost end the CPU turn, Magnetic Call crash (card_ops.shuffle_deck did not exist), Professor Elm's Training Method was scored as Professor Elm. Debug: ISSUE #373 prints.</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>Live: 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>374</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Powers</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>neo3/NP effects wrong: Major Flood / Major Earthquake, Psywave, Resonate, The Gifts, Mix-Up, Rush, Playful Punch, Softboiled, Howl, Electromagnetic Power, Energy Converter, Submerge, Unown [Bear]/[Yield], Lightning Burst, Magma Pool, Allergic Pollen, [Keep].</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>(Renumbered from #363 — that number already belonged to Enervating Pollen.) NP block uses gym1_hit_active; _np_discard_typed; Psywave r4_energy_amount; Resonate via apply_force_switch (defender chooses); The Gifts optional + Energy picked; Playful Punch 20 + turn ends; Softboiled/Howl are triggers; Energy Converter via set_meta (cleared end of turn); Submerge neo3_submerge effect; Allergic Pollen guards discard-pile effects; [Keep] enforced in discard_energy_from_pokemon. Debug: ISSUE #374 prints.</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>Live: 13</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Debug:  50,000 more simulations. Training CPU logic to self learn and grow
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -15926,12 +15926,12 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>Found by the new CPU-vs-bot autotester (Scenes/Autotest): SOFT-LOCKS — every "when you play this onto your Bench" prompt (Time Reversal, Purple Ray, [Engage], Dragon Boost, Delta Switch...) and every "when you evolve" prompt (Manipulate, Flame Vapor, Energy Recharge, Healing Shower...) opened invisibly on the player's turn; Lure / ex Pokémon Reversal picker over the opponent's Bench had no button; a card flight whose node was freed froze all later animations (Prize after Pokémon Center). CARD DUPLICATION — Old Rod and Breeder Fields discarded twice; send_to_discard left hand cards in the hand (Schemer, Rocket's Mission...); Buzzap cloned Electrode; Whirlwind/Teleport swapped twice. HP — evolving a boosted Pokémon went over max (Arbok 90/80); Undersea Ruins devolve kept the evolved HP (Skitty 70/40). CRASHES — Confusion self-KO let the attack run on a null Active; 90 cards with capital letters in their id (ecard H-holos, ex10 Unown) could never load; default coin image missing. LATER RUNS — Brock's Ninetales Shapeshift rewrote EVERY copy of the card (card objects shared one metadata dictionary) and the form card vanished on KO; Bubble Turn lost the Marill under Azumarill. Retreating into Octillery's Suction Cups discarded the retreat-cost Energy twice (same card twice in the discard pile). Peek (Mankey) screen could never be closed; the Hidden Power guess (ex10 text choice) crashed; Revive Friends (neo2 Kabuto) could never find a Kabuto. CPU never played most Stadiums (the "generic stadium heuristic" never existed), Pokémon Personality Test, Holon Farmer, Digger, Venture Bomb, base3 Mysterious Fossil (found via the new CPU-usage tracking). CPU attack choice should reason like a person (user examples: Voltorb Paralysis vs Confusion, Teddiursa Teary Eyes vs Scratch, Misdreavus Gift of Spite) — for EVERY card with the same kind of attack. Cancelling the Energy-type picker (Buzzap / Shift / Conversion) left the effect suspended; using it again froze the match. CPU-usage report round 2: 13 Trainers had a FLAT score below the play threshold (never playable) and Clefairy Doll / Blaine's Quizzes could never reach it. CPU played Rare Candy when it held a Stage 1 (useless) and held it with a Stage 2 (the whole point). Lt. Surge's Secret Plan card shuffled away by Mr. Fuji vanished. User requests: Blaine's Quiz CPU guessing by opponent class; Rocket's Secret Experiment, devolution effects, Memory Berry / TMs, Swoop! Teleporter, Surprise! Time Machine played when they fit the board. CPU Tools went onto the first Benched Pokémon. CPU with a stranded Active (no payable attack, no Energy in hand) refused to bench Basics (threshold) and passed every turn. Windstorm counted the CPU's own Stadium as a target and one target scored under the play threshold. CPU-usage "always" review: Here Comes Team Rocket! and both Pokémon Reversals had flat scores just over the threshold, so the CPU played them every time. Here Comes Team Rocket! did nothing (its side-wide face-up flags were never read). User rule: the CPU must not know its face-down Prizes.</t>
+          <t>Found by the new CPU-vs-bot autotester (Scenes/Autotest): SOFT-LOCKS — every "when you play this onto your Bench" prompt (Time Reversal, Purple Ray, [Engage], Dragon Boost, Delta Switch...) and every "when you evolve" prompt (Manipulate, Flame Vapor, Energy Recharge, Healing Shower...) opened invisibly on the player's turn; Lure / ex Pokémon Reversal picker over the opponent's Bench had no button; a card flight whose node was freed froze all later animations (Prize after Pokémon Center). CARD DUPLICATION — Old Rod and Breeder Fields discarded twice; send_to_discard left hand cards in the hand (Schemer, Rocket's Mission...); Buzzap cloned Electrode; Whirlwind/Teleport swapped twice. HP — evolving a boosted Pokémon went over max (Arbok 90/80); Undersea Ruins devolve kept the evolved HP (Skitty 70/40). CRASHES — Confusion self-KO let the attack run on a null Active; 90 cards with capital letters in their id (ecard H-holos, ex10 Unown) could never load; default coin image missing. LATER RUNS — Brock's Ninetales Shapeshift rewrote EVERY copy of the card (card objects shared one metadata dictionary) and the form card vanished on KO; Bubble Turn lost the Marill under Azumarill. Retreating into Octillery's Suction Cups discarded the retreat-cost Energy twice (same card twice in the discard pile). Peek (Mankey) screen could never be closed; the Hidden Power guess (ex10 text choice) crashed; Revive Friends (neo2 Kabuto) could never find a Kabuto. CPU never played most Stadiums (the "generic stadium heuristic" never existed), Pokémon Personality Test, Holon Farmer, Digger, Venture Bomb, base3 Mysterious Fossil (found via the new CPU-usage tracking). CPU attack choice should reason like a person (user examples: Voltorb Paralysis vs Confusion, Teddiursa Teary Eyes vs Scratch, Misdreavus Gift of Spite) — for EVERY card with the same kind of attack. Cancelling the Energy-type picker (Buzzap / Shift / Conversion) left the effect suspended; using it again froze the match. CPU-usage report round 2: 13 Trainers had a FLAT score below the play threshold (never playable) and Clefairy Doll / Blaine's Quizzes could never reach it. CPU played Rare Candy when it held a Stage 1 (useless) and held it with a Stage 2 (the whole point). Lt. Surge's Secret Plan card shuffled away by Mr. Fuji vanished. User requests: Blaine's Quiz CPU guessing by opponent class; Rocket's Secret Experiment, devolution effects, Memory Berry / TMs, Swoop! Teleporter, Surprise! Time Machine played when they fit the board. CPU Tools went onto the first Benched Pokémon. CPU with a stranded Active (no payable attack, no Energy in hand) refused to bench Basics (threshold) and passed every turn. Windstorm counted the CPU's own Stadium as a target and one target scored under the play threshold. CPU-usage "always" review: Here Comes Team Rocket! and both Pokémon Reversals had flat scores just over the threshold, so the CPU played them every time. Here Comes Team Rocket! did nothing (its side-wide face-up flags were never read). User rule: the CPU must not know its face-down Prizes. CPU ignored the cost of conditions its own attack puts on itself (Foul Odor / Dream Dance confuse or sleep BOTH Actives).</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>add_pokemon_to_bench triggers split into run_bench_from_hand_triggers (awaited after landing, not in setup); perform_evolution(is_opp, defer_after) + _after_evolution awaited after the evolve animation; forced-switch picker keeps its action button and the action handler only hands the pick back (waiters swap via animate_retreat); animate_card_a_to_b survives freed nodes; Old Rod/Breeder Fields no re-append; send_to_discard removes from hand; _buzzap_attach_electrode moves the real Electrode after the KO; evolution/devolve HP via get_max_hp; Undersea Ruins via _ex2_devolve_pokemon(discard) + KO check; confusion/blind bails return "stopped" + perform_attack null guard; get_card_metadata case-insensitive; tex_heads default = Pikachu Silver. ASSETS for the user: ex10-? (Unown ?) can't have a Windows filename; ex5-102 image missing. Debug: ISSUE #375 prints. card_object._init deep-copies its metadata; send_card_to_discard discards the Shapeshift form and restores Ninetales; Bubble Turn uses gym1_return_pokemon_to_hand (which now also resets pre-evolution HP); both devolve helpers use get_max_hp. animate_energies_to_discard skips Energy that is no longer attached, and still discards (without animating) when the Pokémon has no on-screen rect — it used to return and leave the retreat cost unpaid. Peek uses card_ops.show_cards; _ex10_choose_index returns the index (int/str wrappers); Revive Friends searches by exact name Kabuto (any stage). CPU_AI: _cpu_score_stadium_generic (own stadium never replaced, +value for removing the player's, board-specific for Strange Cave / Giant Stump / Holon Ruins / Cursed Stone / Mt. Moon / Tricky Gym / Broken Ground / Healing Field), _cpu_score_personality_test, _cpu_score_holon_farmer, _cpu_score_ko_10_coin (Digger/Venture Bomb only to finish a 10-HP Pokémon), base3-62 via _cpu_score_fossil. CPU_AI.cpu_status_value(): a Special Condition is worth what it stops x the turns it sticks (retreat cost, HP, threat, empty bench), flips x0.5 — used by attack scoring AND every choose-a-Special-Condition effect (cpu_pick_status via choose_special_condition). Energy-discard costs refunded fully on a certain KO, half on a likely one; r4_cpu_spend_energy / _cpu_type_surplus spend doomed Energy. Damage-reduction attacks compare HP saved vs damage dealt (stall to build). Estimator: +N per Energy attached to self (26 attacks, e.g. Power Blow). cancel_button_pressed_hide_selection_mode now answers energy_type_selected("") for energy_type_selection_active. Situational scorers: Town Volunteers, Energy Root, Crystal Shard, Mysterious Shard, Magnifier, Computer Error / Thought Wave Machine (only when the CPU cannot attack), Mirage Stadium (generic), bench insurance for Clefairy Doll / Lt. Surge's Secret Plan, Blaine's Quizzes scored on the real guessing odds (_cpu_score_quiz). _cpu_score_ex2_rare_candy uses the Stage 2 test Pokémon Breeder uses (_basic_matches_stage2). card_ops.unwrap_secret_plan() in send_card_to_discard / gym1_return_pokemon_to_hand / gym1_shuffle_into_deck / Mr. Fuji. NPC_and_Opponent_Data/Quiz_Knowledge.json + Trainer_Effects._quiz_skill(kind) (sprite-class accuracy; player already guesses via pickers). CPU_AI: _cpu_score_gym2_rockets_secret_experiment (tutor target vs Trainer lock), cpu_devolve_value / cpu_pick_devolution_spray_target(pool, to_basic) for Devolution Spray + Hyper Devolution Spray (status escape, KO with the lower form, alternate evolution in hand), _cpu_score_surprise_time_machine (better evolution in the deck), _cpu_score_attack_granting (TMs / Memory Berry tried on the Active), cpu_best_swoop (shared by score and effect). neo1_attach_tool CPU target = Active, else best Bench recipient. Time Machine damage carry uses get_max_hp. cpu_phase_bench_play lowers the bench threshold to 150 when the Active cannot attack and no Energy is in hand. _cpu_score_ex14_windstorm: player's Tools/Stadium only; 1 target 35, 2 targets 50. Here Comes Team Rocket! (base5-15/71, ex7-111) -100 (face-up Prizes only inform the player); _cpu_score_reversal: CPU-chooses = half Gust of Wind value, player-chooses only to push away a threatening Active. main.prize_is_face_up(card, side) = card flag OR side flag; used by the prize display, the selection screen and cpu_pick_prize (face-down = random, visible = chosen). _cpu_score_here_comes_team_rocket: when the CPU can KO now or leads the Prize race.</t>
+          <t>add_pokemon_to_bench triggers split into run_bench_from_hand_triggers (awaited after landing, not in setup); perform_evolution(is_opp, defer_after) + _after_evolution awaited after the evolve animation; forced-switch picker keeps its action button and the action handler only hands the pick back (waiters swap via animate_retreat); animate_card_a_to_b survives freed nodes; Old Rod/Breeder Fields no re-append; send_to_discard removes from hand; _buzzap_attach_electrode moves the real Electrode after the KO; evolution/devolve HP via get_max_hp; Undersea Ruins via _ex2_devolve_pokemon(discard) + KO check; confusion/blind bails return "stopped" + perform_attack null guard; get_card_metadata case-insensitive; tex_heads default = Pikachu Silver. ASSETS for the user: ex10-? (Unown ?) can't have a Windows filename; ex5-102 image missing. Debug: ISSUE #375 prints. card_object._init deep-copies its metadata; send_card_to_discard discards the Shapeshift form and restores Ninetales; Bubble Turn uses gym1_return_pokemon_to_hand (which now also resets pre-evolution HP); both devolve helpers use get_max_hp. animate_energies_to_discard skips Energy that is no longer attached, and still discards (without animating) when the Pokémon has no on-screen rect — it used to return and leave the retreat cost unpaid. Peek uses card_ops.show_cards; _ex10_choose_index returns the index (int/str wrappers); Revive Friends searches by exact name Kabuto (any stage). CPU_AI: _cpu_score_stadium_generic (own stadium never replaced, +value for removing the player's, board-specific for Strange Cave / Giant Stump / Holon Ruins / Cursed Stone / Mt. Moon / Tricky Gym / Broken Ground / Healing Field), _cpu_score_personality_test, _cpu_score_holon_farmer, _cpu_score_ko_10_coin (Digger/Venture Bomb only to finish a 10-HP Pokémon), base3-62 via _cpu_score_fossil. CPU_AI.cpu_status_value(): a Special Condition is worth what it stops x the turns it sticks (retreat cost, HP, threat, empty bench), flips x0.5 — used by attack scoring AND every choose-a-Special-Condition effect (cpu_pick_status via choose_special_condition). Energy-discard costs refunded fully on a certain KO, half on a likely one; r4_cpu_spend_energy / _cpu_type_surplus spend doomed Energy. Damage-reduction attacks compare HP saved vs damage dealt (stall to build). Estimator: +N per Energy attached to self (26 attacks, e.g. Power Blow). cancel_button_pressed_hide_selection_mode now answers energy_type_selected("") for energy_type_selection_active. Situational scorers: Town Volunteers, Energy Root, Crystal Shard, Mysterious Shard, Magnifier, Computer Error / Thought Wave Machine (only when the CPU cannot attack), Mirage Stadium (generic), bench insurance for Clefairy Doll / Lt. Surge's Secret Plan, Blaine's Quizzes scored on the real guessing odds (_cpu_score_quiz). _cpu_score_ex2_rare_candy uses the Stage 2 test Pokémon Breeder uses (_basic_matches_stage2). card_ops.unwrap_secret_plan() in send_card_to_discard / gym1_return_pokemon_to_hand / gym1_shuffle_into_deck / Mr. Fuji. NPC_and_Opponent_Data/Quiz_Knowledge.json + Trainer_Effects._quiz_skill(kind) (sprite-class accuracy; player already guesses via pickers). CPU_AI: _cpu_score_gym2_rockets_secret_experiment (tutor target vs Trainer lock), cpu_devolve_value / cpu_pick_devolution_spray_target(pool, to_basic) for Devolution Spray + Hyper Devolution Spray (status escape, KO with the lower form, alternate evolution in hand), _cpu_score_surprise_time_machine (better evolution in the deck), _cpu_score_attack_granting (TMs / Memory Berry tried on the Active), cpu_best_swoop (shared by score and effect). neo1_attach_tool CPU target = Active, else best Bench recipient. Time Machine damage carry uses get_max_hp. cpu_phase_bench_play lowers the bench threshold to 150 when the Active cannot attack and no Energy is in hand. _cpu_score_ex14_windstorm: player's Tools/Stadium only; 1 target 35, 2 targets 50. Here Comes Team Rocket! (base5-15/71, ex7-111) -100 (face-up Prizes only inform the player); _cpu_score_reversal: CPU-chooses = half Gust of Wind value, player-chooses only to push away a threatening Active. main.prize_is_face_up(card, side) = card flag OR side flag; used by the prize display, the selection screen and cpu_pick_prize (face-down = random, visible = chosen). _cpu_score_here_comes_team_rocket: when the CPU can KO now or leads the Prize race. _cpu_attack_context_adjust: self-target status = a cost (Confused by lost damage x retreat cost, Asleep/Paralyzed more, none if already affected, x0.3 when doomed). | SELF-PLAY TUNING (2026-10-09): 65 CPU_AI scoring numbers now read CpuWeights.g(key, default) (Scripts/Main_Match_Gameplay_Scripts/CPU_Weights.gd; multipliers from res://NPC_and_Opponent_Data/CPU_Weights.json, absent = original). Autotest_Runner --tune mode + Scripts/Autotest/cpu_tuner.py driver (paired-seed hill climbing vs the smart bot, crash-safe resume). Oracle now skips boards with set flags / Special Energy; LOG TEXT no longer flags card names containing "error". | 2026-10-09 eve: apply_card_text_effects skips Defending-Pokemon effects when the Defender is gone (null; was a script error at Attack_Effects.gd:2502). LEARNED SYNERGY: CPU_AI.cpu_synergy_bonus() adds a self-play synergy table (CpuWeights.synergy(); shipped res://NPC_and_Opponent_Data/CPU_Synergy.json, absent = none) to cpu_rank_keep_value + cpu_search_deck_for_best_card/_pokemon, scaled by tunable search.synergy; tuner-only exploration (CpuWeights.explore_pick) randomises 25% of free fetches in exploration games. Tester: MISSED KO bookkeeping (reset per attack phase, attack_begin records, CPU-won / blocked turns skipped), NO ENERGY counts Basic Energy only and respects Crystal Beam lock, ILLEGAL ENERGY ignores attach-time-only conditions (Bounce Energy), log scan ignores Computer Error / Terror card names.</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">

</xml_diff>

<commit_message>
Map Data: Changed day-night cycle and fixed map issues
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J379"/>
+  <dimension ref="A1:J380"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -16017,6 +16017,41 @@
       <c r="H379" t="inlineStr">
         <is>
           <t>09/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>378</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Overworld</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>The water shader used by surfacing Pokemon (PokemonSurfacer), Pokemon that jump into water (PokemonSkittish) and the fishing minigame's caught Pokemon drew the sprite too dark: it did texture(TEXTURE, UV) * COLOR, but in Godot 4.6 COLOR already contains the texture, so the sprite colour was squared. Found while building the time-of-day colour grade (verified by render: an identity shader using that line came out ~51/255 darker than the plain sprite).</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Pokemon_Surfacer.gd WATER_SHADER: c = COLOR instead of texture(TEXTURE, UV) * COLOR. One shared shader, so this covers all three users (surfacer, skittish water escape, fishing catch). Sprites will now look brighter while surfacing/diving than before -- check WATER_COLOUR / DEEP_COLOUR / ABOVE_TINT still look right with the corrected brightness. Debug: 'ISSUE #378 FIX ACTIVE' prints once when the shader is first built.</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deck Data: Created about 30 more decks ready to add to Opponents
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C20FF9B-5C5C-4536-A3FF-E91D82B5614C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCD4B1A-44E0-4F27-81E9-EC4067F550A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14715" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,12 +25,25 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Game_Issues!$A$1:$I$79</definedName>
     <definedName name="StatusList">'Data Validation'!$A$2:$A$8</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3251" uniqueCount="1419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3275" uniqueCount="1426">
   <si>
     <t>#</t>
   </si>
@@ -4478,6 +4491,28 @@
   </si>
   <si>
     <t xml:space="preserve">For things like porygon conversion, any effect or attack that changes weakness, resistance, or self typing (like a pokemon power that changes a cards typing) have another status symbol the same as what we have for the status conditions (like paralysis, burn, confused, sleep) with " [TYPE] RESIST" " [TYPE] TYPE" or " [TYPE] WEAK". These 3 status icons exist, but you will need to add the icon of the energy that is effected. </t>
+  </si>
+  <si>
+    <t>The new "Lights" layer in the overworld doesn't fade out when the scene fades in/out so the screen goes black but the "lights" tilesheet can still be seen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add a "Clear Filter" button to the left of "Search &amp; Filter" that only appears whe a search is active and simply resets the filter entirely and puts you back to the last set you were on. For the reset button on the actual search page, change the functionality so it only clears the search on hitting save (hit reset THEN save) and keep the filter on if you hit reset then cancel. </t>
+  </si>
+  <si>
+    <t>IF the player accidentally makes a large search, the search can't be cancelled or altered. The search &amp; Filter button can be pressed to reopen the filter page but the search continues and blocks player input so they can't just cancel it. If the search &amp; filter button is pressed, continue loading but have the filter page appear OVER the Loading blocker so you can clear the search and search for something new while it loads in the background or hit cancel and see the search fully loaded without loading again.</t>
+  </si>
+  <si>
+    <t>When the player hits save on a deck, pop up one of the floating labels with "DECK SAVED!" (the screen doesn’t vanish so not obvious the deck is saved)</t>
+  </si>
+  <si>
+    <t>I think we changed from rendering the lower quality (small) images for cards in deck view mode and sleeves in sleeve selection. I thought this wouldn't add a noticeable time onto loading but it has so if so put the smaller images back to small. If shift is pressed, then load the high res version but in standard views the cards and sleeves should all be the lower res versions.</t>
+  </si>
+  <si>
+    <t>Duplication</t>
+  </si>
+  <si>
+    <t>A lot of pokemon sets have a duplicate Holo rare and a normal rare. This was bad in Jungle and Fossil such that half the cards were duplicates. I have deleted all the non-holo variants from Jungle and Fossil but for compatibility I have kept their data in the card set data JSON. HOWEVER i have removed it from the player owned card set data and the seed data so that to the player that card doesn't exist, they can't see them and they can't unlock/earn it, and it isn't counted in the set's total counts. Now do the same with the Neo-ex cards. Find anything that is an exact duplicate of itself (e.g from ecard there is Gengar 13 as a holo and gengar 48 which is identical except it's a non-holo rare. The ONLY difference is the rarity. Find all cards that are these EXACT duplicates and remove the non holo version so it can't be obtained. Do not remove anything else that isn't an exact 1-1 copy with every single same attack, HP. Somo holo rares in later sets have a completely different illustration but the rest of the data remains the same so find these but let me know about them, still delete them unless it's a secret rare vs holo rare (e.g the gym leaders have a holo and non holo but the non holo has different art but it's fine to lose them. Only delete things that are obviously, no ambiguity, no assumptions made definitely a direct 1 to 1 replicata except for the rareness. (e.g there are 2 bayleefs in Neo genesis but they are different. Neo discovery has 2 different espeons, but the forretress, houndoom, kabutops etc are all duplicated in non holo form.)
+Also, there are a lot of cards that are duplicated across different sets (ignore basic energies) but stuff like pokemon trainer cards across the EX era. Find me all these duplicates</t>
   </si>
 </sst>
 </file>
@@ -5083,7 +5118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J393"/>
+  <dimension ref="A1:J399"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
@@ -15195,6 +15230,108 @@
       </c>
       <c r="G393" s="6" t="s">
         <v>351</v>
+      </c>
+    </row>
+    <row r="394" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A394" s="5">
+        <v>391</v>
+      </c>
+      <c r="B394" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C394" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D394" s="6" t="s">
+        <v>1419</v>
+      </c>
+      <c r="G394" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="395" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A395" s="5">
+        <v>392</v>
+      </c>
+      <c r="B395" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C395" s="5" t="s">
+        <v>1408</v>
+      </c>
+      <c r="D395" s="6" t="s">
+        <v>1420</v>
+      </c>
+      <c r="G395" s="6" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="396" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A396" s="5">
+        <v>393</v>
+      </c>
+      <c r="B396" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C396" s="5" t="s">
+        <v>1408</v>
+      </c>
+      <c r="D396" s="6" t="s">
+        <v>1421</v>
+      </c>
+      <c r="G396" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="397" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A397" s="5">
+        <v>394</v>
+      </c>
+      <c r="B397" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C397" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D397" s="6" t="s">
+        <v>1422</v>
+      </c>
+      <c r="G397" s="6" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="398" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A398" s="5">
+        <v>395</v>
+      </c>
+      <c r="B398" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C398" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D398" s="6" t="s">
+        <v>1423</v>
+      </c>
+      <c r="G398" s="6" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="399" spans="1:7" ht="225" x14ac:dyDescent="0.25">
+      <c r="A399" s="5">
+        <v>396</v>
+      </c>
+      <c r="B399" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="C399" s="5" t="s">
+        <v>1424</v>
+      </c>
+      <c r="D399" s="6" t="s">
+        <v>1425</v>
+      </c>
+      <c r="G399" s="6" t="s">
+        <v>1404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Card Data: Removed non-holo duplicates of holo rares within a set entirely
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCD4B1A-44E0-4F27-81E9-EC4067F550A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2662342-25A0-4764-A4B4-B8B8C993CC00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14715" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3275" uniqueCount="1426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3271" uniqueCount="1424">
   <si>
     <t>#</t>
   </si>
@@ -4506,13 +4506,6 @@
   </si>
   <si>
     <t>I think we changed from rendering the lower quality (small) images for cards in deck view mode and sleeves in sleeve selection. I thought this wouldn't add a noticeable time onto loading but it has so if so put the smaller images back to small. If shift is pressed, then load the high res version but in standard views the cards and sleeves should all be the lower res versions.</t>
-  </si>
-  <si>
-    <t>Duplication</t>
-  </si>
-  <si>
-    <t>A lot of pokemon sets have a duplicate Holo rare and a normal rare. This was bad in Jungle and Fossil such that half the cards were duplicates. I have deleted all the non-holo variants from Jungle and Fossil but for compatibility I have kept their data in the card set data JSON. HOWEVER i have removed it from the player owned card set data and the seed data so that to the player that card doesn't exist, they can't see them and they can't unlock/earn it, and it isn't counted in the set's total counts. Now do the same with the Neo-ex cards. Find anything that is an exact duplicate of itself (e.g from ecard there is Gengar 13 as a holo and gengar 48 which is identical except it's a non-holo rare. The ONLY difference is the rarity. Find all cards that are these EXACT duplicates and remove the non holo version so it can't be obtained. Do not remove anything else that isn't an exact 1-1 copy with every single same attack, HP. Somo holo rares in later sets have a completely different illustration but the rest of the data remains the same so find these but let me know about them, still delete them unless it's a secret rare vs holo rare (e.g the gym leaders have a holo and non holo but the non holo has different art but it's fine to lose them. Only delete things that are obviously, no ambiguity, no assumptions made definitely a direct 1 to 1 replicata except for the rareness. (e.g there are 2 bayleefs in Neo genesis but they are different. Neo discovery has 2 different espeons, but the forretress, houndoom, kabutops etc are all duplicated in non holo form.)
-Also, there are a lot of cards that are duplicated across different sets (ignore basic energies) but stuff like pokemon trainer cards across the EX era. Find me all these duplicates</t>
   </si>
 </sst>
 </file>
@@ -5118,7 +5111,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J399"/>
+  <dimension ref="A1:J398"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
@@ -15317,26 +15310,9 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="399" spans="1:7" ht="225" x14ac:dyDescent="0.25">
-      <c r="A399" s="5">
-        <v>396</v>
-      </c>
-      <c r="B399" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="C399" s="5" t="s">
-        <v>1424</v>
-      </c>
-      <c r="D399" s="6" t="s">
-        <v>1425</v>
-      </c>
-      <c r="G399" s="6" t="s">
-        <v>1404</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:I79" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A2:J1000">
+  <conditionalFormatting sqref="A2:J999">
     <cfRule type="expression" dxfId="15" priority="1" stopIfTrue="1">
       <formula>OR($G2="New Issue",$G2="Fix Failed",$G2="Improve Further",$G2="New Functionality")</formula>
     </cfRule>

</xml_diff>

<commit_message>
Debug: Changed, amended and fixed a load of issues with the new intros
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A984F81-6DE6-431C-B437-C2B540FD819A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708C23A2-2DB1-4C5C-A224-C85FA7130D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14715" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3436" uniqueCount="1476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3692" uniqueCount="1561">
   <si>
     <t>#</t>
   </si>
@@ -3137,6 +3137,249 @@
     <t>[19/10/2026] Gengar, Shuppet, Code, Umbreon and Sharpedo had near-black (four of them flat) chrome bars, so there was no visible gradient and selections fell back to accent. All five, Dark and Light, now have a bold three-stop gradient from their own accent hues (deep / signature / complementary), each stop dark enough for the white bar text at 4.5:1: Gengar 7340C8&gt;C8357A&gt;B05A0A, Shuppet 4A4FC8&gt;1F72C8&gt;C9463A, Code 4A50C8&gt;007F78&gt;D01A63 (teal is the middle/signature stop so selections stay Code-cyan), Umbreon 286A82&gt;2F7A90&gt;957012, Sharpedo 2A4F94&gt;2C68C0&gt;B85D1C. Their keylines are now transparent, like the other vivid bars. The selected fill (chrome_grad_b) is now that bold middle colour on every theme. Button art rebuilt for all 16 themes; Theme_Audit PASS, 0 failures, warnings down from 12 to 2. Checked by rendering all five.</t>
   </si>
   <si>
+    <t>at the start of the match when choosing the coin flip, make the coins 50% bigger but move them way further into the center of the screen so they aren't as far apart. Reduce the gap size to only about 20% of what it is now</t>
+  </si>
+  <si>
+    <t>[21/10/2026] choose_heads_or_tails() (Main_Match_Core_Gameplay_Script): COIN_CALL_SIZE 258 -&gt; 387 (50% bigger); the coins were centred at 25%/75% of the screen (~702px edge gap) and now sit COIN_CALL_GAP 140px apart (~20%) either side of centre. Also new: heads flies in from the left and tails from the right, fading up from transparent over COIN_CALL_FLY_TIME 1.0s; clicks wait until they land.</t>
+  </si>
+  <si>
+    <t>21/10/2026</t>
+  </si>
+  <si>
+    <t>when the coin flips it starts and lands ever so slightly overlapping the message box. Instead, have the coin's base position upwards so there's about 5-15px of seperation between the top of the message box and the bottom of the coin. In fact go the other way the messagebox got moved up I think when we put yes/no underneath it. However in a match the messagebox should never need the yes/no as every choice is presented differently so in a match move the messagebox back down so that there is only a few pixels from the bottom of the screen below the message and that the whole messagebox fits neatly and in the center of the footer such that the top of the message box and bottom of the messagebox are inside the footer on the screen with equal distance above and below the messagebox to the top and bottom of the footer. The coin can probably stay where it is then</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Main_Match_Core_Gameplay_Script._ensure_match_msgbox(): the in-match box (never has Yes/No) now set_panel_bottom()s to 1080 - (BOARD_BOT_H 162 - MATCH_MSGBOX_HEIGHT 138)/2 = 1068, so it sits centred inside the footer with 12px above and below (was the overworld spot, bottom 1034, which leaves room for buttons). Coin left where it was, as asked. Also (user request): new DynamicMessageBox.set_fill_alpha(); the match box is MATCH_MSGBOX_FILL_ALPHA 0.985 opaque (overworld stays 0.94).</t>
+  </si>
+  <si>
+    <t>Intro redesign: 4 familiarity starts (new / rules / played / expert + Hard Mode) with different start days, phone calls, decks, Olly instead of Ellie, no moving-in, starter box and shop starter set removed, new tutorial system (scripted / guided / generic), Options toggle for tutorial messages, hard mode no rematches and no x3.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] GameState INTRO_PROFILES + ARRIVAL NIGHT + OLLY'S INTRO sections; Olly_Intro_Cutscene.gd (arrival, deck choice IntroDeckChoice, Hard Mode draft + deck builder draft mode, forced battle with per-fight overrides, post-match gifts); Tutorial_Director.gd (stacked decks, gates, messages, labels); Phone_Calls.json intro_call_*; Shopkeeper date-based greetings; MapManager no-rematch notice; outro time advance + hard mode cash.</t>
+  </si>
+  <si>
+    <t>Time advance: day 1 = 2 battles per time slot (incl. Olly), day 2 = 3, day 3+ = 4. Days 1-2 count new wins only; day 3+ every match (wins, losses, rematches).</t>
+  </si>
+  <si>
+    <t>[21/10/2026] GameState.matches_to_advance_time() 2/3/4 and count_match_toward_time(); outro calls it once per finished match.</t>
+  </si>
+  <si>
+    <t>Day 1: Olly should not say Ellie is at the pier. Newby farewell: 'El has gone out for the day and is back tonight, Alexander is covering the shop for me this evening...'. Olly always says 'Alexander', never 'Alex'.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Olly_Intro_Cutscene LINES_NEW_GOODBYE / LINES_RULES_GOODBYE rewritten; FISH rota day 1 = Olly M,A / Alexander E,N to match.</t>
+  </si>
+  <si>
+    <t>'I know the rules a bit' start: arrive evening 1 (not night 0), new phone call (tournament finished early, Olly comes round now), player stops short of the door facing up during the call, Olly runs in when he hangs up; 'Hey!' opener; after the match 'Alexander is covering the shop... pick up that rod from him'.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] INTRO_PROFILES rules = start_date 1 Evening, olly_meets 'taxi'; intro_call_rules; Celeste_Harbour._hand_over_to_olly(); LINES_OPEN_EVENING / LINES_RULES_GOODBYE.</t>
+  </si>
+  <si>
+    <t>FISH first-visit intro should be played by whoever is behind the counter; Alexander tells it in the third person about Olly.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Fish_Shop_Intro_Cutscene takes name/sprite/colour from the scheduled keeper; LINES_*_ALEXANDER variants.</t>
+  </si>
+  <si>
+    <t>FISH intro: drop the 'took over FISH a couple of months back' line; the player has just picked fishing up for the first time ('I knew you'd come round to fishing eventually', 'You'll probably be really good at it...', 'Good luck!').</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Removed the takeover line from both keepers' pitches; reworded the 'used to love fishing' lines and the closing lines.</t>
+  </si>
+  <si>
+    <t>Starting a new game the taxi intro showed evening colours instead of night (lights were on).</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Celeste_Harbour taxi path skipped BaseMapScene._ready, so the time-of-day grade was never applied; it now calls _setup_time_of_day_grade() and TimeOfDayGrade.style_lights().</t>
+  </si>
+  <si>
+    <t>Taxi intro: remove the pause at the door when the phone call is already over.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] INTRO_UNLOCK_PAUSE removed; only a call still running gets the look-down / look-up / short pause.</t>
+  </si>
+  <si>
+    <t>After reading Mum's note show 'I'll call mum tomorrow...'.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Player_House_Downstairs NOTE_AFTER_TEXT shown when the note closes.</t>
+  </si>
+  <si>
+    <t>When the starter deck is gifted show the deck box art (starterdeck1_a-d), fading in, instead of spinning cards.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] MapManager.show_pack_reveal() (new 'pack' gift kind, card-box size, fade-in); Olly_Intro_Cutscene DECK_ART_*. Bonus packs use it too.</t>
+  </si>
+  <si>
+    <t>'You got the starter deck!' screen could not be clicked away (Enter worked).</t>
+  </si>
+  <si>
+    <t>[21/10/2026] The gift reveal's dim overlay stayed MOUSE_FILTER_STOP after the reveal, swallowing every click; it is set back to IGNORE when the reveal ends, and 'pack' got a reveal duration.</t>
+  </si>
+  <si>
+    <t>Deck choice decks should fly and fade in from the bottom one after another (1s each, 0.5s apart), replayed after a No; coin choices: heads flies in from the left, tails from the right, meeting in the middle.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] IntroDeckChoice._play_entrance(); choose_heads_or_tails() coin fly-in. Clicks wait until they land.</t>
+  </si>
+  <si>
+    <t>In a match the message box should be fully opaque so the board under it doesn't make it hard to read.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] DynamicMessageBox.set_fill_alpha(); MATCH_MSGBOX_FILL_ALPHA 1.0 (overworld box unchanged at 94%).</t>
+  </si>
+  <si>
+    <t>Quitting the tutorial match mid-way counted as a loss. Checkpoints only at stepping outside and at win/loss; quitting before that resets to stepping outside (deck choice can be changed, Hard Mode packs re-roll; pack cards only kept once the deck is saved).</t>
+  </si>
+  <si>
+    <t>[21/10/2026] GameState INTRO CHECKPOINT: slot files copied when Olly's scene starts (and when the Hard Mode deck is saved), restored by load_slot() until the outro decides the match; bonus pack given once only.</t>
+  </si>
+  <si>
+    <t>Match start transition: the overworld breaks into pixels and dissolves away, the intro background dissolves in the same way, sprites/names keep their fly/fade at double time; then made 3x quicker and the pause before it removed.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Pixel_Dissolve.gdshader + PixelDissolve.gd (reads the live screen, no snapshot stall); OUT_TIME 0.55 / IN_TIME 0.47; Match_Start_Intro ENTRANCE_SCALE 2.0 with BattleFrame.fade_foreground.</t>
+  </si>
+  <si>
+    <t>Punctuation pauses only for NPC / opponent / shop / cutscene speech (overworld and intro/outro), not for system messages, signs or in-match messages.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] DynamicMessageBox._build_pauses() returns early for the system variant or a box with no speaker name pill.</t>
+  </si>
+  <si>
+    <t>Buttons (e.g. the big Cancel) drew over the in-match message box when a pile was opened.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] msgbox_container z_index raised to Z_CHROME + 25 (above the footer buttons and tutorial captions; draw order only).</t>
+  </si>
+  <si>
+    <t>Clicking a deck can't view it, so remove the tutorial 'you are viewing your deck' message on deck clicks.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Deck icon click handler and both deck PILE_LINES removed.</t>
+  </si>
+  <si>
+    <t>Tutorial pile messages (bench, prizes, discard, opponent hand) repeat on every click until the end of the player's first turn, then only show for a pile not yet explained.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Tutorial_Director.on_pile_viewed(); new prize-card lines added.</t>
+  </si>
+  <si>
+    <t>For a newby player, their SECOND match plays the start-of-turn key tips (Shift preview, Caps Lock log, Escape forfeit).</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Tutorial_Director 'tips' mode, armed by GameState.TUTORIAL_TIPS_KEY when the newby wins Olly's match, cleared when that match ends.</t>
+  </si>
+  <si>
+    <t>Energy cards gift: fly and fade in from the bottom, left to right, 0.2s apart. All fly-ins (coins, decks, energies) slow down, overshoot a few px and fall back.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] UIKit.fly_in() (FLY_OVERSHOOT_PX 12); MapManager 'card_fly' gift kind (CARD_FLY_* consts).</t>
+  </si>
+  <si>
+    <t>Newby: cancelling an action (e.g. backing out of attaching energy) leaves no instructions; repeat the step's instruction and the energy requirement explanation.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Attach-screen explanation replays every time until attached; NEWBY_REMINDERS line on reopening the hand in the same step.</t>
+  </si>
+  <si>
+    <t>Double the delay between HP damage blocks greying out.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] HP_BLOCK_STEP 0.07 -&gt; 0.14 (healing does not animate per block).</t>
+  </si>
+  <si>
+    <t>A tutorial block (e.g. energy onto the wrong Voltorb) closed the attach screen as if the action had happened.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] perform_energy_attachment block now reopens the attach screen with the same Energy.</t>
+  </si>
+  <si>
+    <t>Match log button in the in-match Escape menu; tutorial messages recorded in the log, visually distinct; 'Press [CAPS LOCK] To read back any of these help messages' at match start; Caps Lock over a message doesn't advance it.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Pause menu 'Match log' button; show_message log_kind 'tutorial' -&gt; Match_Log_Panel tinted HELP rows; Tutorial_Director CAPS_HINT. Caps Lock over a message already worked (log swallows all input).</t>
+  </si>
+  <si>
+    <t>When a card is played, the hand / selection screen and its buttons fade out and the board fades in instead of snapping.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Main_Match_Core SCREEN SWAP FADE (SCREEN_SWAP_FADE 0.15).</t>
+  </si>
+  <si>
+    <t>Half the speed and double the life of every floating label across the game.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Match show_floating_label 5.0s rise / 3.0s fade; deck builder MSG_*; bulk sell CARD/TOTAL_LABEL_*; fishing NEW_TAG_* (also the Fish Coin tag); Info cheat toast.</t>
+  </si>
+  <si>
+    <t>Newby tutorial timing broken by the fighting energy count. Swap one of the opponent's Water Energy for Energy Removal and have Olly play it on Machop before Dratini's Pound.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Basic Battle Deck: 18 Water + 1 Energy Removal; Professor Oak draws Fighting x5, Rattata, Energy Removal; NEWBY_CPU_PLAN turn 7 Energy Removal on the Active; turn-7 lines restored ('only has 1').</t>
+  </si>
+  <si>
+    <t>Newby first turn: explain the aim of the game, prize cards, energy and attaching to the active Pokemon before 'Click your hand'.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Tutorial_Director NEWBY_T1_AIM (6 lines, [POKEMON] = the active).</t>
+  </si>
+  <si>
+    <t>Deck choice: darken first, old Kenney font on the names, options too high (centre the cards, not the text), deck box art peeking out behind each fan's back card, cards moved left and decks spread wider.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] IntroDeckChoice: DIM 0.8 fades first, names forced to ChakraPetch-Bold, CARDS_MID_Y 540, deck box (BOX_HEIGHT/TUCK/RAISE), GROUP_CENTRES 320/960/1600.</t>
+  </si>
+  <si>
+    <t>Coin flip header hidden; 'Build your bench' header and its two buttons stuck on screen after the coin flip until the hand was next opened.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Both caused by the new card-play fade: the coin call saved the fading bench header/buttons as visible and restored them. _snap_screen_swap() now hides fading-out pieces and runs before the coin call.</t>
+  </si>
+  <si>
+    <t>Tutorial 'Opponent's hand' label not visible.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] It drew under the header bar; now z_index Z_CHROME + 20.</t>
+  </si>
+  <si>
+    <t>Double clicking an energy card crashed the game.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] CardDisplay._input carried on after card_clicked played the card and freed the node (get_tree() null); it now returns if the node left the tree.</t>
+  </si>
+  <si>
+    <t>Interior camera completely locked; allow a little movement while keeping the room (mostly) in view.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Player_Object_Script CAMERA_ROOM_SLACK 28 world px either way on axes where the room is smaller than the view.</t>
+  </si>
+  <si>
+    <t>Convert DraftTime (RSE Trick House).mp3 to .ogg; play it during Hard Mode's pack opening, back to the overworld track after, and in the draft deck builder.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Converted with ffmpeg (imageio-ffmpeg); SoundManager BGM_DRAFT_TIME + crossfade_bgm(); Olly_Intro_Cutscene and deck builder draft mode use it.</t>
+  </si>
+  <si>
+    <t>Hard Mode: no gap between the energies and being forced into the deck builder. Gift the energies, close the gift screen, then 'Hey, let's try building a deck right now!...' before the deck builder.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] LINE_HARD_AFTER_PACKS reworded; LINES_HARD_BUILD said after the energy reveal closes.</t>
+  </si>
+  <si>
+    <t>Sort by '# Owned', and remember the previous sort order so sorts stack (newest first, earlier ones as tie-breakers).</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Card_Search_Overlay '# OWNED' mode + _sort_chain; deck builder _sort_search_results() sorts by the whole chain.</t>
+  </si>
+  <si>
+    <t>Olly doesn't walk down far enough before going left and gets stuck on the player's wall; he should run to the path then up off screen towards FISH.</t>
+  </si>
+  <si>
+    <t>[21/10/2026] Exit is now a glide (no collision): down to the path, along to EXIT_PATH_X -712, up EXIT_RUN_UP 700; player watches him go.</t>
+  </si>
+  <si>
     <t>UID</t>
   </si>
   <si>
@@ -4649,10 +4892,22 @@
     <t>Fix Failed</t>
   </si>
   <si>
-    <t>at the start of the match when choosing the coin flip, make the coins 50% bigger but move them way further into the center of the screen so they aren't as far apart. Reduce the gap size to only about 20% of what it is now</t>
-  </si>
-  <si>
-    <t>when the coin flips it starts and lands ever so slightly overlapping the message box. Instead, have the coin's base position upwards so there's about 5-15px of seperation between the top of the message box and the bottom of the coin. In fact go the other way the messagebox got moved up I think when we put yes/no underneath it. However in a match the messagebox should never need the yes/no as every choice is presented differently so in a match move the messagebox back down so that there is only a few pixels from the bottom of the screen below the message and that the whole messagebox fits neatly and in the center of the footer such that the top of the message box and bottom of the messagebox are inside the footer on the screen with equal distance above and below the messagebox to the top and bottom of the footer. The coin can probably stay where it is then</t>
+    <t>The opponent used gust of wind when for a pokemon with the same HP which it was already a guarenteed knockout for. It provided no value. Then it attached two pluspowers putting it to +20 damage over what it needed when it didn't need any at all. It was mewtwo using psyburn on an ekans, gust of winding it for venonat, then knocking venonat out</t>
+  </si>
+  <si>
+    <t>Also the opponent just played plus power on hitmonchan against ekans, it used jab for 30hp danage, 2 x 20hp jabs would have done the same. Pluspower should have been kept</t>
+  </si>
+  <si>
+    <t>the CPU then retreated hitmonchan with 2 discards for mewtwo on the bench for no reason when ekans had 10hp and was knokced out by jab and player had nothing to return fire with</t>
+  </si>
+  <si>
+    <t>and again mewtwo attached pluspower for 50 damage when player only had 30</t>
+  </si>
+  <si>
+    <t>When playing professor oak (so most liekly any effect that draws multiple cards, the cards vanish quicker than they animate moving to the discard pile, they should only vanish AS the card moves</t>
+  </si>
+  <si>
+    <t>The CPU had a spearow, attached a pluspower which would have knocked out pikachu with 20hp but then evolved to fearow when only one energy was attached insteaqd of guarenteeing the kill</t>
   </si>
 </sst>
 </file>
@@ -5258,7 +5513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J415"/>
+  <dimension ref="A1:J459"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
@@ -5270,8 +5525,8 @@
     <col min="7" max="7" width="19" style="6" customWidth="1"/>
     <col min="8" max="9" width="11.140625" style="7" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="7" hidden="1" customWidth="1"/>
-    <col min="11" max="27" width="9.140625" style="7" customWidth="1"/>
-    <col min="28" max="16384" width="9.140625" style="7"/>
+    <col min="11" max="29" width="9.140625" style="7" customWidth="1"/>
+    <col min="30" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -15989,7 +16244,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="413" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A413" s="5">
         <v>411</v>
       </c>
@@ -16000,13 +16255,19 @@
         <v>45</v>
       </c>
       <c r="D413" s="6" t="s">
-        <v>1474</v>
+        <v>970</v>
+      </c>
+      <c r="E413" t="s">
+        <v>971</v>
       </c>
       <c r="G413" s="6" t="s">
-        <v>1471</v>
-      </c>
-    </row>
-    <row r="414" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="H413" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="414" spans="1:10" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A414" s="5">
         <v>412</v>
       </c>
@@ -16017,10 +16278,16 @@
         <v>45</v>
       </c>
       <c r="D414" s="6" t="s">
-        <v>1475</v>
+        <v>973</v>
+      </c>
+      <c r="E414" t="s">
+        <v>974</v>
       </c>
       <c r="G414" s="6" t="s">
-        <v>1471</v>
+        <v>19</v>
+      </c>
+      <c r="H414" t="s">
+        <v>972</v>
       </c>
     </row>
     <row r="415" spans="1:10" x14ac:dyDescent="0.25">
@@ -16035,6 +16302,982 @@
       </c>
       <c r="G415" s="6" t="s">
         <v>351</v>
+      </c>
+    </row>
+    <row r="416" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A416">
+        <v>414</v>
+      </c>
+      <c r="B416" t="s">
+        <v>181</v>
+      </c>
+      <c r="C416" t="s">
+        <v>351</v>
+      </c>
+      <c r="D416" t="s">
+        <v>975</v>
+      </c>
+      <c r="E416" t="s">
+        <v>976</v>
+      </c>
+      <c r="G416" t="s">
+        <v>19</v>
+      </c>
+      <c r="H416" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="417" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A417">
+        <v>415</v>
+      </c>
+      <c r="B417" t="s">
+        <v>181</v>
+      </c>
+      <c r="C417" t="s">
+        <v>561</v>
+      </c>
+      <c r="D417" t="s">
+        <v>977</v>
+      </c>
+      <c r="E417" t="s">
+        <v>978</v>
+      </c>
+      <c r="G417" t="s">
+        <v>19</v>
+      </c>
+      <c r="H417" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="418" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A418">
+        <v>416</v>
+      </c>
+      <c r="B418" t="s">
+        <v>100</v>
+      </c>
+      <c r="C418" t="s">
+        <v>101</v>
+      </c>
+      <c r="D418" t="s">
+        <v>979</v>
+      </c>
+      <c r="E418" t="s">
+        <v>980</v>
+      </c>
+      <c r="G418" t="s">
+        <v>19</v>
+      </c>
+      <c r="H418" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="419" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A419">
+        <v>417</v>
+      </c>
+      <c r="B419" t="s">
+        <v>181</v>
+      </c>
+      <c r="C419" t="s">
+        <v>351</v>
+      </c>
+      <c r="D419" t="s">
+        <v>981</v>
+      </c>
+      <c r="E419" t="s">
+        <v>982</v>
+      </c>
+      <c r="G419" t="s">
+        <v>19</v>
+      </c>
+      <c r="H419" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="420" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A420">
+        <v>418</v>
+      </c>
+      <c r="B420" t="s">
+        <v>95</v>
+      </c>
+      <c r="C420" t="s">
+        <v>351</v>
+      </c>
+      <c r="D420" t="s">
+        <v>983</v>
+      </c>
+      <c r="E420" t="s">
+        <v>984</v>
+      </c>
+      <c r="G420" t="s">
+        <v>19</v>
+      </c>
+      <c r="H420" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="421" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A421">
+        <v>419</v>
+      </c>
+      <c r="B421" t="s">
+        <v>100</v>
+      </c>
+      <c r="C421" t="s">
+        <v>101</v>
+      </c>
+      <c r="D421" t="s">
+        <v>985</v>
+      </c>
+      <c r="E421" t="s">
+        <v>986</v>
+      </c>
+      <c r="G421" t="s">
+        <v>19</v>
+      </c>
+      <c r="H421" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="422" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A422">
+        <v>420</v>
+      </c>
+      <c r="B422" t="s">
+        <v>21</v>
+      </c>
+      <c r="C422" t="s">
+        <v>45</v>
+      </c>
+      <c r="D422" t="s">
+        <v>987</v>
+      </c>
+      <c r="E422" t="s">
+        <v>988</v>
+      </c>
+      <c r="G422" t="s">
+        <v>19</v>
+      </c>
+      <c r="H422" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="423" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A423">
+        <v>421</v>
+      </c>
+      <c r="B423" t="s">
+        <v>95</v>
+      </c>
+      <c r="C423" t="s">
+        <v>110</v>
+      </c>
+      <c r="D423" t="s">
+        <v>989</v>
+      </c>
+      <c r="E423" t="s">
+        <v>990</v>
+      </c>
+      <c r="G423" t="s">
+        <v>19</v>
+      </c>
+      <c r="H423" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="424" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A424">
+        <v>422</v>
+      </c>
+      <c r="B424" t="s">
+        <v>100</v>
+      </c>
+      <c r="C424" t="s">
+        <v>30</v>
+      </c>
+      <c r="D424" t="s">
+        <v>991</v>
+      </c>
+      <c r="E424" t="s">
+        <v>992</v>
+      </c>
+      <c r="G424" t="s">
+        <v>19</v>
+      </c>
+      <c r="H424" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="425" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A425">
+        <v>423</v>
+      </c>
+      <c r="B425" t="s">
+        <v>21</v>
+      </c>
+      <c r="C425" t="s">
+        <v>45</v>
+      </c>
+      <c r="D425" t="s">
+        <v>993</v>
+      </c>
+      <c r="E425" t="s">
+        <v>994</v>
+      </c>
+      <c r="G425" t="s">
+        <v>19</v>
+      </c>
+      <c r="H425" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="426" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A426">
+        <v>424</v>
+      </c>
+      <c r="B426" t="s">
+        <v>21</v>
+      </c>
+      <c r="C426" t="s">
+        <v>78</v>
+      </c>
+      <c r="D426" t="s">
+        <v>995</v>
+      </c>
+      <c r="E426" t="s">
+        <v>996</v>
+      </c>
+      <c r="G426" t="s">
+        <v>19</v>
+      </c>
+      <c r="H426" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="427" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A427">
+        <v>425</v>
+      </c>
+      <c r="B427" t="s">
+        <v>21</v>
+      </c>
+      <c r="C427" t="s">
+        <v>45</v>
+      </c>
+      <c r="D427" t="s">
+        <v>997</v>
+      </c>
+      <c r="E427" t="s">
+        <v>998</v>
+      </c>
+      <c r="G427" t="s">
+        <v>19</v>
+      </c>
+      <c r="H427" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="428" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A428">
+        <v>426</v>
+      </c>
+      <c r="B428" t="s">
+        <v>21</v>
+      </c>
+      <c r="C428" t="s">
+        <v>45</v>
+      </c>
+      <c r="D428" t="s">
+        <v>999</v>
+      </c>
+      <c r="E428" t="s">
+        <v>1000</v>
+      </c>
+      <c r="G428" t="s">
+        <v>19</v>
+      </c>
+      <c r="H428" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="429" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A429">
+        <v>427</v>
+      </c>
+      <c r="B429" t="s">
+        <v>181</v>
+      </c>
+      <c r="C429" t="s">
+        <v>561</v>
+      </c>
+      <c r="D429" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E429" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G429" t="s">
+        <v>19</v>
+      </c>
+      <c r="H429" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="430" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A430">
+        <v>428</v>
+      </c>
+      <c r="B430" t="s">
+        <v>44</v>
+      </c>
+      <c r="C430" t="s">
+        <v>351</v>
+      </c>
+      <c r="D430" t="s">
+        <v>1003</v>
+      </c>
+      <c r="E430" t="s">
+        <v>1004</v>
+      </c>
+      <c r="G430" t="s">
+        <v>19</v>
+      </c>
+      <c r="H430" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="431" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A431">
+        <v>429</v>
+      </c>
+      <c r="B431" t="s">
+        <v>100</v>
+      </c>
+      <c r="C431" t="s">
+        <v>30</v>
+      </c>
+      <c r="D431" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E431" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G431" t="s">
+        <v>19</v>
+      </c>
+      <c r="H431" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="432" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A432">
+        <v>430</v>
+      </c>
+      <c r="B432" t="s">
+        <v>21</v>
+      </c>
+      <c r="C432" t="s">
+        <v>45</v>
+      </c>
+      <c r="D432" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E432" t="s">
+        <v>1008</v>
+      </c>
+      <c r="G432" t="s">
+        <v>19</v>
+      </c>
+      <c r="H432" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="433" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A433">
+        <v>431</v>
+      </c>
+      <c r="B433" t="s">
+        <v>181</v>
+      </c>
+      <c r="C433" t="s">
+        <v>78</v>
+      </c>
+      <c r="D433" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E433" t="s">
+        <v>1010</v>
+      </c>
+      <c r="G433" t="s">
+        <v>19</v>
+      </c>
+      <c r="H433" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="434" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A434">
+        <v>432</v>
+      </c>
+      <c r="B434" t="s">
+        <v>100</v>
+      </c>
+      <c r="C434" t="s">
+        <v>30</v>
+      </c>
+      <c r="D434" t="s">
+        <v>1011</v>
+      </c>
+      <c r="E434" t="s">
+        <v>1012</v>
+      </c>
+      <c r="G434" t="s">
+        <v>19</v>
+      </c>
+      <c r="H434" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="435" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A435">
+        <v>433</v>
+      </c>
+      <c r="B435" t="s">
+        <v>181</v>
+      </c>
+      <c r="C435" t="s">
+        <v>351</v>
+      </c>
+      <c r="D435" t="s">
+        <v>1013</v>
+      </c>
+      <c r="E435" t="s">
+        <v>1014</v>
+      </c>
+      <c r="G435" t="s">
+        <v>19</v>
+      </c>
+      <c r="H435" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="436" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A436">
+        <v>434</v>
+      </c>
+      <c r="B436" t="s">
+        <v>21</v>
+      </c>
+      <c r="C436" t="s">
+        <v>45</v>
+      </c>
+      <c r="D436" t="s">
+        <v>1015</v>
+      </c>
+      <c r="E436" t="s">
+        <v>1016</v>
+      </c>
+      <c r="G436" t="s">
+        <v>19</v>
+      </c>
+      <c r="H436" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="437" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A437">
+        <v>435</v>
+      </c>
+      <c r="B437" t="s">
+        <v>181</v>
+      </c>
+      <c r="C437" t="s">
+        <v>561</v>
+      </c>
+      <c r="D437" t="s">
+        <v>1017</v>
+      </c>
+      <c r="E437" t="s">
+        <v>1018</v>
+      </c>
+      <c r="G437" t="s">
+        <v>19</v>
+      </c>
+      <c r="H437" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="438" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A438">
+        <v>436</v>
+      </c>
+      <c r="B438" t="s">
+        <v>44</v>
+      </c>
+      <c r="C438" t="s">
+        <v>432</v>
+      </c>
+      <c r="D438" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E438" t="s">
+        <v>1020</v>
+      </c>
+      <c r="G438" t="s">
+        <v>19</v>
+      </c>
+      <c r="H438" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="439" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A439">
+        <v>437</v>
+      </c>
+      <c r="B439" t="s">
+        <v>181</v>
+      </c>
+      <c r="C439" t="s">
+        <v>561</v>
+      </c>
+      <c r="D439" t="s">
+        <v>1021</v>
+      </c>
+      <c r="E439" t="s">
+        <v>1022</v>
+      </c>
+      <c r="G439" t="s">
+        <v>19</v>
+      </c>
+      <c r="H439" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="440" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A440">
+        <v>438</v>
+      </c>
+      <c r="B440" t="s">
+        <v>21</v>
+      </c>
+      <c r="C440" t="s">
+        <v>351</v>
+      </c>
+      <c r="D440" t="s">
+        <v>1023</v>
+      </c>
+      <c r="E440" t="s">
+        <v>1024</v>
+      </c>
+      <c r="G440" t="s">
+        <v>19</v>
+      </c>
+      <c r="H440" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="441" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A441">
+        <v>439</v>
+      </c>
+      <c r="B441" t="s">
+        <v>44</v>
+      </c>
+      <c r="C441" t="s">
+        <v>351</v>
+      </c>
+      <c r="D441" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E441" t="s">
+        <v>1026</v>
+      </c>
+      <c r="G441" t="s">
+        <v>19</v>
+      </c>
+      <c r="H441" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="442" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A442">
+        <v>440</v>
+      </c>
+      <c r="B442" t="s">
+        <v>44</v>
+      </c>
+      <c r="C442" t="s">
+        <v>432</v>
+      </c>
+      <c r="D442" t="s">
+        <v>1027</v>
+      </c>
+      <c r="E442" t="s">
+        <v>1028</v>
+      </c>
+      <c r="G442" t="s">
+        <v>19</v>
+      </c>
+      <c r="H442" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="443" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A443">
+        <v>441</v>
+      </c>
+      <c r="B443" t="s">
+        <v>181</v>
+      </c>
+      <c r="C443" t="s">
+        <v>79</v>
+      </c>
+      <c r="D443" t="s">
+        <v>1029</v>
+      </c>
+      <c r="E443" t="s">
+        <v>1030</v>
+      </c>
+      <c r="G443" t="s">
+        <v>19</v>
+      </c>
+      <c r="H443" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="444" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A444">
+        <v>442</v>
+      </c>
+      <c r="B444" t="s">
+        <v>100</v>
+      </c>
+      <c r="C444" t="s">
+        <v>30</v>
+      </c>
+      <c r="D444" t="s">
+        <v>1031</v>
+      </c>
+      <c r="E444" t="s">
+        <v>1032</v>
+      </c>
+      <c r="G444" t="s">
+        <v>19</v>
+      </c>
+      <c r="H444" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="445" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A445">
+        <v>443</v>
+      </c>
+      <c r="B445" t="s">
+        <v>21</v>
+      </c>
+      <c r="C445" t="s">
+        <v>45</v>
+      </c>
+      <c r="D445" t="s">
+        <v>1033</v>
+      </c>
+      <c r="E445" t="s">
+        <v>1034</v>
+      </c>
+      <c r="G445" t="s">
+        <v>19</v>
+      </c>
+      <c r="H445" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="446" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A446">
+        <v>444</v>
+      </c>
+      <c r="B446" t="s">
+        <v>21</v>
+      </c>
+      <c r="C446" t="s">
+        <v>30</v>
+      </c>
+      <c r="D446" t="s">
+        <v>1035</v>
+      </c>
+      <c r="E446" t="s">
+        <v>1036</v>
+      </c>
+      <c r="G446" t="s">
+        <v>19</v>
+      </c>
+      <c r="H446" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="447" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A447">
+        <v>445</v>
+      </c>
+      <c r="B447" t="s">
+        <v>21</v>
+      </c>
+      <c r="C447" t="s">
+        <v>45</v>
+      </c>
+      <c r="D447" t="s">
+        <v>1037</v>
+      </c>
+      <c r="E447" t="s">
+        <v>1038</v>
+      </c>
+      <c r="G447" t="s">
+        <v>19</v>
+      </c>
+      <c r="H447" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="448" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A448">
+        <v>446</v>
+      </c>
+      <c r="B448" t="s">
+        <v>181</v>
+      </c>
+      <c r="C448" t="s">
+        <v>161</v>
+      </c>
+      <c r="D448" t="s">
+        <v>1039</v>
+      </c>
+      <c r="E448" t="s">
+        <v>1040</v>
+      </c>
+      <c r="G448" t="s">
+        <v>19</v>
+      </c>
+      <c r="H448" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="449" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A449">
+        <v>447</v>
+      </c>
+      <c r="B449" t="s">
+        <v>95</v>
+      </c>
+      <c r="C449" t="s">
+        <v>21</v>
+      </c>
+      <c r="D449" t="s">
+        <v>1041</v>
+      </c>
+      <c r="E449" t="s">
+        <v>1042</v>
+      </c>
+      <c r="G449" t="s">
+        <v>19</v>
+      </c>
+      <c r="H449" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="450" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A450">
+        <v>448</v>
+      </c>
+      <c r="B450" t="s">
+        <v>342</v>
+      </c>
+      <c r="C450" t="s">
+        <v>342</v>
+      </c>
+      <c r="D450" t="s">
+        <v>1043</v>
+      </c>
+      <c r="E450" t="s">
+        <v>1044</v>
+      </c>
+      <c r="G450" t="s">
+        <v>19</v>
+      </c>
+      <c r="H450" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="451" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A451">
+        <v>449</v>
+      </c>
+      <c r="B451" t="s">
+        <v>100</v>
+      </c>
+      <c r="C451" t="s">
+        <v>30</v>
+      </c>
+      <c r="D451" t="s">
+        <v>1045</v>
+      </c>
+      <c r="E451" t="s">
+        <v>1046</v>
+      </c>
+      <c r="G451" t="s">
+        <v>19</v>
+      </c>
+      <c r="H451" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="452" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A452">
+        <v>450</v>
+      </c>
+      <c r="B452" t="s">
+        <v>247</v>
+      </c>
+      <c r="C452" t="s">
+        <v>351</v>
+      </c>
+      <c r="D452" t="s">
+        <v>1047</v>
+      </c>
+      <c r="E452" t="s">
+        <v>1048</v>
+      </c>
+      <c r="G452" t="s">
+        <v>19</v>
+      </c>
+      <c r="H452" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="453" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A453">
+        <v>451</v>
+      </c>
+      <c r="B453" t="s">
+        <v>95</v>
+      </c>
+      <c r="C453" t="s">
+        <v>193</v>
+      </c>
+      <c r="D453" t="s">
+        <v>1049</v>
+      </c>
+      <c r="E453" t="s">
+        <v>1050</v>
+      </c>
+      <c r="G453" t="s">
+        <v>19</v>
+      </c>
+      <c r="H453" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="454" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A454" s="5">
+        <v>452</v>
+      </c>
+      <c r="B454" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C454" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D454" s="6" t="s">
+        <v>1555</v>
+      </c>
+      <c r="G454" s="6" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="455" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A455" s="5">
+        <v>453</v>
+      </c>
+      <c r="B455" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C455" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D455" s="6" t="s">
+        <v>1556</v>
+      </c>
+      <c r="G455" s="6" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="456" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A456" s="5">
+        <v>454</v>
+      </c>
+      <c r="B456" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C456" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D456" s="6" t="s">
+        <v>1557</v>
+      </c>
+      <c r="G456" s="6" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="457" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A457" s="5">
+        <v>455</v>
+      </c>
+      <c r="B457" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C457" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D457" s="6" t="s">
+        <v>1558</v>
+      </c>
+      <c r="G457" s="6" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="458" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A458" s="5">
+        <v>456</v>
+      </c>
+      <c r="B458" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C458" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D458" s="6" t="s">
+        <v>1559</v>
+      </c>
+      <c r="G458" s="6" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="459" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A459" s="5">
+        <v>457</v>
+      </c>
+      <c r="B459" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C459" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D459" s="6" t="s">
+        <v>1560</v>
+      </c>
+      <c r="G459" s="6" t="s">
+        <v>1552</v>
       </c>
     </row>
   </sheetData>
@@ -16053,7 +17296,7 @@
       <formula>$G2="Manual Fix"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G83 G85:G1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>StatusList</formula1>
     </dataValidation>
@@ -16074,862 +17317,862 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>970</v>
+        <v>1051</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>971</v>
+        <v>1052</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>972</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>973</v>
+        <v>1054</v>
       </c>
       <c r="B2" t="s">
-        <v>974</v>
+        <v>1055</v>
       </c>
       <c r="C2" t="s">
-        <v>975</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>976</v>
+        <v>1057</v>
       </c>
       <c r="B3" t="s">
-        <v>977</v>
+        <v>1058</v>
       </c>
       <c r="C3" t="s">
-        <v>975</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>978</v>
+        <v>1059</v>
       </c>
       <c r="B4" t="s">
-        <v>979</v>
+        <v>1060</v>
       </c>
       <c r="C4" t="s">
-        <v>975</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>980</v>
+        <v>1061</v>
       </c>
       <c r="B5" t="s">
-        <v>981</v>
+        <v>1062</v>
       </c>
       <c r="C5" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>983</v>
+        <v>1064</v>
       </c>
       <c r="B6" t="s">
-        <v>984</v>
+        <v>1065</v>
       </c>
       <c r="C6" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>985</v>
+        <v>1066</v>
       </c>
       <c r="B7" t="s">
-        <v>986</v>
+        <v>1067</v>
       </c>
       <c r="C7" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>987</v>
+        <v>1068</v>
       </c>
       <c r="B8" t="s">
-        <v>988</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>989</v>
+        <v>1070</v>
       </c>
       <c r="B9" t="s">
-        <v>990</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>991</v>
+        <v>1072</v>
       </c>
       <c r="B10" t="s">
-        <v>992</v>
+        <v>1073</v>
       </c>
       <c r="C10" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>993</v>
+        <v>1074</v>
       </c>
       <c r="B11" t="s">
-        <v>994</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>995</v>
+        <v>1076</v>
       </c>
       <c r="B12" t="s">
-        <v>996</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>997</v>
+        <v>1078</v>
       </c>
       <c r="B13" t="s">
-        <v>998</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>999</v>
+        <v>1080</v>
       </c>
       <c r="B14" t="s">
-        <v>1000</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>1001</v>
+        <v>1082</v>
       </c>
       <c r="B15" t="s">
-        <v>1002</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>1003</v>
+        <v>1084</v>
       </c>
       <c r="B16" t="s">
-        <v>1004</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>1005</v>
+        <v>1086</v>
       </c>
       <c r="B17" t="s">
-        <v>1006</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>1007</v>
+        <v>1088</v>
       </c>
       <c r="B18" t="s">
-        <v>1008</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>1009</v>
+        <v>1090</v>
       </c>
       <c r="B19" t="s">
-        <v>1010</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>1011</v>
+        <v>1092</v>
       </c>
       <c r="B20" t="s">
-        <v>1012</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>1013</v>
+        <v>1094</v>
       </c>
       <c r="B21" t="s">
-        <v>1014</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>1015</v>
+        <v>1096</v>
       </c>
       <c r="B22" t="s">
-        <v>1016</v>
+        <v>1097</v>
       </c>
       <c r="C22" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>1017</v>
+        <v>1098</v>
       </c>
       <c r="B23" t="s">
-        <v>1018</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>1019</v>
+        <v>1100</v>
       </c>
       <c r="B24" t="s">
-        <v>1020</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1021</v>
+        <v>1102</v>
       </c>
       <c r="B25" t="s">
-        <v>1022</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>1023</v>
+        <v>1104</v>
       </c>
       <c r="B26" t="s">
-        <v>1024</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1025</v>
+        <v>1106</v>
       </c>
       <c r="B27" t="s">
-        <v>1026</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>1027</v>
+        <v>1108</v>
       </c>
       <c r="B28" t="s">
-        <v>1028</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>1029</v>
+        <v>1110</v>
       </c>
       <c r="B29" t="s">
-        <v>1030</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>1031</v>
+        <v>1112</v>
       </c>
       <c r="B30" t="s">
-        <v>1032</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>1033</v>
+        <v>1114</v>
       </c>
       <c r="B31" t="s">
-        <v>1034</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>1035</v>
+        <v>1116</v>
       </c>
       <c r="B32" t="s">
-        <v>1036</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>1037</v>
+        <v>1118</v>
       </c>
       <c r="B33" t="s">
-        <v>1038</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1039</v>
+        <v>1120</v>
       </c>
       <c r="B34" t="s">
-        <v>1040</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1041</v>
+        <v>1122</v>
       </c>
       <c r="B35" t="s">
-        <v>1042</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>1043</v>
+        <v>1124</v>
       </c>
       <c r="B36" t="s">
-        <v>1044</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>1045</v>
+        <v>1126</v>
       </c>
       <c r="B37" t="s">
-        <v>1046</v>
+        <v>1127</v>
       </c>
       <c r="C37" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1047</v>
+        <v>1128</v>
       </c>
       <c r="B38" t="s">
-        <v>1048</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>1049</v>
+        <v>1130</v>
       </c>
       <c r="B39" t="s">
-        <v>1050</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>1051</v>
+        <v>1132</v>
       </c>
       <c r="B40" t="s">
-        <v>1052</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>1053</v>
+        <v>1134</v>
       </c>
       <c r="B41" t="s">
-        <v>1054</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>1055</v>
+        <v>1136</v>
       </c>
       <c r="B42" t="s">
-        <v>1056</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1057</v>
+        <v>1138</v>
       </c>
       <c r="B43" t="s">
-        <v>1058</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>1059</v>
+        <v>1140</v>
       </c>
       <c r="B44" t="s">
-        <v>1060</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1061</v>
+        <v>1142</v>
       </c>
       <c r="B45" t="s">
-        <v>1062</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1063</v>
+        <v>1144</v>
       </c>
       <c r="B46" t="s">
-        <v>1064</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1065</v>
+        <v>1146</v>
       </c>
       <c r="B47" t="s">
-        <v>1066</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1067</v>
+        <v>1148</v>
       </c>
       <c r="B48" t="s">
-        <v>1068</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1069</v>
+        <v>1150</v>
       </c>
       <c r="B49" t="s">
-        <v>1070</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>1071</v>
+        <v>1152</v>
       </c>
       <c r="B50" t="s">
-        <v>1072</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>1073</v>
+        <v>1154</v>
       </c>
       <c r="B51" t="s">
-        <v>1074</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>1075</v>
+        <v>1156</v>
       </c>
       <c r="B52" t="s">
-        <v>1076</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>1077</v>
+        <v>1158</v>
       </c>
       <c r="B53" t="s">
-        <v>1078</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>1079</v>
+        <v>1160</v>
       </c>
       <c r="B54" t="s">
-        <v>1080</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>1081</v>
+        <v>1162</v>
       </c>
       <c r="B55" t="s">
-        <v>1082</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>1083</v>
+        <v>1164</v>
       </c>
       <c r="B56" t="s">
-        <v>1084</v>
+        <v>1165</v>
       </c>
       <c r="C56" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>1085</v>
+        <v>1166</v>
       </c>
       <c r="B57" t="s">
-        <v>1086</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>1087</v>
+        <v>1168</v>
       </c>
       <c r="B58" t="s">
-        <v>1088</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>1089</v>
+        <v>1170</v>
       </c>
       <c r="B59" t="s">
-        <v>1090</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>1091</v>
+        <v>1172</v>
       </c>
       <c r="B60" t="s">
-        <v>1092</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>1093</v>
+        <v>1174</v>
       </c>
       <c r="B61" t="s">
-        <v>1094</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>1095</v>
+        <v>1176</v>
       </c>
       <c r="B62" t="s">
-        <v>1096</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>1097</v>
+        <v>1178</v>
       </c>
       <c r="B63" t="s">
-        <v>1098</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>1099</v>
+        <v>1180</v>
       </c>
       <c r="B64" t="s">
-        <v>1100</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>1101</v>
+        <v>1182</v>
       </c>
       <c r="B65" t="s">
-        <v>1102</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>1103</v>
+        <v>1184</v>
       </c>
       <c r="B66" t="s">
-        <v>1104</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>1105</v>
+        <v>1186</v>
       </c>
       <c r="B67" t="s">
-        <v>1106</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>1107</v>
+        <v>1188</v>
       </c>
       <c r="B68" t="s">
-        <v>1108</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>1109</v>
+        <v>1190</v>
       </c>
       <c r="B69" t="s">
-        <v>1110</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>1111</v>
+        <v>1192</v>
       </c>
       <c r="B70" t="s">
-        <v>1112</v>
+        <v>1193</v>
       </c>
       <c r="C70" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>1113</v>
+        <v>1194</v>
       </c>
       <c r="B71" t="s">
-        <v>1114</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>1115</v>
+        <v>1196</v>
       </c>
       <c r="B72" t="s">
-        <v>1116</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>1117</v>
+        <v>1198</v>
       </c>
       <c r="B73" t="s">
-        <v>1118</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>1119</v>
+        <v>1200</v>
       </c>
       <c r="B74" t="s">
-        <v>1120</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>1121</v>
+        <v>1202</v>
       </c>
       <c r="B75" t="s">
-        <v>1122</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>1123</v>
+        <v>1204</v>
       </c>
       <c r="B76" t="s">
-        <v>1124</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>1125</v>
+        <v>1206</v>
       </c>
       <c r="B77" t="s">
-        <v>1126</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>1127</v>
+        <v>1208</v>
       </c>
       <c r="B78" t="s">
-        <v>1128</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>1129</v>
+        <v>1210</v>
       </c>
       <c r="B79" t="s">
-        <v>1130</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>1131</v>
+        <v>1212</v>
       </c>
       <c r="B80" t="s">
-        <v>1132</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>1133</v>
+        <v>1214</v>
       </c>
       <c r="B81" t="s">
-        <v>1134</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>1135</v>
+        <v>1216</v>
       </c>
       <c r="B82" t="s">
-        <v>1136</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>1137</v>
+        <v>1218</v>
       </c>
       <c r="B83" t="s">
-        <v>1138</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>1139</v>
+        <v>1220</v>
       </c>
       <c r="B84" t="s">
-        <v>1140</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>1141</v>
+        <v>1222</v>
       </c>
       <c r="B85" t="s">
-        <v>1142</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>1143</v>
+        <v>1224</v>
       </c>
       <c r="B86" t="s">
-        <v>1144</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>1145</v>
+        <v>1226</v>
       </c>
       <c r="B87" t="s">
-        <v>1146</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>1147</v>
+        <v>1228</v>
       </c>
       <c r="B88" t="s">
-        <v>1148</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>1149</v>
+        <v>1230</v>
       </c>
       <c r="B89" t="s">
-        <v>1150</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>1151</v>
+        <v>1232</v>
       </c>
       <c r="B90" t="s">
-        <v>1152</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>1153</v>
+        <v>1234</v>
       </c>
       <c r="B91" t="s">
-        <v>1154</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>1155</v>
+        <v>1236</v>
       </c>
       <c r="B92" t="s">
-        <v>1156</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1157</v>
+        <v>1238</v>
       </c>
       <c r="B93" t="s">
-        <v>1158</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>1159</v>
+        <v>1240</v>
       </c>
       <c r="B94" t="s">
-        <v>1160</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>1161</v>
+        <v>1242</v>
       </c>
       <c r="B95" t="s">
-        <v>1162</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>1163</v>
+        <v>1244</v>
       </c>
       <c r="B96" t="s">
-        <v>1164</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>1165</v>
+        <v>1246</v>
       </c>
       <c r="B97" t="s">
-        <v>1166</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>1167</v>
+        <v>1248</v>
       </c>
       <c r="B98" t="s">
-        <v>1168</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>1169</v>
+        <v>1250</v>
       </c>
       <c r="B99" t="s">
-        <v>1170</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>1171</v>
+        <v>1252</v>
       </c>
       <c r="B100" t="s">
-        <v>1172</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1173</v>
+        <v>1254</v>
       </c>
       <c r="B101" t="s">
-        <v>1174</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1175</v>
+        <v>1256</v>
       </c>
       <c r="B102" t="s">
-        <v>1176</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1177</v>
+        <v>1258</v>
       </c>
       <c r="B103" t="s">
-        <v>1178</v>
+        <v>1259</v>
       </c>
     </row>
   </sheetData>
@@ -16964,400 +18207,400 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>970</v>
+        <v>1051</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>971</v>
+        <v>1052</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>972</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1179</v>
+        <v>1260</v>
       </c>
       <c r="B2" t="s">
-        <v>1180</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1181</v>
+        <v>1262</v>
       </c>
       <c r="B3" t="s">
-        <v>1024</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1182</v>
+        <v>1263</v>
       </c>
       <c r="B4" t="s">
-        <v>1183</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1184</v>
+        <v>1265</v>
       </c>
       <c r="B5" t="s">
-        <v>1185</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1186</v>
+        <v>1267</v>
       </c>
       <c r="B6" t="s">
-        <v>1187</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1188</v>
+        <v>1269</v>
       </c>
       <c r="B7" t="s">
-        <v>1189</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1190</v>
+        <v>1271</v>
       </c>
       <c r="B8" t="s">
-        <v>1191</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1192</v>
+        <v>1273</v>
       </c>
       <c r="B9" t="s">
-        <v>1193</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1194</v>
+        <v>1275</v>
       </c>
       <c r="B10" t="s">
-        <v>1195</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1196</v>
+        <v>1277</v>
       </c>
       <c r="B11" t="s">
-        <v>1197</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1198</v>
+        <v>1279</v>
       </c>
       <c r="B12" t="s">
-        <v>1199</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1200</v>
+        <v>1281</v>
       </c>
       <c r="B13" t="s">
-        <v>1201</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1202</v>
+        <v>1283</v>
       </c>
       <c r="B14" t="s">
-        <v>1203</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>1204</v>
+        <v>1285</v>
       </c>
       <c r="B15" t="s">
-        <v>1205</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>1206</v>
+        <v>1287</v>
       </c>
       <c r="B16" t="s">
-        <v>1207</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>1208</v>
+        <v>1289</v>
       </c>
       <c r="B17" t="s">
-        <v>1209</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>1210</v>
+        <v>1291</v>
       </c>
       <c r="B18" t="s">
-        <v>1211</v>
+        <v>1292</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>982</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>1212</v>
+        <v>1293</v>
       </c>
       <c r="B19" t="s">
-        <v>1213</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>1214</v>
+        <v>1295</v>
       </c>
       <c r="B20" t="s">
-        <v>1215</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>1216</v>
+        <v>1297</v>
       </c>
       <c r="B21" t="s">
-        <v>1217</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>1218</v>
+        <v>1299</v>
       </c>
       <c r="B22" t="s">
-        <v>1219</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>1220</v>
+        <v>1301</v>
       </c>
       <c r="B23" t="s">
-        <v>1221</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>1222</v>
+        <v>1303</v>
       </c>
       <c r="B24" t="s">
-        <v>1223</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1224</v>
+        <v>1305</v>
       </c>
       <c r="B25" t="s">
-        <v>1225</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>1226</v>
+        <v>1307</v>
       </c>
       <c r="B26" t="s">
-        <v>1227</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1228</v>
+        <v>1309</v>
       </c>
       <c r="B27" t="s">
-        <v>1229</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>1230</v>
+        <v>1311</v>
       </c>
       <c r="B28" t="s">
-        <v>1231</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>1232</v>
+        <v>1313</v>
       </c>
       <c r="B29" t="s">
-        <v>1233</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>1234</v>
+        <v>1315</v>
       </c>
       <c r="B30" t="s">
-        <v>1235</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>1236</v>
+        <v>1317</v>
       </c>
       <c r="B31" t="s">
-        <v>1237</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>1238</v>
+        <v>1319</v>
       </c>
       <c r="B32" t="s">
-        <v>1239</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>1240</v>
+        <v>1321</v>
       </c>
       <c r="B33" t="s">
-        <v>1241</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1242</v>
+        <v>1323</v>
       </c>
       <c r="B34" t="s">
-        <v>1243</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1244</v>
+        <v>1325</v>
       </c>
       <c r="B35" t="s">
-        <v>1245</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>1246</v>
+        <v>1327</v>
       </c>
       <c r="B36" t="s">
-        <v>1247</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>1248</v>
+        <v>1329</v>
       </c>
       <c r="B37" t="s">
-        <v>1249</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1250</v>
+        <v>1331</v>
       </c>
       <c r="B38" t="s">
-        <v>1251</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>1252</v>
+        <v>1333</v>
       </c>
       <c r="B39" t="s">
-        <v>1253</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>1254</v>
+        <v>1335</v>
       </c>
       <c r="B40" t="s">
-        <v>1255</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>1256</v>
+        <v>1337</v>
       </c>
       <c r="B41" t="s">
-        <v>1257</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>1258</v>
+        <v>1339</v>
       </c>
       <c r="B42" t="s">
-        <v>1259</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1260</v>
+        <v>1341</v>
       </c>
       <c r="B43" t="s">
-        <v>1261</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>1262</v>
+        <v>1343</v>
       </c>
       <c r="B44" t="s">
-        <v>1263</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1264</v>
+        <v>1345</v>
       </c>
       <c r="B45" t="s">
-        <v>1092</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1265</v>
+        <v>1346</v>
       </c>
       <c r="B46" t="s">
-        <v>1266</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1267</v>
+        <v>1348</v>
       </c>
       <c r="B47" t="s">
-        <v>1268</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1269</v>
+        <v>1350</v>
       </c>
       <c r="B48" t="s">
-        <v>1270</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1271</v>
+        <v>1352</v>
       </c>
       <c r="B49" t="s">
-        <v>1272</v>
+        <v>1353</v>
       </c>
     </row>
   </sheetData>
@@ -17388,389 +18631,389 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>970</v>
+        <v>1051</v>
       </c>
       <c r="B1" t="s">
-        <v>971</v>
+        <v>1052</v>
       </c>
       <c r="C1" t="s">
-        <v>972</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1273</v>
+        <v>1354</v>
       </c>
       <c r="B2" t="s">
-        <v>1274</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1275</v>
+        <v>1356</v>
       </c>
       <c r="B3" t="s">
-        <v>1276</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1277</v>
+        <v>1358</v>
       </c>
       <c r="B4" t="s">
-        <v>1278</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1279</v>
+        <v>1360</v>
       </c>
       <c r="B5" t="s">
-        <v>1280</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1281</v>
+        <v>1362</v>
       </c>
       <c r="B6" t="s">
-        <v>1282</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1283</v>
+        <v>1364</v>
       </c>
       <c r="B7" t="s">
-        <v>1040</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1284</v>
+        <v>1365</v>
       </c>
       <c r="B8" t="s">
-        <v>1285</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1286</v>
+        <v>1367</v>
       </c>
       <c r="B9" t="s">
-        <v>1287</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1288</v>
+        <v>1369</v>
       </c>
       <c r="B10" t="s">
-        <v>1289</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1290</v>
+        <v>1371</v>
       </c>
       <c r="B11" t="s">
-        <v>1291</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1292</v>
+        <v>1373</v>
       </c>
       <c r="B12" t="s">
-        <v>1000</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1293</v>
+        <v>1374</v>
       </c>
       <c r="B13" t="s">
-        <v>1294</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1295</v>
+        <v>1376</v>
       </c>
       <c r="B14" t="s">
-        <v>1296</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>1297</v>
+        <v>1378</v>
       </c>
       <c r="B15" t="s">
-        <v>1010</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>1298</v>
+        <v>1379</v>
       </c>
       <c r="B16" t="s">
-        <v>1014</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>1299</v>
+        <v>1380</v>
       </c>
       <c r="B17" t="s">
-        <v>1300</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>1301</v>
+        <v>1382</v>
       </c>
       <c r="B18" t="s">
-        <v>1302</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>1303</v>
+        <v>1384</v>
       </c>
       <c r="B19" t="s">
-        <v>1076</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>1304</v>
+        <v>1385</v>
       </c>
       <c r="B20" t="s">
-        <v>1305</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>1306</v>
+        <v>1387</v>
       </c>
       <c r="B21" t="s">
-        <v>1307</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>1308</v>
+        <v>1389</v>
       </c>
       <c r="B22" t="s">
-        <v>1309</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>1310</v>
+        <v>1391</v>
       </c>
       <c r="B23" t="s">
-        <v>1311</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>1312</v>
+        <v>1393</v>
       </c>
       <c r="B24" t="s">
-        <v>1313</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1314</v>
+        <v>1395</v>
       </c>
       <c r="B25" t="s">
-        <v>1052</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>1315</v>
+        <v>1396</v>
       </c>
       <c r="B26" t="s">
-        <v>1316</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1317</v>
+        <v>1398</v>
       </c>
       <c r="B27" t="s">
-        <v>1318</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>1319</v>
+        <v>1400</v>
       </c>
       <c r="B28" t="s">
-        <v>1320</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>1321</v>
+        <v>1402</v>
       </c>
       <c r="B29" t="s">
-        <v>1322</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>1323</v>
+        <v>1404</v>
       </c>
       <c r="B30" t="s">
-        <v>1324</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>1325</v>
+        <v>1406</v>
       </c>
       <c r="B31" t="s">
-        <v>1326</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>1327</v>
+        <v>1408</v>
       </c>
       <c r="B32" t="s">
-        <v>1328</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>1329</v>
+        <v>1410</v>
       </c>
       <c r="B33" t="s">
-        <v>1330</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1331</v>
+        <v>1412</v>
       </c>
       <c r="B34" t="s">
-        <v>1332</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1333</v>
+        <v>1414</v>
       </c>
       <c r="B35" t="s">
-        <v>1334</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>1335</v>
+        <v>1416</v>
       </c>
       <c r="B36" t="s">
-        <v>1336</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>1337</v>
+        <v>1418</v>
       </c>
       <c r="B37" t="s">
-        <v>1338</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1339</v>
+        <v>1420</v>
       </c>
       <c r="B38" t="s">
-        <v>1340</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>1341</v>
+        <v>1422</v>
       </c>
       <c r="B39" t="s">
-        <v>1342</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>1343</v>
+        <v>1424</v>
       </c>
       <c r="B40" t="s">
-        <v>1344</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>1345</v>
+        <v>1426</v>
       </c>
       <c r="B41" t="s">
-        <v>1346</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>1347</v>
+        <v>1428</v>
       </c>
       <c r="B42" t="s">
-        <v>1348</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1349</v>
+        <v>1430</v>
       </c>
       <c r="B43" t="s">
-        <v>1350</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>1351</v>
+        <v>1432</v>
       </c>
       <c r="B44" t="s">
-        <v>1352</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1353</v>
+        <v>1434</v>
       </c>
       <c r="B45" t="s">
-        <v>1354</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1355</v>
+        <v>1436</v>
       </c>
       <c r="B46" t="s">
-        <v>1356</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1357</v>
+        <v>1438</v>
       </c>
       <c r="B47" t="s">
-        <v>1358</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1359</v>
+        <v>1440</v>
       </c>
       <c r="B48" t="s">
-        <v>1360</v>
+        <v>1441</v>
       </c>
     </row>
   </sheetData>
@@ -17801,541 +19044,541 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>970</v>
+        <v>1051</v>
       </c>
       <c r="B1" t="s">
-        <v>971</v>
+        <v>1052</v>
       </c>
       <c r="C1" t="s">
-        <v>972</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1361</v>
+        <v>1442</v>
       </c>
       <c r="B2" t="s">
-        <v>1362</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1363</v>
+        <v>1444</v>
       </c>
       <c r="B3" t="s">
-        <v>1364</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1365</v>
+        <v>1446</v>
       </c>
       <c r="B4" t="s">
-        <v>1366</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1367</v>
+        <v>1448</v>
       </c>
       <c r="B5" t="s">
-        <v>1368</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1369</v>
+        <v>1450</v>
       </c>
       <c r="B6" t="s">
-        <v>1370</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1371</v>
+        <v>1452</v>
       </c>
       <c r="B7" t="s">
-        <v>1372</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1373</v>
+        <v>1454</v>
       </c>
       <c r="B8" t="s">
-        <v>1374</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1375</v>
+        <v>1456</v>
       </c>
       <c r="B9" t="s">
-        <v>1376</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1377</v>
+        <v>1458</v>
       </c>
       <c r="B10" t="s">
-        <v>1378</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1379</v>
+        <v>1460</v>
       </c>
       <c r="B11" t="s">
-        <v>1380</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1381</v>
+        <v>1462</v>
       </c>
       <c r="B12" t="s">
-        <v>1382</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1383</v>
+        <v>1464</v>
       </c>
       <c r="B13" t="s">
-        <v>1384</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1385</v>
+        <v>1466</v>
       </c>
       <c r="B14" t="s">
-        <v>1386</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>1387</v>
+        <v>1468</v>
       </c>
       <c r="B15" t="s">
-        <v>1388</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>1389</v>
+        <v>1470</v>
       </c>
       <c r="B16" t="s">
-        <v>1390</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>1391</v>
+        <v>1472</v>
       </c>
       <c r="B17" t="s">
-        <v>1392</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>1393</v>
+        <v>1474</v>
       </c>
       <c r="B18" t="s">
-        <v>1394</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>1395</v>
+        <v>1476</v>
       </c>
       <c r="B19" t="s">
-        <v>1396</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>1397</v>
+        <v>1478</v>
       </c>
       <c r="B20" t="s">
-        <v>1398</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>1399</v>
+        <v>1480</v>
       </c>
       <c r="B21" t="s">
-        <v>1400</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>1401</v>
+        <v>1482</v>
       </c>
       <c r="B22" t="s">
-        <v>1402</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>1403</v>
+        <v>1484</v>
       </c>
       <c r="B23" t="s">
-        <v>1404</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>1405</v>
+        <v>1486</v>
       </c>
       <c r="B24" t="s">
-        <v>1406</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1407</v>
+        <v>1488</v>
       </c>
       <c r="B25" t="s">
-        <v>1408</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>1409</v>
+        <v>1490</v>
       </c>
       <c r="B26" t="s">
-        <v>1410</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1411</v>
+        <v>1492</v>
       </c>
       <c r="B27" t="s">
-        <v>1412</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>1413</v>
+        <v>1494</v>
       </c>
       <c r="B28" t="s">
-        <v>1414</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>1415</v>
+        <v>1496</v>
       </c>
       <c r="B29" t="s">
-        <v>1416</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>1417</v>
+        <v>1498</v>
       </c>
       <c r="B30" t="s">
-        <v>1418</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>1419</v>
+        <v>1500</v>
       </c>
       <c r="B31" t="s">
-        <v>1420</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>1421</v>
+        <v>1502</v>
       </c>
       <c r="B32" t="s">
-        <v>1422</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>1423</v>
+        <v>1504</v>
       </c>
       <c r="B33" t="s">
-        <v>1424</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1425</v>
+        <v>1506</v>
       </c>
       <c r="B34" t="s">
-        <v>1050</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1426</v>
+        <v>1507</v>
       </c>
       <c r="B35" t="s">
-        <v>1058</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>1427</v>
+        <v>1508</v>
       </c>
       <c r="B36" t="s">
-        <v>984</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>1428</v>
+        <v>1509</v>
       </c>
       <c r="B37" t="s">
-        <v>1068</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1429</v>
+        <v>1510</v>
       </c>
       <c r="B38" t="s">
-        <v>1430</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>1431</v>
+        <v>1512</v>
       </c>
       <c r="B39" t="s">
-        <v>1070</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>1432</v>
+        <v>1513</v>
       </c>
       <c r="B40" t="s">
-        <v>1034</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>1433</v>
+        <v>1514</v>
       </c>
       <c r="B41" t="s">
-        <v>1074</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>1434</v>
+        <v>1515</v>
       </c>
       <c r="B42" t="s">
-        <v>1247</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1435</v>
+        <v>1516</v>
       </c>
       <c r="B43" t="s">
-        <v>1328</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>1436</v>
+        <v>1517</v>
       </c>
       <c r="B44" t="s">
-        <v>1332</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1437</v>
+        <v>1518</v>
       </c>
       <c r="B45" t="s">
-        <v>1078</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1438</v>
+        <v>1519</v>
       </c>
       <c r="B46" t="s">
-        <v>1080</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1439</v>
+        <v>1520</v>
       </c>
       <c r="B47" t="s">
-        <v>1082</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1440</v>
+        <v>1521</v>
       </c>
       <c r="B48" t="s">
-        <v>1255</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1441</v>
+        <v>1522</v>
       </c>
       <c r="B49" t="s">
-        <v>1257</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>1442</v>
+        <v>1523</v>
       </c>
       <c r="B50" t="s">
-        <v>1261</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>1443</v>
+        <v>1524</v>
       </c>
       <c r="B51" t="s">
-        <v>1096</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>1444</v>
+        <v>1525</v>
       </c>
       <c r="B52" t="s">
-        <v>1342</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>1445</v>
+        <v>1526</v>
       </c>
       <c r="B53" t="s">
-        <v>1098</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>1446</v>
+        <v>1527</v>
       </c>
       <c r="B54" t="s">
-        <v>1346</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>1447</v>
+        <v>1528</v>
       </c>
       <c r="B55" t="s">
-        <v>986</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>1448</v>
+        <v>1529</v>
       </c>
       <c r="B56" t="s">
-        <v>1108</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>1449</v>
+        <v>1530</v>
       </c>
       <c r="B57" t="s">
-        <v>1350</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>1450</v>
+        <v>1531</v>
       </c>
       <c r="B58" t="s">
-        <v>1451</v>
+        <v>1532</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>1452</v>
+        <v>1533</v>
       </c>
       <c r="B59" t="s">
-        <v>1453</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>1454</v>
+        <v>1535</v>
       </c>
       <c r="B60" t="s">
-        <v>1455</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>1456</v>
+        <v>1537</v>
       </c>
       <c r="B61" t="s">
-        <v>1457</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>1458</v>
+        <v>1539</v>
       </c>
       <c r="B62" t="s">
-        <v>1459</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>1460</v>
+        <v>1541</v>
       </c>
       <c r="B63" t="s">
-        <v>1461</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>1462</v>
+        <v>1543</v>
       </c>
       <c r="B64" t="s">
-        <v>1463</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>1464</v>
+        <v>1545</v>
       </c>
       <c r="B65" t="s">
-        <v>1465</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>1466</v>
+        <v>1547</v>
       </c>
       <c r="B66" t="s">
-        <v>1467</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>1468</v>
+        <v>1549</v>
       </c>
       <c r="B67" t="s">
-        <v>1469</v>
+        <v>1550</v>
       </c>
     </row>
   </sheetData>
@@ -18364,12 +19607,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>1470</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1471</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -18384,7 +19627,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1472</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -18399,7 +19642,7 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1473</v>
+        <v>1554</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Story: Added story for day 2 morning and afternoon.
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708C23A2-2DB1-4C5C-A224-C85FA7130D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14715" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,20 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Game_Issues!$A$1:$I$79</definedName>
     <definedName name="StatusList">'Data Validation'!$A$2:$A$8</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>

<commit_message>
Debug: Added card animations, polished café cutscenes & tutorials. Multiple bug fixes
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game_Issues'!$A$1:$I$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base1'!$A$1:$C$103</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J471"/>
+  <dimension ref="A1:J510"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -700,8 +700,8 @@
     <col width="19" customWidth="1" style="6" min="7" max="7"/>
     <col hidden="1" width="11.140625" customWidth="1" style="7" min="8" max="9"/>
     <col hidden="1" width="16" customWidth="1" style="7" min="10" max="10"/>
-    <col width="9.140625" customWidth="1" style="7" min="11" max="29"/>
-    <col width="9.140625" customWidth="1" style="7" min="30" max="16384"/>
+    <col width="9.140625" customWidth="1" style="7" min="11" max="30"/>
+    <col width="9.140625" customWidth="1" style="7" min="31" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16236,6 +16236,11 @@
           <t>Manual Fix</t>
         </is>
       </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="385" ht="30" customHeight="1">
       <c r="A385" s="5" t="n">
@@ -17429,17 +17434,32 @@
       </c>
       <c r="B415" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C415" s="5" t="inlineStr">
         <is>
-          <t>Aesthetic</t>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Intro redesign: 4 familiarity starts (new / rules / played / expert + Hard Mode) with different start days, phone calls, decks, Olly instead of Ellie, no moving-in, starter box and shop starter set removed, new tutorial system (scripted / guided / generic), Options toggle for tutorial messages, hard mode no rematches and no x3.</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>[21/10/2026] GameState INTRO_PROFILES + ARRIVAL NIGHT + OLLY'S INTRO sections; Olly_Intro_Cutscene.gd (arrival, deck choice IntroDeckChoice, Hard Mode draft + deck builder draft mode, forced battle with per-fight overrides, post-match gifts); Tutorial_Director.gd (stacked decks, gates, messages, labels); Phone_Calls.json intro_call_*; Shopkeeper date-based greetings; MapManager no-rematch notice; outro time advance + hard mode cash.</t>
         </is>
       </c>
       <c r="G415" s="6" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
         </is>
       </c>
     </row>
@@ -17454,17 +17474,17 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Logic</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>Intro redesign: 4 familiarity starts (new / rules / played / expert + Hard Mode) with different start days, phone calls, decks, Olly instead of Ellie, no moving-in, starter box and shop starter set removed, new tutorial system (scripted / guided / generic), Options toggle for tutorial messages, hard mode no rematches and no x3.</t>
+          <t>Time advance: day 1 = 2 battles per time slot (incl. Olly), day 2 = 3, day 3+ = 4. Days 1-2 count new wins only; day 3+ every match (wins, losses, rematches).</t>
         </is>
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>[21/10/2026] GameState INTRO_PROFILES + ARRIVAL NIGHT + OLLY'S INTRO sections; Olly_Intro_Cutscene.gd (arrival, deck choice IntroDeckChoice, Hard Mode draft + deck builder draft mode, forced battle with per-fight overrides, post-match gifts); Tutorial_Director.gd (stacked decks, gates, messages, labels); Phone_Calls.json intro_call_*; Shopkeeper date-based greetings; MapManager no-rematch notice; outro time advance + hard mode cash.</t>
+          <t>[21/10/2026] GameState.matches_to_advance_time() 2/3/4 and count_match_toward_time(); outro calls it once per finished match.</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -17484,22 +17504,22 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Logic</t>
+          <t>Rewording</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Time advance: day 1 = 2 battles per time slot (incl. Olly), day 2 = 3, day 3+ = 4. Days 1-2 count new wins only; day 3+ every match (wins, losses, rematches).</t>
+          <t>Day 1: Olly should not say Ellie is at the pier. Newby farewell: 'El has gone out for the day and is back tonight, Alexander is covering the shop for me this evening...'. Olly always says 'Alexander', never 'Alex'.</t>
         </is>
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>[21/10/2026] GameState.matches_to_advance_time() 2/3/4 and count_match_toward_time(); outro calls it once per finished match.</t>
+          <t>[21/10/2026] Olly_Intro_Cutscene LINES_NEW_GOODBYE / LINES_RULES_GOODBYE rewritten; FISH rota day 1 = Olly M,A / Alexander E,N to match.</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -17519,22 +17539,22 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Rewording</t>
+          <t>New Functionality</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Day 1: Olly should not say Ellie is at the pier. Newby farewell: 'El has gone out for the day and is back tonight, Alexander is covering the shop for me this evening...'. Olly always says 'Alexander', never 'Alex'.</t>
+          <t>'I know the rules a bit' start: arrive evening 1 (not night 0), new phone call (tournament finished early, Olly comes round now), player stops short of the door facing up during the call, Olly runs in when he hangs up; 'Hey!' opener; after the match 'Alexander is covering the shop... pick up that rod from him'.</t>
         </is>
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>[21/10/2026] Olly_Intro_Cutscene LINES_NEW_GOODBYE / LINES_RULES_GOODBYE rewritten; FISH rota day 1 = Olly M,A / Alexander E,N to match.</t>
+          <t>[21/10/2026] INTRO_PROFILES rules = start_date 1 Evening, olly_meets 'taxi'; intro_call_rules; Celeste_Harbour._hand_over_to_olly(); LINES_OPEN_EVENING / LINES_RULES_GOODBYE.</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -17554,7 +17574,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>Overworld</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -17564,12 +17584,12 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>'I know the rules a bit' start: arrive evening 1 (not night 0), new phone call (tournament finished early, Olly comes round now), player stops short of the door facing up during the call, Olly runs in when he hangs up; 'Hey!' opener; after the match 'Alexander is covering the shop... pick up that rod from him'.</t>
+          <t>FISH first-visit intro should be played by whoever is behind the counter; Alexander tells it in the third person about Olly.</t>
         </is>
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>[21/10/2026] INTRO_PROFILES rules = start_date 1 Evening, olly_meets 'taxi'; intro_call_rules; Celeste_Harbour._hand_over_to_olly(); LINES_OPEN_EVENING / LINES_RULES_GOODBYE.</t>
+          <t>[21/10/2026] Fish_Shop_Intro_Cutscene takes name/sprite/colour from the scheduled keeper; LINES_*_ALEXANDER variants.</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
@@ -17589,22 +17609,22 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Overworld</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Rewording</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>FISH first-visit intro should be played by whoever is behind the counter; Alexander tells it in the third person about Olly.</t>
+          <t>FISH intro: drop the 'took over FISH a couple of months back' line; the player has just picked fishing up for the first time ('I knew you'd come round to fishing eventually', 'You'll probably be really good at it...', 'Good luck!').</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>[21/10/2026] Fish_Shop_Intro_Cutscene takes name/sprite/colour from the scheduled keeper; LINES_*_ALEXANDER variants.</t>
+          <t>[21/10/2026] Removed the takeover line from both keepers' pitches; reworded the 'used to love fishing' lines and the closing lines.</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
@@ -17624,22 +17644,22 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Rewording</t>
+          <t>Aesthetic</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>FISH intro: drop the 'took over FISH a couple of months back' line; the player has just picked fishing up for the first time ('I knew you'd come round to fishing eventually', 'You'll probably be really good at it...', 'Good luck!').</t>
+          <t>Starting a new game the taxi intro showed evening colours instead of night (lights were on).</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>[21/10/2026] Removed the takeover line from both keepers' pitches; reworded the 'used to love fishing' lines and the closing lines.</t>
+          <t>[21/10/2026] Celeste_Harbour taxi path skipped BaseMapScene._ready, so the time-of-day grade was never applied; it now calls _setup_time_of_day_grade() and TimeOfDayGrade.style_lights().</t>
         </is>
       </c>
       <c r="G421" t="inlineStr">
@@ -17659,22 +17679,22 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Overworld</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Aesthetic</t>
+          <t>Sequence Break</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Starting a new game the taxi intro showed evening colours instead of night (lights were on).</t>
+          <t>Taxi intro: remove the pause at the door when the phone call is already over.</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>[21/10/2026] Celeste_Harbour taxi path skipped BaseMapScene._ready, so the time-of-day grade was never applied; it now calls _setup_time_of_day_grade() and TimeOfDayGrade.style_lights().</t>
+          <t>[21/10/2026] INTRO_UNLOCK_PAUSE removed; only a call still running gets the look-down / look-up / short pause.</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
@@ -17694,22 +17714,22 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Overworld</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Sequence Break</t>
+          <t>Messages</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Taxi intro: remove the pause at the door when the phone call is already over.</t>
+          <t>After reading Mum's note show 'I'll call mum tomorrow...'.</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>[21/10/2026] INTRO_UNLOCK_PAUSE removed; only a call still running gets the look-down / look-up / short pause.</t>
+          <t>[21/10/2026] Player_House_Downstairs NOTE_AFTER_TEXT shown when the note closes.</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
@@ -17729,22 +17749,22 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Messages</t>
+          <t>Aesthetic</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>After reading Mum's note show 'I'll call mum tomorrow...'.</t>
+          <t>When the starter deck is gifted show the deck box art (starterdeck1_a-d), fading in, instead of spinning cards.</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>[21/10/2026] Player_House_Downstairs NOTE_AFTER_TEXT shown when the note closes.</t>
+          <t>[21/10/2026] MapManager.show_pack_reveal() (new 'pack' gift kind, card-box size, fade-in); Olly_Intro_Cutscene DECK_ART_*. Bonus packs use it too.</t>
         </is>
       </c>
       <c r="G424" t="inlineStr">
@@ -17769,17 +17789,17 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Aesthetic</t>
+          <t>Player input</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>When the starter deck is gifted show the deck box art (starterdeck1_a-d), fading in, instead of spinning cards.</t>
+          <t>'You got the starter deck!' screen could not be clicked away (Enter worked).</t>
         </is>
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>[21/10/2026] MapManager.show_pack_reveal() (new 'pack' gift kind, card-box size, fade-in); Olly_Intro_Cutscene DECK_ART_*. Bonus packs use it too.</t>
+          <t>[21/10/2026] The gift reveal's dim overlay stayed MOUSE_FILTER_STOP after the reveal, swallowing every click; it is set back to IGNORE when the reveal ends, and 'pack' got a reveal duration.</t>
         </is>
       </c>
       <c r="G425" t="inlineStr">
@@ -17804,17 +17824,17 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Player input</t>
+          <t>Aesthetic</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>'You got the starter deck!' screen could not be clicked away (Enter worked).</t>
+          <t>Deck choice decks should fly and fade in from the bottom one after another (1s each, 0.5s apart), replayed after a No; coin choices: heads flies in from the left, tails from the right, meeting in the middle.</t>
         </is>
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>[21/10/2026] The gift reveal's dim overlay stayed MOUSE_FILTER_STOP after the reveal, swallowing every click; it is set back to IGNORE when the reveal ends, and 'pack' got a reveal duration.</t>
+          <t>[21/10/2026] IntroDeckChoice._play_entrance(); choose_heads_or_tails() coin fly-in. Clicks wait until they land.</t>
         </is>
       </c>
       <c r="G426" t="inlineStr">
@@ -17844,12 +17864,12 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Deck choice decks should fly and fade in from the bottom one after another (1s each, 0.5s apart), replayed after a No; coin choices: heads flies in from the left, tails from the right, meeting in the middle.</t>
+          <t>In a match the message box should be fully opaque so the board under it doesn't make it hard to read.</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>[21/10/2026] IntroDeckChoice._play_entrance(); choose_heads_or_tails() coin fly-in. Clicks wait until they land.</t>
+          <t>[21/10/2026] DynamicMessageBox.set_fill_alpha(); MATCH_MSGBOX_FILL_ALPHA 1.0 (overworld box unchanged at 94%).</t>
         </is>
       </c>
       <c r="G427" t="inlineStr">
@@ -17869,22 +17889,22 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Aesthetic</t>
+          <t>Logic</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>In a match the message box should be fully opaque so the board under it doesn't make it hard to read.</t>
+          <t>Quitting the tutorial match mid-way counted as a loss. Checkpoints only at stepping outside and at win/loss; quitting before that resets to stepping outside (deck choice can be changed, Hard Mode packs re-roll; pack cards only kept once the deck is saved).</t>
         </is>
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>[21/10/2026] DynamicMessageBox.set_fill_alpha(); MATCH_MSGBOX_FILL_ALPHA 1.0 (overworld box unchanged at 94%).</t>
+          <t>[21/10/2026] GameState INTRO CHECKPOINT: slot files copied when Olly's scene starts (and when the Hard Mode deck is saved), restored by load_slot() until the outro decides the match; bonus pack given once only.</t>
         </is>
       </c>
       <c r="G428" t="inlineStr">
@@ -17904,22 +17924,22 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>Animation</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>Logic</t>
+          <t>New Functionality</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Quitting the tutorial match mid-way counted as a loss. Checkpoints only at stepping outside and at win/loss; quitting before that resets to stepping outside (deck choice can be changed, Hard Mode packs re-roll; pack cards only kept once the deck is saved).</t>
+          <t>Match start transition: the overworld breaks into pixels and dissolves away, the intro background dissolves in the same way, sprites/names keep their fly/fade at double time; then made 3x quicker and the pause before it removed.</t>
         </is>
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>[21/10/2026] GameState INTRO CHECKPOINT: slot files copied when Olly's scene starts (and when the Hard Mode deck is saved), restored by load_slot() until the outro decides the match; bonus pack given once only.</t>
+          <t>[21/10/2026] Pixel_Dissolve.gdshader + PixelDissolve.gd (reads the live screen, no snapshot stall); OUT_TIME 0.55 / IN_TIME 0.47; Match_Start_Intro ENTRANCE_SCALE 2.0 with BattleFrame.fade_foreground.</t>
         </is>
       </c>
       <c r="G429" t="inlineStr">
@@ -17939,22 +17959,22 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Animation</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Messages</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Match start transition: the overworld breaks into pixels and dissolves away, the intro background dissolves in the same way, sprites/names keep their fly/fade at double time; then made 3x quicker and the pause before it removed.</t>
+          <t>Punctuation pauses only for NPC / opponent / shop / cutscene speech (overworld and intro/outro), not for system messages, signs or in-match messages.</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>[21/10/2026] Pixel_Dissolve.gdshader + PixelDissolve.gd (reads the live screen, no snapshot stall); OUT_TIME 0.55 / IN_TIME 0.47; Match_Start_Intro ENTRANCE_SCALE 2.0 with BattleFrame.fade_foreground.</t>
+          <t>[21/10/2026] DynamicMessageBox._build_pauses() returns early for the system variant or a box with no speaker name pill.</t>
         </is>
       </c>
       <c r="G430" t="inlineStr">
@@ -17974,22 +17994,22 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Messages</t>
+          <t>Aesthetic</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Punctuation pauses only for NPC / opponent / shop / cutscene speech (overworld and intro/outro), not for system messages, signs or in-match messages.</t>
+          <t>Buttons (e.g. the big Cancel) drew over the in-match message box when a pile was opened.</t>
         </is>
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>[21/10/2026] DynamicMessageBox._build_pauses() returns early for the system variant or a box with no speaker name pill.</t>
+          <t>[21/10/2026] msgbox_container z_index raised to Z_CHROME + 25 (above the footer buttons and tutorial captions; draw order only).</t>
         </is>
       </c>
       <c r="G431" t="inlineStr">
@@ -18009,22 +18029,22 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>Aesthetic</t>
+          <t>Player input</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Buttons (e.g. the big Cancel) drew over the in-match message box when a pile was opened.</t>
+          <t>Clicking a deck can't view it, so remove the tutorial 'you are viewing your deck' message on deck clicks.</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>[21/10/2026] msgbox_container z_index raised to Z_CHROME + 25 (above the footer buttons and tutorial captions; draw order only).</t>
+          <t>[21/10/2026] Deck icon click handler and both deck PILE_LINES removed.</t>
         </is>
       </c>
       <c r="G432" t="inlineStr">
@@ -18044,22 +18064,22 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>Player input</t>
+          <t>Messages</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Clicking a deck can't view it, so remove the tutorial 'you are viewing your deck' message on deck clicks.</t>
+          <t>Tutorial pile messages (bench, prizes, discard, opponent hand) repeat on every click until the end of the player's first turn, then only show for a pile not yet explained.</t>
         </is>
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>[21/10/2026] Deck icon click handler and both deck PILE_LINES removed.</t>
+          <t>[21/10/2026] Tutorial_Director.on_pile_viewed(); new prize-card lines added.</t>
         </is>
       </c>
       <c r="G433" t="inlineStr">
@@ -18079,22 +18099,22 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Messages</t>
+          <t>New Functionality</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Tutorial pile messages (bench, prizes, discard, opponent hand) repeat on every click until the end of the player's first turn, then only show for a pile not yet explained.</t>
+          <t>For a newby player, their SECOND match plays the start-of-turn key tips (Shift preview, Caps Lock log, Escape forfeit).</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>[21/10/2026] Tutorial_Director.on_pile_viewed(); new prize-card lines added.</t>
+          <t>[21/10/2026] Tutorial_Director 'tips' mode, armed by GameState.TUTORIAL_TIPS_KEY when the newby wins Olly's match, cleared when that match ends.</t>
         </is>
       </c>
       <c r="G434" t="inlineStr">
@@ -18114,22 +18134,22 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Aesthetic</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>For a newby player, their SECOND match plays the start-of-turn key tips (Shift preview, Caps Lock log, Escape forfeit).</t>
+          <t>Energy cards gift: fly and fade in from the bottom, left to right, 0.2s apart. All fly-ins (coins, decks, energies) slow down, overshoot a few px and fall back.</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>[21/10/2026] Tutorial_Director 'tips' mode, armed by GameState.TUTORIAL_TIPS_KEY when the newby wins Olly's match, cleared when that match ends.</t>
+          <t>[21/10/2026] UIKit.fly_in() (FLY_OVERSHOOT_PX 12); MapManager 'card_fly' gift kind (CARD_FLY_* consts).</t>
         </is>
       </c>
       <c r="G435" t="inlineStr">
@@ -18149,22 +18169,22 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Aesthetic</t>
+          <t>Logic</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Energy cards gift: fly and fade in from the bottom, left to right, 0.2s apart. All fly-ins (coins, decks, energies) slow down, overshoot a few px and fall back.</t>
+          <t>Newby: cancelling an action (e.g. backing out of attaching energy) leaves no instructions; repeat the step's instruction and the energy requirement explanation.</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>[21/10/2026] UIKit.fly_in() (FLY_OVERSHOOT_PX 12); MapManager 'card_fly' gift kind (CARD_FLY_* consts).</t>
+          <t>[21/10/2026] Attach-screen explanation replays every time until attached; NEWBY_REMINDERS line on reopening the hand in the same step.</t>
         </is>
       </c>
       <c r="G436" t="inlineStr">
@@ -18184,22 +18204,22 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>Animation</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Logic</t>
+          <t>Values</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Newby: cancelling an action (e.g. backing out of attaching energy) leaves no instructions; repeat the step's instruction and the energy requirement explanation.</t>
+          <t>Double the delay between HP damage blocks greying out.</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>[21/10/2026] Attach-screen explanation replays every time until attached; NEWBY_REMINDERS line on reopening the hand in the same step.</t>
+          <t>[21/10/2026] HP_BLOCK_STEP 0.07 -&gt; 0.14 (healing does not animate per block).</t>
         </is>
       </c>
       <c r="G437" t="inlineStr">
@@ -18219,22 +18239,22 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>Animation</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>Values</t>
+          <t>Logic</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Double the delay between HP damage blocks greying out.</t>
+          <t>A tutorial block (e.g. energy onto the wrong Voltorb) closed the attach screen as if the action had happened.</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>[21/10/2026] HP_BLOCK_STEP 0.07 -&gt; 0.14 (healing does not animate per block).</t>
+          <t>[21/10/2026] perform_energy_attachment block now reopens the attach screen with the same Energy.</t>
         </is>
       </c>
       <c r="G438" t="inlineStr">
@@ -18254,22 +18274,22 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Logic</t>
+          <t>New Functionality</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>A tutorial block (e.g. energy onto the wrong Voltorb) closed the attach screen as if the action had happened.</t>
+          <t>Match log button in the in-match Escape menu; tutorial messages recorded in the log, visually distinct; 'Press [CAPS LOCK] To read back any of these help messages' at match start; Caps Lock over a message doesn't advance it.</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>[21/10/2026] perform_energy_attachment block now reopens the attach screen with the same Energy.</t>
+          <t>[21/10/2026] Pause menu 'Match log' button; show_message log_kind 'tutorial' -&gt; Match_Log_Panel tinted HELP rows; Tutorial_Director CAPS_HINT. Caps Lock over a message already worked (log swallows all input).</t>
         </is>
       </c>
       <c r="G439" t="inlineStr">
@@ -18289,7 +18309,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Animation</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -18299,12 +18319,12 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Match log button in the in-match Escape menu; tutorial messages recorded in the log, visually distinct; 'Press [CAPS LOCK] To read back any of these help messages' at match start; Caps Lock over a message doesn't advance it.</t>
+          <t>When a card is played, the hand / selection screen and its buttons fade out and the board fades in instead of snapping.</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>[21/10/2026] Pause menu 'Match log' button; show_message log_kind 'tutorial' -&gt; Match_Log_Panel tinted HELP rows; Tutorial_Director CAPS_HINT. Caps Lock over a message already worked (log swallows all input).</t>
+          <t>[21/10/2026] Main_Match_Core SCREEN SWAP FADE (SCREEN_SWAP_FADE 0.15).</t>
         </is>
       </c>
       <c r="G440" t="inlineStr">
@@ -18329,17 +18349,17 @@
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Values</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>When a card is played, the hand / selection screen and its buttons fade out and the board fades in instead of snapping.</t>
+          <t>Half the speed and double the life of every floating label across the game.</t>
         </is>
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>[21/10/2026] Main_Match_Core SCREEN SWAP FADE (SCREEN_SWAP_FADE 0.15).</t>
+          <t>[21/10/2026] Match show_floating_label 5.0s rise / 3.0s fade; deck builder MSG_*; bulk sell CARD/TOTAL_LABEL_*; fishing NEW_TAG_* (also the Fish Coin tag); Info cheat toast.</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
@@ -18359,22 +18379,22 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Animation</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Values</t>
+          <t>Incorrect Logic</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Half the speed and double the life of every floating label across the game.</t>
+          <t>Newby tutorial timing broken by the fighting energy count. Swap one of the opponent's Water Energy for Energy Removal and have Olly play it on Machop before Dratini's Pound.</t>
         </is>
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>[21/10/2026] Match show_floating_label 5.0s rise / 3.0s fade; deck builder MSG_*; bulk sell CARD/TOTAL_LABEL_*; fishing NEW_TAG_* (also the Fish Coin tag); Info cheat toast.</t>
+          <t>[21/10/2026] Basic Battle Deck: 18 Water + 1 Energy Removal; Professor Oak draws Fighting x5, Rattata, Energy Removal; NEWBY_CPU_PLAN turn 7 Energy Removal on the Active; turn-7 lines restored ('only has 1').</t>
         </is>
       </c>
       <c r="G442" t="inlineStr">
@@ -18394,22 +18414,22 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Incorrect Logic</t>
+          <t>Messages</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Newby tutorial timing broken by the fighting energy count. Swap one of the opponent's Water Energy for Energy Removal and have Olly play it on Machop before Dratini's Pound.</t>
+          <t>Newby first turn: explain the aim of the game, prize cards, energy and attaching to the active Pokemon before 'Click your hand'.</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>[21/10/2026] Basic Battle Deck: 18 Water + 1 Energy Removal; Professor Oak draws Fighting x5, Rattata, Energy Removal; NEWBY_CPU_PLAN turn 7 Energy Removal on the Active; turn-7 lines restored ('only has 1').</t>
+          <t>[21/10/2026] Tutorial_Director NEWBY_T1_AIM (6 lines, [POKEMON] = the active).</t>
         </is>
       </c>
       <c r="G443" t="inlineStr">
@@ -18429,22 +18449,22 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Messages</t>
+          <t>Aesthetic</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>Newby first turn: explain the aim of the game, prize cards, energy and attaching to the active Pokemon before 'Click your hand'.</t>
+          <t>Deck choice: darken first, old Kenney font on the names, options too high (centre the cards, not the text), deck box art peeking out behind each fan's back card, cards moved left and decks spread wider.</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>[21/10/2026] Tutorial_Director NEWBY_T1_AIM (6 lines, [POKEMON] = the active).</t>
+          <t>[21/10/2026] IntroDeckChoice: DIM 0.8 fades first, names forced to ChakraPetch-Bold, CARDS_MID_Y 540, deck box (BOX_HEIGHT/TUCK/RAISE), GROUP_CENTRES 320/960/1600.</t>
         </is>
       </c>
       <c r="G444" t="inlineStr">
@@ -18469,17 +18489,17 @@
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Aesthetic</t>
+          <t>Messages</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>Deck choice: darken first, old Kenney font on the names, options too high (centre the cards, not the text), deck box art peeking out behind each fan's back card, cards moved left and decks spread wider.</t>
+          <t>Coin flip header hidden; 'Build your bench' header and its two buttons stuck on screen after the coin flip until the hand was next opened.</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>[21/10/2026] IntroDeckChoice: DIM 0.8 fades first, names forced to ChakraPetch-Bold, CARDS_MID_Y 540, deck box (BOX_HEIGHT/TUCK/RAISE), GROUP_CENTRES 320/960/1600.</t>
+          <t>[21/10/2026] Both caused by the new card-play fade: the coin call saved the fading bench header/buttons as visible and restored them. _snap_screen_swap() now hides fading-out pieces and runs before the coin call.</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
@@ -18504,17 +18524,17 @@
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>Messages</t>
+          <t>Aesthetic</t>
         </is>
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>Coin flip header hidden; 'Build your bench' header and its two buttons stuck on screen after the coin flip until the hand was next opened.</t>
+          <t>Tutorial 'Opponent's hand' label not visible.</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>[21/10/2026] Both caused by the new card-play fade: the coin call saved the fading bench header/buttons as visible and restored them. _snap_screen_swap() now hides fading-out pieces and runs before the coin call.</t>
+          <t>[21/10/2026] It drew under the header bar; now z_index Z_CHROME + 20.</t>
         </is>
       </c>
       <c r="G446" t="inlineStr">
@@ -18534,22 +18554,22 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Aesthetic</t>
+          <t>Crash</t>
         </is>
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Tutorial 'Opponent's hand' label not visible.</t>
+          <t>Double clicking an energy card crashed the game.</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>[21/10/2026] It drew under the header bar; now z_index Z_CHROME + 20.</t>
+          <t>[21/10/2026] CardDisplay._input carried on after card_clicked played the card and freed the node (get_tree() null); it now returns if the node left the tree.</t>
         </is>
       </c>
       <c r="G447" t="inlineStr">
@@ -18569,22 +18589,22 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>Overworld</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>Crash</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>Double clicking an energy card crashed the game.</t>
+          <t>Interior camera completely locked; allow a little movement while keeping the room (mostly) in view.</t>
         </is>
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t>[21/10/2026] CardDisplay._input carried on after card_clicked played the card and freed the node (get_tree() null); it now returns if the node left the tree.</t>
+          <t>[21/10/2026] Player_Object_Script CAMERA_ROOM_SLACK 28 world px either way on axes where the room is smaller than the view.</t>
         </is>
       </c>
       <c r="G448" t="inlineStr">
@@ -18604,22 +18624,22 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>Overworld</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>Interior camera completely locked; allow a little movement while keeping the room (mostly) in view.</t>
+          <t>Convert DraftTime (RSE Trick House).mp3 to .ogg; play it during Hard Mode's pack opening, back to the overworld track after, and in the draft deck builder.</t>
         </is>
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>[21/10/2026] Player_Object_Script CAMERA_ROOM_SLACK 28 world px either way on axes where the room is smaller than the view.</t>
+          <t>[21/10/2026] Converted with ffmpeg (imageio-ffmpeg); SoundManager BGM_DRAFT_TIME + crossfade_bgm(); Olly_Intro_Cutscene and deck builder draft mode use it.</t>
         </is>
       </c>
       <c r="G449" t="inlineStr">
@@ -18639,22 +18659,22 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>Messages</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Convert DraftTime (RSE Trick House).mp3 to .ogg; play it during Hard Mode's pack opening, back to the overworld track after, and in the draft deck builder.</t>
+          <t>Hard Mode: no gap between the energies and being forced into the deck builder. Gift the energies, close the gift screen, then 'Hey, let's try building a deck right now!...' before the deck builder.</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>[21/10/2026] Converted with ffmpeg (imageio-ffmpeg); SoundManager BGM_DRAFT_TIME + crossfade_bgm(); Olly_Intro_Cutscene and deck builder draft mode use it.</t>
+          <t>[21/10/2026] LINE_HARD_AFTER_PACKS reworded; LINES_HARD_BUILD said after the energy reveal closes.</t>
         </is>
       </c>
       <c r="G450" t="inlineStr">
@@ -18674,22 +18694,22 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Deck Builder</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>Messages</t>
+          <t>New Functionality</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Hard Mode: no gap between the energies and being forced into the deck builder. Gift the energies, close the gift screen, then 'Hey, let's try building a deck right now!...' before the deck builder.</t>
+          <t>Sort by '# Owned', and remember the previous sort order so sorts stack (newest first, earlier ones as tie-breakers).</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>[21/10/2026] LINE_HARD_AFTER_PACKS reworded; LINES_HARD_BUILD said after the energy reveal closes.</t>
+          <t>[21/10/2026] Card_Search_Overlay '# OWNED' mode + _sort_chain; deck builder _sort_search_results() sorts by the whole chain.</t>
         </is>
       </c>
       <c r="G451" t="inlineStr">
@@ -18709,22 +18729,22 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>Deck Builder</t>
+          <t>Overworld</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>NPC Location</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>Sort by '# Owned', and remember the previous sort order so sorts stack (newest first, earlier ones as tie-breakers).</t>
+          <t>Olly doesn't walk down far enough before going left and gets stuck on the player's wall; he should run to the path then up off screen towards FISH.</t>
         </is>
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>[21/10/2026] Card_Search_Overlay '# OWNED' mode + _sort_chain; deck builder _sort_search_results() sorts by the whole chain.</t>
+          <t>[21/10/2026] Exit is now a glide (no collision): down to the path, along to EXIT_PATH_X -712, up EXIT_RUN_UP 700; player watches him go.</t>
         </is>
       </c>
       <c r="G452" t="inlineStr">
@@ -18744,22 +18764,22 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>Overworld</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>NPC Location</t>
+          <t>Incorrect Logic</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>Olly doesn't walk down far enough before going left and gets stuck on the player's wall; he should run to the path then up off screen towards FISH.</t>
+          <t>The opponent used gust of wind when for a pokemon with the same HP which it was already a guarenteed knockout for. It provided no value. Then it attached two pluspowers putting it to +20 damage over what it needed when it didn't need any at all. It was mewtwo using psyburn on an ekans, gust of winding it for venonat, then knocking venonat out</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>[21/10/2026] Exit is now a glide (no collision): down to the path, along to EXIT_PATH_X -712, up EXIT_RUN_UP 700; player watches him go.</t>
+          <t>CPU_AI _cpu_score_gust_of_wind_base: if the player's Active is already a sure KO (_cpu_can_ko_now), a gust onto a Benched Pokemon is skipped unless that target is worth more to KO (_gust_ko_worth: Prizes x100, +25 evolved, +15 per Energy). Print: ISSUE #451.</t>
         </is>
       </c>
       <c r="G453" t="inlineStr">
@@ -18769,7 +18789,12 @@
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
         </is>
       </c>
     </row>
@@ -18789,12 +18814,12 @@
       </c>
       <c r="D454" s="6" t="inlineStr">
         <is>
-          <t>The opponent used gust of wind when for a pokemon with the same HP which it was already a guarenteed knockout for. It provided no value. Then it attached two pluspowers putting it to +20 damage over what it needed when it didn't need any at all. It was mewtwo using psyburn on an ekans, gust of winding it for venonat, then knocking venonat out</t>
+          <t>Also the opponent just played plus power on hitmonchan against ekans, it used jab for 30hp danage, 2 x 20hp jabs would have done the same. Pluspower should have been kept</t>
         </is>
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>CPU_AI _cpu_score_gust_of_wind_base: if the player's Active is already a sure KO (_cpu_can_ko_now), a gust onto a Benched Pokemon is skipped unless that target is worth more to KO (_gust_ko_worth: Prizes x100, +25 evolved, +15 per Energy). Print: ISSUE #452.</t>
+          <t>CPU_AI _cpu_score_pluspower rewritten: PlusPower is added after W/R, so it is a flat +10 on top of the attack (attached PlusPowers counted). Held (0) when an attack already KOs, played at 90 when it creates a KO, at 30 only when it cuts the number of hits the KO needs (Jab 20 vs 40 HP = 2 hits either way -&gt; held). Also covers #454. Print: ISSUE #452.</t>
         </is>
       </c>
       <c r="G454" s="6" t="inlineStr">
@@ -18809,7 +18834,7 @@
       </c>
       <c r="J454" t="inlineStr">
         <is>
-          <t>Live: 1</t>
+          <t>Live: 2</t>
         </is>
       </c>
     </row>
@@ -18829,12 +18854,12 @@
       </c>
       <c r="D455" s="6" t="inlineStr">
         <is>
-          <t>Also the opponent just played plus power on hitmonchan against ekans, it used jab for 30hp danage, 2 x 20hp jabs would have done the same. Pluspower should have been kept</t>
+          <t>the CPU then retreated hitmonchan with 2 discards for mewtwo on the bench for no reason when ekans had 10hp and was knokced out by jab and player had nothing to return fire with</t>
         </is>
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>CPU_AI _cpu_score_pluspower rewritten: PlusPower is added after W/R, so it is a flat +10 on top of the attack (attached PlusPowers counted). Held (0) when an attack already KOs, played at 90 when it creates a KO, at 30 only when it cuts the number of hits the KO needs (Jab 20 vs 40 HP = 2 hits either way -&gt; held). Also covers #455. Print: ISSUE #453.</t>
+          <t>CPU_AI _offensive_retreat_target: returns null when the Active's best usable damage already KOs the player's Active -- overkill damage no longer counts as an 'offensive upgrade' worth a retreat. Print: ISSUE #453.</t>
         </is>
       </c>
       <c r="G455" s="6" t="inlineStr">
@@ -18849,7 +18874,7 @@
       </c>
       <c r="J455" t="inlineStr">
         <is>
-          <t>Live: 2</t>
+          <t>Live: 1</t>
         </is>
       </c>
     </row>
@@ -18869,12 +18894,12 @@
       </c>
       <c r="D456" s="6" t="inlineStr">
         <is>
-          <t>the CPU then retreated hitmonchan with 2 discards for mewtwo on the bench for no reason when ekans had 10hp and was knokced out by jab and player had nothing to return fire with</t>
+          <t>and again mewtwo attached pluspower for 50 damage when player only had 30</t>
         </is>
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t>CPU_AI _offensive_retreat_target: returns null when the Active's best usable damage already KOs the player's Active -- overkill damage no longer counts as an 'offensive upgrade' worth a retreat. Print: ISSUE #454.</t>
+          <t>Same fix as #452 (_cpu_score_pluspower holds PlusPower when the attack already Knocks Out).</t>
         </is>
       </c>
       <c r="G456" s="6" t="inlineStr">
@@ -18885,11 +18910,6 @@
       <c r="H456" t="inlineStr">
         <is>
           <t>23/10/2026</t>
-        </is>
-      </c>
-      <c r="J456" t="inlineStr">
-        <is>
-          <t>Live: 1</t>
         </is>
       </c>
     </row>
@@ -18909,12 +18929,12 @@
       </c>
       <c r="D457" s="6" t="inlineStr">
         <is>
-          <t>and again mewtwo attached pluspower for 50 damage when player only had 30</t>
+          <t>When playing professor oak (so most liekly any effect that draws multiple cards, the cards vanish quicker than they animate moving to the discard pile, they should only vanish AS the card moves</t>
         </is>
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>Same fix as #453 (_cpu_score_pluspower holds PlusPower when the attack already Knocks Out).</t>
+          <t>Trainer_Effects: Professor Oak, Impostor Professor Oak and Lass hid a hand slot every 0.1s while card flights queue one at a time (#243), so the hand emptied before the cards flew. Each flight is now awaited (same total time). Lass also erased cards from the hand array mid-loop without a redraw, so later flights hid the WRONG slot -- cards now leave the arrays after the flights. No Removal Gym tax loop redraws between its cards for the same reason. Print: ISSUE #455.</t>
         </is>
       </c>
       <c r="G457" s="6" t="inlineStr">
@@ -18925,6 +18945,11 @@
       <c r="H457" t="inlineStr">
         <is>
           <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
         </is>
       </c>
     </row>
@@ -18934,7 +18959,7 @@
       </c>
       <c r="B458" s="5" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>CPU logic</t>
         </is>
       </c>
       <c r="C458" s="5" t="inlineStr">
@@ -18944,12 +18969,12 @@
       </c>
       <c r="D458" s="6" t="inlineStr">
         <is>
-          <t>When playing professor oak (so most liekly any effect that draws multiple cards, the cards vanish quicker than they animate moving to the discard pile, they should only vanish AS the card moves</t>
+          <t>The CPU had a spearow, attached a pluspower which would have knocked out pikachu with 20hp but then evolved to fearow when only one energy was attached insteaqd of guarenteeing the kill</t>
         </is>
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>Trainer_Effects: Professor Oak, Impostor Professor Oak and Lass hid a hand slot every 0.1s while card flights queue one at a time (#243), so the hand emptied before the cards flew. Each flight is now awaited (same total time). Lass also erased cards from the hand array mid-loop without a redraw, so later flights hid the WRONG slot -- cards now leave the arrays after the flights. No Removal Gym tax loop redraws between its cards for the same reason. Print: ISSUE #456.</t>
+          <t>CPU_AI evaluate_evolution_pair: -600 when the Active can KO the Defending Pokemon right now (PlusPowers counted) and the evolved form can't attack this turn (allowing for one more Energy from hand if the attach is unused). Print: ISSUE #456.</t>
         </is>
       </c>
       <c r="G458" s="6" t="inlineStr">
@@ -18964,7 +18989,7 @@
       </c>
       <c r="J458" t="inlineStr">
         <is>
-          <t>Live: 2</t>
+          <t>Live: 1</t>
         </is>
       </c>
     </row>
@@ -18974,22 +18999,22 @@
       </c>
       <c r="B459" s="5" t="inlineStr">
         <is>
-          <t>CPU logic</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C459" s="5" t="inlineStr">
         <is>
-          <t>Incorrect Logic</t>
+          <t>New Functionality</t>
         </is>
       </c>
       <c r="D459" s="6" t="inlineStr">
         <is>
-          <t>The CPU had a spearow, attached a pluspower which would have knocked out pikachu with 20hp but then evolved to fearow when only one energy was attached insteaqd of guarenteeing the kill</t>
+          <t>When attempting to go to bed and it's too early, have different message each timeslot. Morning = "I've only just woken up, I'm not getting back in bed now!" Afternoon= "I'd love an afternoon nap… but I'd end up sleeping for hours…" Evening= the current nothing wrong with an early night</t>
         </is>
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>CPU_AI evaluate_evolution_pair: -600 when the Active can KO the Defending Pokemon right now (PlusPowers counted) and the evolved form can't attack this turn (allowing for one more Energy from hand if the attach is unused). Print: ISSUE #457.</t>
+          <t>Player_House_Upstairs.gd and Interactables_Script.gd: BED_TOO_EARLY_TEXT is now one line per slot (Morning / Afternoon / Evening, Evening as fallback) with the user's text. Print: ISSUE #457.</t>
         </is>
       </c>
       <c r="G459" s="6" t="inlineStr">
@@ -19014,22 +19039,22 @@
       </c>
       <c r="B460" s="5" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C460" s="5" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Incorrect Logic</t>
         </is>
       </c>
       <c r="D460" s="6" t="inlineStr">
         <is>
-          <t>When attempting to go to bed and it's too early, have different message each timeslot. Morning = "I've only just woken up, I'm not getting back in bed now!" Afternoon= "I'd love an afternoon nap… but I'd end up sleeping for hours…" Evening= the current nothing wrong with an early night</t>
+          <t>Autotester: Charizard delta (ex14-4) Peal of Thunder attached every Energy from the top 5 cards with no legality check, so R Energy (Dark/Rocket's only) ended up on Gyarados delta.</t>
         </is>
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>Player_House_Upstairs.gd and Interactables_Script.gd: BED_TOO_EARLY_TEXT is now one line per slot (Morning / Afternoon / Evening, Evening as fallback) with the user's text. Print: ISSUE #458.</t>
+          <t>Powers_And_Bodies_Effects trigger_ex14_peal_of_thunder: Energy is filtered through special_energy_effects.can_attach_to for the chosen Pokemon; illegal ones are discarded with the rest of the looked-at cards. Replay 2026-10-23T16-09-05:67 now clean. Print: ISSUE #458.</t>
         </is>
       </c>
       <c r="G460" s="6" t="inlineStr">
@@ -19048,13 +19073,13 @@
         </is>
       </c>
     </row>
-    <row r="461">
+    <row r="461" ht="30" customHeight="1">
       <c r="A461" s="5" t="n">
         <v>459</v>
       </c>
       <c r="B461" s="5" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>CPU logic</t>
         </is>
       </c>
       <c r="C461" s="5" t="inlineStr">
@@ -19064,12 +19089,12 @@
       </c>
       <c r="D461" s="6" t="inlineStr">
         <is>
-          <t>Autotester: Charizard delta (ex14-4) Peal of Thunder attached every Energy from the top 5 cards with no legality check, so R Energy (Dark/Rocket's only) ended up on Gyarados delta.</t>
+          <t>CPU passed up guaranteed Knock Outs for weaker attacks (autotester MISSED KO, ~8 per 150 matches).</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>Powers_And_Bodies_Effects trigger_ex14_peal_of_thunder: Energy is filtered through special_energy_effects.can_attach_to for the chosen Pokemon; illegal ones are discarded with the rest of the looked-at cards. Replay 2026-10-23T16-09-05:67 now clean. Print: ISSUE #459.</t>
+          <t>CPU_Lookahead.attack_value only credited a KO NEXT turn (+160 for a set-up attack, 0 for the KO now) -- now counts the Prize taken this turn. CPU_AI cpu_phase_attack: if any payable attack is a sure KO (min damage after W/R &gt;= HP, not flagged 'does nothing', no self-KO recoil) the best-scoring KO attack is used. The estimate also honours 'isn't affected by (Weakness or) Resistance' (46 attacks). 100-match run after: 1 miss -&gt; 0 expected after the Resistance fix. Print: ISSUE #459.</t>
         </is>
       </c>
       <c r="G461" s="6" t="inlineStr">
@@ -19094,22 +19119,23 @@
       </c>
       <c r="B462" s="5" t="inlineStr">
         <is>
-          <t>CPU logic</t>
+          <t>Overworld</t>
         </is>
       </c>
       <c r="C462" s="5" t="inlineStr">
         <is>
-          <t>Incorrect Logic</t>
+          <t>New Functionality</t>
         </is>
       </c>
       <c r="D462" s="6" t="inlineStr">
         <is>
-          <t>CPU passed up guaranteed Knock Outs for weaker attacks (autotester MISSED KO, ~8 per 150 matches).</t>
+          <t>Windmill Mewtwo: spawn him properly, remove the MEWTWO? picture; after his defeat he stands there, says 'MEW' and vanishes for good.</t>
         </is>
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>CPU_Lookahead.attack_value only credited a KO NEXT turn (+160 for a set-up attack, 0 for the KO now) -- now counts the Prize taken this turn. CPU_AI cpu_phase_attack: if any payable attack is a sure KO (min damage after W/R &gt;= HP, not flagged 'does nothing', no self-KO recoil) the best-scoring KO attack is used. The estimate also honours 'isn't affected by (Weakness or) Resistance' (46 attacks). 100-match run after: 1 miss -&gt; 0 expected after the Resistance fix. Print: ISSUE #460.</t>
+          <t>Windmill.json: at [229,10] (was ~300px under the floor), requires 'not flag: mewtwo_vanished'. MEWTWO? TextureRect + Character_Sprites/Mewtwo.png removed. Windmill.gd: once beaten, his talk is a cutscene line 'MEW' (talk bubble, no challenge), then a white flare + squeeze vanish and the flag is raised. Opponent_Object_Script.bubble_override added.
+Follow-up: he now says MEW and vanishes the moment the player is back from beating him (Windmill._ready, after an 0.8s beat and any open box). Talking to him stays as the fallback if they quit first.</t>
         </is>
       </c>
       <c r="G462" s="6" t="inlineStr">
@@ -19129,7 +19155,7 @@
       </c>
       <c r="B463" s="5" t="inlineStr">
         <is>
-          <t>Overworld</t>
+          <t>Story</t>
         </is>
       </c>
       <c r="C463" s="5" t="inlineStr">
@@ -19139,13 +19165,13 @@
       </c>
       <c r="D463" s="6" t="inlineStr">
         <is>
-          <t>Windmill Mewtwo: spawn him properly, remove the MEWTWO? picture; after his defeat he stands there, says 'MEW' and vanishes for good.</t>
+          <t>Café morning reminder calls: first from whoever didn't invite you (10 NPC talks OR 2 interior-&gt;outside trips), second from Alexander (25 talks OR 5 trips).</t>
         </is>
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>Windmill.json: at [229,10] (was ~300px under the floor), requires 'not flag: mewtwo_vanished'. MEWTWO? TextureRect + Character_Sprites/Mewtwo.png removed. Windmill.gd: once beaten, his talk is a cutscene line 'MEW' (talk bubble, no challenge), then a white flare + squeeze vanish and the flag is raised. Opponent_Object_Script.bubble_override added.
-Follow-up: he now says MEW and vanishes the moment the player is back from beating him (Windmill._ready, after an 0.8s beat and any open box). Talking to him stays as the fallback if they quit first.</t>
+          <t>Phone_Calls.json cafe_reminder_olly / _ellie / _alexander. CafeBreakfastCutscene REMINDERS + note_npc_talk / note_exterior_return / reminder_due / reminder_played (counts from the invitation until first sat down). MapManager rings it when the player is free (_try_story_reminder, every 0.5s). Olly's line 'I've been gotta' typed as 'I've gotta'.
+Follow-up: bonus call cafe_reminder_fishing -- Olly rings once 5 fish are landed after the invitation while he is still at the café (new/rules, before his match). Separate from the two reminders; rings when the fishing session closes.</t>
         </is>
       </c>
       <c r="G463" s="6" t="inlineStr">
@@ -19159,13 +19185,13 @@
         </is>
       </c>
     </row>
-    <row r="464">
+    <row r="464" ht="30" customHeight="1">
       <c r="A464" s="5" t="n">
         <v>462</v>
       </c>
       <c r="B464" s="5" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Battle</t>
         </is>
       </c>
       <c r="C464" s="5" t="inlineStr">
@@ -19175,13 +19201,12 @@
       </c>
       <c r="D464" s="6" t="inlineStr">
         <is>
-          <t>Café morning reminder calls: first from whoever didn't invite you (10 NPC talks OR 2 interior-&gt;outside trips), second from Alexander (25 talks OR 5 trips).</t>
+          <t>Attack hit feedback: attacker tilts, lunges and bumps the defender; defender flashes white, is knocked back and wiggles.</t>
         </is>
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>Phone_Calls.json cafe_reminder_olly / _ellie / _alexander. CafeBreakfastCutscene REMINDERS + note_npc_talk / note_exterior_return / reminder_due / reminder_played (counts from the invitation until first sat down). MapManager rings it when the player is free (_try_story_reminder, every 0.5s). Olly's line 'I've been gotta' typed as 'I've gotta'.
-Follow-up: bonus call cafe_reminder_fishing -- Olly rings once 5 fish are landed after the invitation while he is still at the café (new/rules, before his match). Separate from the two reminders; rings when the fishing session closes.</t>
+          <t>Main_Match_Core play_attack_hit() (Active vs Active, damage &gt; 0), called from display_and_apply_attack_damage before the damage numbers. Ghost copies of the two card images, so layout is untouched. HIT_* consts are the tweakables.</t>
         </is>
       </c>
       <c r="G464" s="6" t="inlineStr">
@@ -19201,7 +19226,7 @@
       </c>
       <c r="B465" s="5" t="inlineStr">
         <is>
-          <t>Battle</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="C465" s="5" t="inlineStr">
@@ -19211,12 +19236,12 @@
       </c>
       <c r="D465" s="6" t="inlineStr">
         <is>
-          <t>Attack hit feedback: attacker tilts, lunges and bumps the defender; defender flashes white, is knocked back and wiggles.</t>
+          <t>Coin landing sound (placeholder copy of the flip sound for now).</t>
         </is>
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Main_Match_Core play_attack_hit() (Active vs Active, damage &gt; 0), called from display_and_apply_attack_damage before the damage numbers. Ghost copies of the two card images, so layout is untouched. HIT_* consts are the tweakables.</t>
+          <t>Audio/SFX/coin_land_sound.ogg (copy of coin_flip_sound.ogg -- overwrite it with the real one). SFX_coin_land_sound plays when the match coin and the overworld coin-flipper coins land.</t>
         </is>
       </c>
       <c r="G465" s="6" t="inlineStr">
@@ -19246,12 +19271,12 @@
       </c>
       <c r="D466" s="6" t="inlineStr">
         <is>
-          <t>Coin landing sound (placeholder copy of the flip sound for now).</t>
+          <t>Footstep sounds when walking.</t>
         </is>
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>Audio/SFX/coin_land_sound.ogg (copy of coin_flip_sound.ogg -- overwrite it with the real one). SFX_coin_land_sound plays when the match coin and the overworld coin-flipper coins land.</t>
+          <t>Player_Object_Script: plays FOOTSTEP_SFX_PATH (res://Audio/SFX/Footsteps/footstep.ogg) on walk frames 1 and 3 with slight random pitch. Silent until that file exists.</t>
         </is>
       </c>
       <c r="G466" s="6" t="inlineStr">
@@ -19271,7 +19296,7 @@
       </c>
       <c r="B467" s="5" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>UI/Aesthetic</t>
         </is>
       </c>
       <c r="C467" s="5" t="inlineStr">
@@ -19281,12 +19306,12 @@
       </c>
       <c r="D467" s="6" t="inlineStr">
         <is>
-          <t>Footstep sounds when walking.</t>
+          <t>Collection progress in the deck builder, without cluttering the screen.</t>
         </is>
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>Player_Object_Script: plays FOOTSTEP_SFX_PATH (res://Audio/SFX/Footsteps/footstep.ogg) on walk frames 1 and 3 with slight random pitch. Silent until that file exists.</t>
+          <t>Small chip right of the set stepper: distinct cards owned / cards in the set. Hover tooltip: whole collection total.</t>
         </is>
       </c>
       <c r="G467" s="6" t="inlineStr">
@@ -19316,12 +19341,12 @@
       </c>
       <c r="D468" s="6" t="inlineStr">
         <is>
-          <t>Collection progress in the deck builder, without cluttering the screen.</t>
+          <t>Time-of-day pop-down (Morning/Afternoon/Evening/Night/Midnight) when the time changed, after a match or stepping outside.</t>
         </is>
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>Small chip right of the set stepper: distinct cards owned / cards in the set. Hover tooltip: whole collection total.</t>
+          <t>Time_Of_Day_Banner.gd: rounded panel + drawn icon, light blue / yellow / orange-red / dark blue (darker for Midnight). Drops in from the top left, holds 1s, rises out. Triggered in BaseMapScene._ready via GameState.last_seen_time.</t>
         </is>
       </c>
       <c r="G468" s="6" t="inlineStr">
@@ -19341,22 +19366,22 @@
       </c>
       <c r="B469" s="5" t="inlineStr">
         <is>
-          <t>UI/Aesthetic</t>
+          <t>Core Gameplay</t>
         </is>
       </c>
       <c r="C469" s="5" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Incorrect Logic</t>
         </is>
       </c>
       <c r="D469" s="6" t="inlineStr">
         <is>
-          <t>Time-of-day pop-down (Morning/Afternoon/Evening/Night/Midnight) when the time changed, after a match or stepping outside.</t>
+          <t>Autotester: Scramble / Double Rainbow Energy stayed on a Pokemon that evolved into a Pokemon-ex (Graveler -&gt; Golem ex, Charmeleon -&gt; Charizard ex).</t>
         </is>
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>Time_Of_Day_Banner.gd: rounded panel + drawn icon, light blue / yellow / orange-red / dark blue (darker for Midnight). Drops in from the top left, holds 1s, rises out. Triggered in BaseMapScene._ready via GameState.last_seen_time.</t>
+          <t>Special_Energy_Effects: can_attach_to's 'which Pokemon may hold this' block split out as type_lock_check(); discard_now_illegal() re-runs it on every attached Special Energy and discards what no longer qualifies. Called from perform_evolution right after the Energy hand-over, with an orange 'X DISCARDED' figure. Covers R / Aqua / Magma / Miracle / Boost / Scramble / Double Rainbow. Replay clean. Print: ISSUE #467.</t>
         </is>
       </c>
       <c r="G469" s="6" t="inlineStr">
@@ -19369,29 +19394,34 @@
           <t>23/10/2026</t>
         </is>
       </c>
-    </row>
-    <row r="470">
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="470" ht="30" customHeight="1">
       <c r="A470" s="5" t="n">
         <v>468</v>
       </c>
       <c r="B470" s="5" t="inlineStr">
         <is>
-          <t>Core Gameplay</t>
+          <t>Debug</t>
         </is>
       </c>
       <c r="C470" s="5" t="inlineStr">
         <is>
-          <t>Incorrect Logic</t>
+          <t>New Functionality</t>
         </is>
       </c>
       <c r="D470" s="6" t="inlineStr">
         <is>
-          <t>Autotester: Scramble / Double Rainbow Energy stayed on a Pokemon that evolved into a Pokemon-ex (Graveler -&gt; Golem ex, Charmeleon -&gt; Charizard ex).</t>
+          <t>Debug menu CUTSCENES page: every cutscene and variation, jumping to its date/time/place and playing from the start.</t>
         </is>
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>Special_Energy_Effects: can_attach_to's 'which Pokemon may hold this' block split out as type_lock_check(); discard_now_illegal() re-runs it on every attached Special Energy and discards what no longer qualifies. Called from perform_evolution right after the Energy hand-over, with an orange 'X DISCARDED' figure. Covers R / Aqua / Magma / Miracle / Boost / Scramble / Double Rainbow. Replay clean. Print: ISSUE #468.</t>
+          <t>Scripts/Utilities/Debug_Cutscenes.gd (catalogue + launchers, 41 buttons in 8 groups); Debug_Menu CUTSCENES... button opens the page (BACK returns). Each launch wipes the story keys, sets intro answers/date/time, loads the map at the right door/spot; the café table is talked to automatically. Runtime-tested 13 launchers on a throwaway slot. Found + fixed on the way: Phone_Call line loop crashed if the map changed mid-call; MapManager reminder flag stuck on for the session if a reminder call was freed with its map.</t>
         </is>
       </c>
       <c r="G470" s="6" t="inlineStr">
@@ -19411,38 +19441,1576 @@
       </c>
       <c r="B471" s="5" t="inlineStr">
         <is>
-          <t>Debug</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C471" s="5" t="inlineStr">
         <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D471" s="6" t="inlineStr">
+        <is>
+          <t>When opening options in a match now, the background can't be seen and is just black</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>25/10: In-match Options sat on an OPAQUE black click-blocker, and the options screen's own animated background (UIKit.add_field) is at z_index -100, so the blocker drew over it. Blocker is now transparent (still stops clicks). Main_Match_Core _on_pause_options_pressed.</t>
+        </is>
+      </c>
+      <c r="G471" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="5" t="n">
+        <v>470</v>
+      </c>
+      <c r="B472" s="5" t="inlineStr">
+        <is>
+          <t>Player input</t>
+        </is>
+      </c>
+      <c r="C472" s="5" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D472" s="6" t="inlineStr">
+        <is>
+          <t>For the mandatory tutorials at the start of the game, have the option for tutorials turned on, and disabled greyed out so the player can't turn the tutorial off until having it complete making it obvious it's mandatory</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>25/10: New GameState.mandatory_tutorial_running (set/cleared by Tutorial_Director) + tutorial_option_locked() (also true while the newby's follow-up match is pending). Options shows 'Tutorial messages for next match' as On, buttons disabled + greyed (45% alpha) while locked; nothing is saved from it.</t>
+        </is>
+      </c>
+      <c r="G472" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="473" ht="30" customHeight="1">
+      <c r="A473" s="5" t="n">
+        <v>471</v>
+      </c>
+      <c r="B473" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C473" s="5" t="inlineStr">
+        <is>
           <t>New Functionality</t>
         </is>
       </c>
-      <c r="D471" s="6" t="inlineStr">
-        <is>
-          <t>Debug menu CUTSCENES page: every cutscene and variation, jumping to its date/time/place and playing from the start.</t>
-        </is>
-      </c>
-      <c r="E471" t="inlineStr">
-        <is>
-          <t>Scripts/Utilities/Debug_Cutscenes.gd (catalogue + launchers, 41 buttons in 8 groups); Debug_Menu CUTSCENES... button opens the page (BACK returns). Each launch wipes the story keys, sets intro answers/date/time, loads the map at the right door/spot; the café table is talked to automatically. Runtime-tested 13 launchers on a throwaway slot. Found + fixed on the way: Phone_Call line loop crashed if the map changed mid-call; MapManager reminder flag stuck on for the session if a reminder call was freed with its map.</t>
-        </is>
-      </c>
-      <c r="G471" s="6" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H471" t="inlineStr">
-        <is>
-          <t>23/10/2026</t>
-        </is>
-      </c>
+      <c r="D473" s="6" t="inlineStr">
+        <is>
+          <t>When a pokemon attacks another we now have a little animation of it being hit. Also have animations for mutliple other things:
+1) When initially poisoned or taking damage from poison and the messagebox pops up saying "X was posioned" or "X took N poison damage", the card fades to purple and back and shakes side to side a few times slowly. Speed rams up accelerates slowly, then decelerates then stops then changes directions, accelerates, decelerates to a stop, changes direction
+2) When paralyzed or can't attack because paraylsis, card fades to yellow quickly and back and shakes side to side rapidly with no speed ramping
+3) When confused is inflicted, or a coin is flipped to decide if a confused pokemon can or can't attack, draw two stars spinning in in oval like a wide circle at the top of the pokemon card. Have the stars be trailed by a yellow glowing line that fades out as the trail meets the next star in the circle. Also have the pokemon card like poison, slowly move side to side with speed ramping, but also teeter it a small amount left and right while it moves
+4) For sleeping pokemon when they go to sleep or a coin flip fails and they're still asleep, have the letter Z come out of the top left for player pokemon or top right of opponent's pokemon card, angled left or right depending what side they're on, they grow larger as they leave the pokemon card then after about half a second of life they fade out to nothing. Have 3 black letter Z rise and have the card move up and down a small amount really slowly with speed ramping just like a little bob
+5) for burn, have a mix of 1 and 2. A shake side to side, coloured red, but not a slow gentle side to side nor a fast jagged side to side, a bit inbetween so a medium speed shake with the red glow and fade.</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>25/10: New Scripts/Main_Match_Gameplay_Scripts/Card_FX.gd (main.card_fx). Plays on a ghost copy of the card that follows it every frame. Poison: slow sine sway (eases to a stop each end, turns round) + purple fade; Paralysis: fast even jolts + quick yellow flash; Burn: medium sway + red; Confusion: poison sway + teeter + 2 stars circling an ellipse over the card with fading yellow trails; Sleep: slow bob + 3 black Zs drifting up-left (yours) / up-right (theirs), growing, fading after ~0.5s. Triggers: ANY newly-landed status (diff in update_status_icons, so every effect script is covered), poison/burn ticks, 'still asleep', player 'paralyzed/asleep and cannot attack', confusion attack flip. All timings/sizes are TWEAKABLE consts at the top of Card_FX.gd.</t>
+        </is>
+      </c>
+      <c r="G473" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="474" ht="240" customHeight="1">
+      <c r="A474" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="B474" s="5" t="inlineStr">
+        <is>
+          <t>animation</t>
+        </is>
+      </c>
+      <c r="C474" s="5" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D474" s="6" t="inlineStr">
+        <is>
+          <t>Whenever a card is drawn, either as part of an effect, during the tutorial, or at the start of a turn, if a messagebox is to play (e.g a tutorial message, or the opponent is using a trainer card or attaching an energy) after the card is drawn, always have a 1.0  second pause (Times the animation speed modifier) first before displaying a message just so the player can register what has been drawn and has it in mind. the messagebox hides the drawn card. Also have this same thing apply when a card is taken as a prize card, the card is added to the hand but as soon as that is done currently the next pokemon or your pokemon has to be made active, so just wait the second after the prize card is added to the hand. Same with like bill and professor oak, all the cards are put into the opponents hand then the next card is almost immediately played</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>25/10: Generic 'let the draw register' beat: draw_card_from_deck and take_prize_card stamp the landing time; the next show_message, handle_post_knockout (choose new Active after a Prize) and CPU energy/bench/trainer phases wait out the rest of DRAW_SETTLE_TIME (1.0s x animation speed). Covers turn draws, tutorial messages, Bill/Oak draws, Prizes.</t>
+        </is>
+      </c>
+      <c r="G474" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="475" ht="105" customHeight="1">
+      <c r="A475" s="5" t="n">
+        <v>473</v>
+      </c>
+      <c r="B475" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C475" s="5" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D475" s="6" t="inlineStr">
+        <is>
+          <t>For the new attack animation, if the opponent is weak, have the shake and knock back be twice as much. If opponent is resistant half as much. Colour slightly the white flash with weak or resist so a weak will go slightly green tint and a resistant will go slightly red tint. If damage is reduced to 0, the attack animation should still play (it doesn't currently) but the defending pokemon doesn't knock back or flash at all (unless the defender was resistant then flash red a little bit).</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>25/10: play_attack_hit(attacker, defender, damage, weak, resisted). Weak: knock-back + wiggle x2, green-tinted flash. Resisted: x0.5, red-tinted flash. Damage cut to 0: lunge still plays (call site now fires when the attack had printed damage), defender doesn't move/flash, except a faint red flash if Resistance did it. Consts HIT_FLASH_WEAK/RESIST/ZERO_RESIST, HIT_WEAK_MULT, HIT_RESIST_MULT.</t>
+        </is>
+      </c>
+      <c r="G475" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="476" ht="60" customHeight="1">
+      <c r="A476" s="5" t="n">
+        <v>474</v>
+      </c>
+      <c r="B476" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C476" s="5" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D476" s="6" t="inlineStr">
+        <is>
+          <t>For the new attack animation, for any attack whether it does damage or not, when the message pops up that says the pokemon is using the attack, have the pokemon shake left and right 3 times fast. 
+if the attack being made is a no damaging move (it has 0 attack power before any calculation so it only has an effect nad not actual damage, instead of having the attacking card angle and move towards the opponents card, instead have a very very simple effect parser: If the attack tries to inflict something on the opponent e.g a status condition, or blindness, or prevents retreat or anything like that, if the effect specifically is meant to do something to the oppoennt's active pokemon, then play animation 1: 
+1) the attacking card slowly moves side to side with speed ramping. After 0.5 seconds, the defending card does the same motion animation (moving left to right). 
+If the attacking card's effect specifically only does something to the attacking card, e.g harden to prevent damage to itself, swords dance to power up next attack, energy absorption to attach energies, etc etc, if it only affects the attacking card then instead play animation 2:
+2) The attacking card hops up and down on the spot 3 times, then shakes left to right quickly twice
+If the attacking pokemon is doing a bench damaging move or any move that moves damage counters, or applies damage counters to an opponent, or places them on the bench, but doesn't actually do damage to the defending pokemon as part of the actual damage calculation play animation 3:
+3) After the shake left and right, the attack pauses for a short fraction of a second, then hops up on the spot once.
+4) If a pokemon power is activated at any point, have that pokemon shake fast 4-5 times a small amount left to right
+5) If an attack effect doens't auto route through one of these animations, then instead have hte pokemon teeter left and right a few times (angle left right)</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>25/10: Card_FX: every attack declaration (player + CPU) shakes the attacker 3x fast while 'X used Y' shows. A 0-printed-damage attack then plays a gesture instead of the lunge, from a simple text read (Card_FX.classify_attack): damage counters / bench -&gt; pause + one hop (3); Defending Pokemon / status / can't retreat etc. -&gt; attacker sways, defender joins 0.5s later (1); self-only (this Pokemon / attach / heal / own name) -&gt; 3 hops + 2 quick shakes (2); anything else -&gt; teeter (5). Pokemon Power use (player activate_power, CPU announce_cpu_power) -&gt; small fast shake x5 (4).</t>
+        </is>
+      </c>
+      <c r="G476" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>Live: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="477" ht="285" customHeight="1">
+      <c r="A477" s="5" t="n">
+        <v>475</v>
+      </c>
+      <c r="B477" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C477" s="5" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D477" s="6" t="inlineStr">
+        <is>
+          <t>During the intiial tutorial, it currently says press Caps lock to open help messages right at the beginning, but instead move that to a few lines in so it's not the first thing. Have it first say that after saying press your hand to see cards, then immediately after say press caps lock to see the messages again. also have it say it again later on, when you draw ponyta, have a message then again saying "remember you can press caps lock to see the match log and all messages". Have another message directly after pluspower is played with the shift key hint we have already int he second match tutorial, have it say you can press shift to see a card's details.
+For the secondary tutorial, we can remove the first caps lock message all together as it's basically repeated on turn 2 or 3. The press shift to see a card in detail is played first when the first card is drawn and then the second press caps lock message isn't played until after that. on the next avaialble turn with no message to play</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>25/10: Newby: Caps Lock hint removed from the opening screen and played straight after 'Click your hand...'; after Professor Oak (Ponyta drawn) 'Remember you can press [CAPS LOCK] to see the match log and all messages.'; after PlusPower 'You can press [SHIFT] to see a card's details.'. Second match: no opening Caps Lock line; Shift tip on the first turn, Caps Lock on the next turn nothing else is said (FOLLOWUP_TIP_ORDER). See #485.</t>
+        </is>
+      </c>
+      <c r="G477" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="478" ht="135" customHeight="1">
+      <c r="A478" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="B478" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C478" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D478" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">During the tutorial starts when speaking to Olly, at the point where he says "you can't have more than 60 cards in your deck put the rest in your binder. As soon as that message pops up, open the escape key (with the message still on screen), have the glowing gradeint selection we use throughout the game glowing around the cards &amp; deck button with everything else darkened and greyed out, pause on this highlighted deck &amp; card menu escape screen for about 2 seconds, have the cards &amp; deck icon grown and shrink for this 2 seconds as if it's been highlighted but ALSO with the glowing gradient swirling around it, then transition to inside the deck builder screen showing empty slots where the cards should be. Blocking player input, have the viewer scroll down visible in this mode and stop scrolling such that the now top visible row is the first row with an actual pokemon card that should be in it. E.g for the first newby start, the top row should be the one that dugtrio should be on, then have all the players now owned cards (such as 2 dugtrio, 2 machoke, 1 ivysaur, 1 kadabra etc (different cards for different starts) fade in and float down into their slots, if there are 2 cards do the second one the same with a slight delay so they both go simultaneously but start and end the animation off sync, then update the X/X as they fly in and land in their resting place.
+Then Have a message pop up here when the last one is cleared to a system message of "You can look at your owned cards, edit your deck, remove any cards in it and add any new cards on this screen". Close the whole thing when the mesage is cleared. Don't allow the message to be cleared until this screen is viewed for like 2 seconds (2 seconds on menu, 2 seconds on deck build screen).  
+Have the flashing down arrow on a message vanish when it can't be cleared and appear when it can be cleared. 
+After that, Then, find the "Better Deck" in the save slot 1 that is there now, and over the course of about 5 seconds have all the cards visibly minus and add to convert the player's currently set "Your first deck" to the "better deck". Better deck is the "Your first Deck" as a base with some poorer cards taken out such as ponyta and the better new cards added in such as raticate dugtrio and starmie. Therefore the cards added and minus should be such so that e.g the new dugtrio and farfetchd are added 1 card at a time so you can see the numbers go up, then the fire energies go down and the other energies go up. While all this is happening have a message dialogue from Olly that says "With those cards you got in your bonus pack, I would have a deck that looks a little more like this.","It'll have a much stronger selection of cards and you should be able to do a lot better with it!","Don't forget to tweak your deck to your own liking, don't just take my advice!!". For the water fight, grass psy or fire shock starter decks, do the same thing when the additional pack is granted it should have all the additional cards needed to turn the deck from the "Starter" deck version into the deck version that doesn't have "Starter" in it's name. If it's missing some cards in the pack to be able to "upgrade" the starter deck to the non starter version, then instead grant all those missing cards to the player so they have them all, then do the same deck manipulation on screen to show the cards being changed in the deck. 
+When the deck editiing is done, update the name fo the deck from "Your First Deck" to "Better Deck" and when the last message is cleared (or when the deck manipulation animation is finished), "click" the save button so the Deck Saved label appears, but the player can still access Your First Deck if they want to go back to the easier deck. then finally have one last message pop up that says "it's a good idea to write down all your different deck ideas so you can quickly switch from one deck to another. You can go back to using your first deck if you want by pressing Load Deck." Then have the overworld return and the conversation continue
+Then when the coin case is mentioned and it says put the coin in, do the same thing, have the escape menu open, highlight the coin case with everything else darkened out, open the coin case, have the two coins fade and fly in as if from the player's eyes so start large, fade in, then shrink fast into place as if being placed down into the case. </t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>25/10: NOT STARTED -- big enough to need its own session (deck builder 4,300 lines + main menu + coin case + intro cutscene) and some answers first; see the session summary. Left as New Functionality.
+25/10 (2): BUILT. Olly_Intro_Cutscene._deck_walkthrough (newby 'basic' + 'rules' paths): the '60 cards' line stays up (DynamicMessageBox.hold_advance -- can't be cleared, no caret) while the escape menu opens itself with Cards &amp; Deck in the gradient selection ring, pulsing, the other tiles dimmed; after 2s the deck builder opens on its own (Deck_Build walkthrough API, input blocked): the bonus pack's cards start as empty slots, it scrolls to the first row holding one, each copy fades in and floats into its slot (pairs off-sync) and the X / X count ticks up. The line can be cleared once the builder has been up 2s, then the system line 'You can look at your owned cards...'. Then the deck is rebuilt card by card over ~5s (new cards in, cut cards out, Energy down then up) while Olly says his 3 lines; any card the target deck needs that isn't owned is granted first. Target: newby Basic Starter Deck -&gt; 'Better Deck' (your slot-1 deck, shipped as Player_Data/Starter_Decks/Better Deck.json); rules: '&lt;pair&gt; Starter Deck' -&gt; '&lt;pair&gt; Deck'. Deck renamed, Save 'pressed' (pops), DECK SAVED!, old deck kept for Load Deck, final 'write down your deck ideas' line, menu closes, conversation continues ('put them in your binder' line dropped). Coin case: 'Put the coin I just gave you in there' held while the menu opens on the coin case tile, the case opens and each owned coin appears large and faint, fades in and drops into its slot. Runs once (olly_intro_walkthrough_done keys). Olly's own gifted bonus pack now also glides into the pack opening (#487 handoff). Headless-tested both paths on a throwaway slot: saved Fire Shock Deck == shipped deck (60), set active, starter deck kept.</t>
+        </is>
+      </c>
+      <c r="G478" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>Live: 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="479" ht="409.5" customHeight="1">
+      <c r="A479" s="5" t="n">
+        <v>477</v>
+      </c>
+      <c r="B479" s="5" t="inlineStr">
+        <is>
+          <t>Overworld</t>
+        </is>
+      </c>
+      <c r="C479" s="5" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D479" s="6" t="inlineStr">
+        <is>
+          <t>Flying pokemon have a hard limit at the left side of the screen but the world got expanded so now pokemon fly and vanish in front of the player if they're in the left part of the map. Extend the flying pokemon to be the new edges of all the maps we have them in</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>25/10: Flyers read camera.limit_left/right as the map edge, but outdoor cameras have limits DISABLED and the scene still held old numbers (-1000..6500), so flocks despawned mid-screen on the expanded west side. Overworld_Pokemon_Spawner._map_edge now only trusts enabled limits; otherwise measures the union of the map's TileMapLayer used rects (_map_bounds, cached per map). Covers every map with flyers.</t>
+        </is>
+      </c>
+      <c r="G479" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="480" ht="30" customHeight="1">
+      <c r="A480" s="5" t="n">
+        <v>478</v>
+      </c>
+      <c r="B480" s="5" t="inlineStr">
+        <is>
+          <t>Overworld</t>
+        </is>
+      </c>
+      <c r="C480" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D480" s="6" t="inlineStr">
+        <is>
+          <t>when ellie calls the player on day 2, quadruple the amount of steps/distance into the living room they have to get</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>25/10: Player_House_Downstairs: CAFE_CALL_TRIGGER_DISTANCE 32 -&gt; 128 (x4), and now measured as distance actually walked (summed per frame) instead of straight-line displacement, so a small room can't stop it ringing.</t>
+        </is>
+      </c>
+      <c r="G480" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="5" t="n">
+        <v>479</v>
+      </c>
+      <c r="B481" s="5" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="C481" s="5" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D481" s="6" t="inlineStr">
+        <is>
+          <t>For some reason the olly second match at the café his colour is pink in game not blue</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>25/10: Could not reproduce from the data -- Olly 2 is 'aqua' in All_NPC_Constant_Data.json exactly like Olly, the cafe speaker reads that, the match message box uses the theme accent, the outro uses message_colour, and the phone map story blip matches 'Olly 2' to light blue. Need to know WHERE it is pink (match box / outro box / name pill / map dot / sprite) -- left as New Issue.
+25/10 (2): ROOT CAUSE: the Caps Lock match log was configured with the in-match message box's theme key (the UI accent -- pink in your theme), not the opponent's message_colour, so every opponent's pill/dividers/stripes were pink. Now uses opponent_data message_colour (Olly = aqua), falling back to the accent if unset.</t>
+        </is>
+      </c>
+      <c r="G481" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="5" t="n">
+        <v>480</v>
+      </c>
+      <c r="B482" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C482" s="5" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="D482" s="6" t="inlineStr">
+        <is>
+          <t>Instead of "HELP" in the message log when caps lock is pressed have "TUTORIAL"</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>25/10: Match_Log_Panel tutorial row tag 'HELP' -&gt; 'TUTORIAL'.</t>
+        </is>
+      </c>
+      <c r="G482" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="5" t="n">
+        <v>481</v>
+      </c>
+      <c r="B483" s="5" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C483" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D483" s="6" t="inlineStr">
+        <is>
+          <t>When maintenance is played, the cards aren't shown going into the deck and having the deck shuffled. Play this animation ebfore the card is drawn</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>25/10: Player Maintenance now flies each chosen card from the hand into the deck, plays the deck shuffle, then draws (same as the CPU's ISSUE #41 flow).</t>
+        </is>
+      </c>
+      <c r="G483" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="484" ht="30" customHeight="1">
+      <c r="A484" s="5" t="n">
+        <v>482</v>
+      </c>
+      <c r="B484" s="5" t="inlineStr">
+        <is>
+          <t>Tutorial</t>
+        </is>
+      </c>
+      <c r="C484" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D484" s="6" t="inlineStr">
+        <is>
+          <t>When Olly says to the player to meet them at the café or el calls to say meet them at the café and to hurry up. Whoever tells the player to go, have a line before hand saying "Before you get here, call in at the Card Mart and get yourself some new pack!","Make sure your deck is the best it can be and we can battle when you get here!"</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>25/10: Ellie's call (Phone_Calls.json cafe_call_ellie) gets 'Before you get here, call in at the Card Mart and get yourself some new packs!' + 'Make sure your deck is the best it can be and we can battle when you get here!' before her 'come meet us' line. Olly ('played' route, LINES_CAFE_MORNING) says the same before 'El told me to tell you...', reworded to 'get there' / 'they'll want to battle' as he isn't at the cafe himself.</t>
+        </is>
+      </c>
+      <c r="G484" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="485" ht="45" customHeight="1">
+      <c r="A485" s="5" t="n">
+        <v>483</v>
+      </c>
+      <c r="B485" s="5" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C485" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="D485" s="6" t="inlineStr">
+        <is>
+          <t>When the opponent used energy retrieval there was no animation showing the discard to the discard pile and adding of the cards to the hand.</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>25/10: CPU Energy Retrieval: the discarded card flies hand -&gt; discard (face up), then each retrieved Energy flies discard -&gt; hand (face up, it's public), discard pile redrawn between. Player version also animates its discarded card now.</t>
+        </is>
+      </c>
+      <c r="G485" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="486" ht="30" customHeight="1">
+      <c r="A486" s="5" t="n">
+        <v>484</v>
+      </c>
+      <c r="B486" s="5" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C486" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D486" s="6" t="inlineStr">
+        <is>
+          <t>For the café matches specifically with Olly Ellie and Alexander, have Olly play with Never retreating a pokemon. This should make him slightly easier and weaker to battle against. Have Ellie retreat at about a half of the time that she would normally, and have Alexander set to normal retreating</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>25/10: New opponent field cpu_retreat_rate (0.0-1.0, default 1.0) -&gt; CpuWeights.retreat_rate, checked in CPU_AI.execute_cpu_retreat (every voluntary retreat; Switch and forced replacements unaffected). Olly 2 = 0.0 (never retreats), Ellie 3 = 0.5, Alexander 3 unchanged. All_NPC_Constant_Data.json.</t>
+        </is>
+      </c>
+      <c r="G486" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="487" ht="45" customHeight="1">
+      <c r="A487" s="5" t="n">
+        <v>485</v>
+      </c>
+      <c r="B487" s="5" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C487" s="5" t="inlineStr">
+        <is>
+          <t>tutorial</t>
+        </is>
+      </c>
+      <c r="D487" s="6" t="inlineStr">
+        <is>
+          <t>Make sure tutorial messages are kept on for the newby after their first tutorial match so their second match has the generic tutorial messages on as a reminder</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>25/10: The newby's second match (GameState.TUTORIAL_TIPS_KEY) now runs the full GENERIC tutorial (click-hand, at-risk, evolution, pile messages, board labels, turn tips) instead of the key-tips-only 'tips' mode, which is removed. Cleared at match end as before. Option row locked On meanwhile (#470).</t>
+        </is>
+      </c>
+      <c r="G487" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="488" ht="30" customHeight="1">
+      <c r="A488" s="5" t="n">
+        <v>486</v>
+      </c>
+      <c r="B488" s="5" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C488" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D488" s="6" t="inlineStr">
+        <is>
+          <t>When a pokemon is knocked out (either active pokemon or bench) calculate if it is knocked out IMMEDIATELY as the damage is dealt. If the pokemon is knocked out, have them fade to about 25% blackness over 2 seconds so a knocked out pokemon turns black slowishly while the damage is being dealt), after the knockback immediately have it move slowly side to side as if poisoned. When the kncoked out message is cleared then have it unfade from black as it's moving to the discard pile</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>25/10: Card_FX.start_ko: the moment damage leaves a Pokemon on 0 HP (main attack path; check_all_knockouts catches bench/poison/Curse KOs) it darkens to 75% (KO_DARK) over 2s and sways slowly like poison; after 'X WAS KNOCKED OUT!' is cleared it lightens back over 0.5s as it goes to the discard. Survivors (Focus Band etc.) reset at the end of check_all_knockouts.</t>
+        </is>
+      </c>
+      <c r="G488" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="489" ht="60" customHeight="1">
+      <c r="A489" s="5" t="n">
+        <v>487</v>
+      </c>
+      <c r="B489" s="5" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C489" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D489" s="6" t="inlineStr">
+        <is>
+          <t>when a pack of cards is gifted, the pack gift pops up like "You have received X", then the pack vanishes and the opening pack scene kicks in to open it. Instead, the opening pack scene should flow fluidly so the same pack that is shown at the gift screen is the same pack that is opened and the cards come out of without flashing or changing scenes</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>25/10: Match outro: after 'You received a pack' the SAME pack glides (position+size) into PackOpeningManager.get_pack_target_rect() and the opening starts with no fade-in; the reveal is hidden only once the opening's pack is drawn. Same handoff added to MapManager's overworld gift-a-pack path (NPC gifts / free packs) when one pack is shown.</t>
+        </is>
+      </c>
+      <c r="G489" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="490" ht="45" customHeight="1">
+      <c r="A490" s="5" t="n">
+        <v>488</v>
+      </c>
+      <c r="B490" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C490" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D490" s="6" t="inlineStr">
+        <is>
+          <t>When olly is beaten at the café and starts to walk off, when he gets about half way to moving off screen, have ellie face downwards, pause for a second, then while olly is still walking off, pop up a message from ellie saying "Sigh… Don’t worry then I'll pay..." then face the player again, then when Olly is offscreen, or pause a half second, then have Ellie's dialogue continue</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>25/10: Cafe: Olly's walk-off is no longer awaited; at ELLIE_SIGH_AT (50%) of the way off screen Ellie looks down, pauses ELLIE_LOOK_BACK (1s), says 'Sigh... Don't worry then I'll pay...' while he's still walking, turns back; her own lines wait until he's off screen + ELLIE_SIGH_AFTER (0.5s).</t>
+        </is>
+      </c>
+      <c r="G490" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="491" ht="45" customHeight="1">
+      <c r="A491" s="5" t="n">
+        <v>489</v>
+      </c>
+      <c r="B491" s="5" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C491" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D491" s="6" t="inlineStr">
+        <is>
+          <t>So this is a very specific combo but if Pokedex is used by the opponent then they should know how good the cards are coming up and if they have a second trainer in their hand with drawing or shuffling they can play accordingly. E.g they use pokedex and see just 5 energies straight coming, They already have plenty in hand so they use maintenance to shuffle. E.g2: they use pokedex and see they are getting a bill bill energy energy energy. They have plenty of energy but the bills are good value. They don't shuffle their deck using the trainer effect, instead drawing bill first. they then use bill to get bill 2 then shuffle the deck becasue they have plenty of energies. They can also gauge value of discard for professor oak using pokedex this way. E.g I have a charizard in my hand I don't want to discard but If I use professor oak I get charizard on my next draw so I can afford to discard the one in hand</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>25/10: CPU_AI remembers its Pokedex / New Pokedex result (cpu_known_top: card refs, dropped as drawn, forgotten on any shuffle). cpu_known_draw_delta(n) compares the known next draws against an average card (Pokedex priority scale). Maintenance (+Bill's Maintenance family) scores higher when the known top is poor, lower when good (draw into the Bill first). Professor Oak (+Oak's Research) +/- by the known top 7, and a card in hand stops blocking Oak if the same card is coming in those 7. New Pokedex now also sorts its top cards like Pokedex.</t>
+        </is>
+      </c>
+      <c r="G491" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>Live: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="492" ht="105" customHeight="1">
+      <c r="A492" s="5" t="n">
+        <v>490</v>
+      </c>
+      <c r="B492" s="5" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C492" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D492" s="6" t="inlineStr">
+        <is>
+          <t>when potion is played and it's seen discard to the discard pile, only show the recovery as it's moving to discard pile and make sure the green squares are added in sequence not at once immediately.</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>25/10: CPU Potion / Super Potion heal now plays WHILE the card flies to the discard (flight started, not awaited; play_trainer_card waits for it after). card_ops.heal_pokemon redrew the ACTIVE's HP row each step, so a benched Pokemon's green blocks came back all at once at the end -- now refresh_pokemon_hp_display per block, HEAL_BLOCK_STEP 0.25s; '+N HP' label centred via float_label_over. Covers every heal effect that uses heal_pokemon.</t>
+        </is>
+      </c>
+      <c r="G492" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="493" ht="30" customHeight="1">
+      <c r="A493" s="5" t="n">
+        <v>491</v>
+      </c>
+      <c r="B493" s="5" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C493" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D493" s="6" t="inlineStr">
+        <is>
+          <t>Opponent retreated doduo with a fightning weakness against a machoke with 40/80hp remaining and only one fighting energy. They swapped in for a pikachu? Not only was doduo resistance, had 30hp left so couldn't even be knocked out if machoke could attack, machoke couldn't attack, and pikachu has a fighting weakness. this makes no sense</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>25/10: CPU_AI._offensive_retreat_target skips a Benched Pokemon with a worse Weakness/Resistance matchup vs the Defending Pokemon (Weak where the Active isn't, or the Active Resists and it doesn't) unless it KOs straight away (_type_matchup_worse). Doduo (Resists Fighting) no longer swaps for Pikachu (Weak to Fighting).</t>
+        </is>
+      </c>
+      <c r="G493" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="494" ht="45" customHeight="1">
+      <c r="A494" s="5" t="n">
+        <v>492</v>
+      </c>
+      <c r="B494" s="5" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C494" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D494" s="6" t="inlineStr">
+        <is>
+          <t>The CPU THEN THE NEXT TURN PLAYED SWITCH TO SWAP PIKACHU WITH RATTATA THEN RETREATED RATTATA FOR PIKACHU!!! NONSENSE</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>25/10: One change of Active per turn: _turn_start_active recorded at the start of the CPU turn; both retreat passes refuse once the Active already changed (Switch etc.), and _cpu_score_switch returns 0 after a retreat/switch. Switch also now needs the same 'swap gains something' test the retreat uses (survival / offensive / idle Active / guaranteed KO), on a fresh evaluation.</t>
+        </is>
+      </c>
+      <c r="G494" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>Live: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="B495" s="5" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C495" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D495" s="6" t="inlineStr">
+        <is>
+          <t>Omg then I thought the CPU was going to win, it pulled a pro move, Gust of winded a diglett with pikachu as their active, removed diglett for staryu. THEN RETREATED PIKACHU FOR DODUO, THEY HAD A GUARENTEED WIN IF PIKACHU USED THUNDERJOLT WHICH IT COULD</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>25/10: ROOT CAUSE: cpu_eval was built at Phase 4, then Phase 4b played Gust of Wind/Switch, and the Phase 5 retreat used that stale snapshot (it still thought Pikachu faced the Gusted-away Diglett). The evaluation is now rebuilt right before the retreat pass.</t>
+        </is>
+      </c>
+      <c r="G495" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="496" ht="30" customHeight="1">
+      <c r="A496" s="5" t="n">
+        <v>494</v>
+      </c>
+      <c r="B496" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C496" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D496" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When alexander says "Are you ready to lose now" or the player returns for his match, have Alexander look down and the player look up </t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>25/10: _ask_alex turns Alexander to face down and the player up before 'Are you ready to lose now?' (also when the player comes back for his match).</t>
+        </is>
+      </c>
+      <c r="G496" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="5" t="n">
+        <v>495</v>
+      </c>
+      <c r="B497" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C497" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D497" s="6" t="inlineStr">
+        <is>
+          <t>Increase the time delay between the end turn and start turn labels. Maybe have the start turn just after the card is drawn if more time is required</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>25/10: New main.turn_label_gap(): TURN_LABEL_GAP 0.9s (x animation speed) before each side's 'Start turn' label (player_start_turn_checks and CPU opponent_start_turn_checks).</t>
+        </is>
+      </c>
+      <c r="G497" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="498" ht="30" customHeight="1">
+      <c r="A498" s="5" t="n">
+        <v>496</v>
+      </c>
+      <c r="B498" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C498" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D498" s="6" t="inlineStr">
+        <is>
+          <t>Make the animation speeds for SLOW 10% slower. For medium set it 10% faster. For fast set it to 10% faster</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>25/10: MATCH_SPEED_PRESETS / ITEM_SPEED_PRESETS: slow 1.0 -&gt; 0.9, medium 1.25 -&gt; 1.375, fast 2.2 -&gt; 2.42. Pack-opening presets left as they were.</t>
+        </is>
+      </c>
+      <c r="G498" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="5" t="n">
+        <v>497</v>
+      </c>
+      <c r="B499" s="5" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C499" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D499" s="6" t="inlineStr">
+        <is>
+          <t>opponent is far too reatreat heavy. Farfetched 20hp posioned vs weedle 10hp. Opponent retreats 10hp weedle for rattata with 10hp. Rattata has the guarenteed knockout but so did weedle without discarding an energy for the same hp with the poison damage guaranteed at the end of the turn. Should have kept in low damage weedle without discarding to knockout</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>25/10: 'Already Knocks Out' now counts the player's certain Poison/Burn tick at the end of this turn (_player_active_hp_to_ko): used by _cpu_active_can_ko_player_active, _cpu_bench_ko_retreat_target and _offensive_retreat_target. Weedle's 10 + poison on a 20 HP Farfetch'd = KO, so no retreat into Rattata.</t>
+        </is>
+      </c>
+      <c r="G499" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="500" ht="45" customHeight="1">
+      <c r="A500" s="5" t="n">
+        <v>498</v>
+      </c>
+      <c r="B500" s="5" t="inlineStr">
+        <is>
+          <t>Cutscene</t>
+        </is>
+      </c>
+      <c r="C500" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D500" s="6" t="inlineStr">
+        <is>
+          <t>when ellie and alexander go to the shop to get more cards, the cutscene ends and it fades to black. It shouldn't have a cut, a fade or a scene reload at all. If a scene reload is required for them to be shown in the card mart on the map just have them already there as soon as the battle with alexander ends. All cutscenes should be smooth and transitionless where possible. The black fade in and out for the cafe was only so avoid having the player having to try and get off and on a chair</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>25/10: Cafe closing scene has no fade or reload now: Ellie walks out to the aisle and up to the cafe door, fades through it (0.3s), waits 1.5s and comes back out; Alexander and the player walk down from the table to their spots meanwhile. At the end the map is NOT reloaded -- the clock already moved to Afternoon on the way back from Alexander's match (settle_after_load), so the Card Mart duo is already in place; the cutscene just finishes. ALEX_STAND_X / PLAYER_STEP_DOWN_Y / ELLIE_DOOR_FADE / ELLIE_INSIDE_TIME tweakable.</t>
+        </is>
+      </c>
+      <c r="G500" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="501" ht="60" customHeight="1">
+      <c r="A501" s="5" t="n">
+        <v>499</v>
+      </c>
+      <c r="B501" s="5" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C501" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D501" s="6" t="inlineStr">
+        <is>
+          <t>Opponent used recycle as it's first move, picking recyle to put back on top of the deck. Recyle should only be played for good well scored cards. When considering playing recycle, consider the scoring of every card it can pick to play such that if it finds a card like bill or prof oak which would be really good in this instance now so would get a good score in the hand, then play it for that</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>25/10: Recycle scored on the best card it could actually fetch (cpu_rank_keep_value over the discard, never another Recycle) minus RECYCLE_KEEP_FLOOR 40 (only worth it for a 70+ keep card: Bill/Oak when good, an Evolution with its base out...). The CPU's pick inside Recycle uses the same keep value and never takes a Recycle.</t>
+        </is>
+      </c>
+      <c r="G501" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="502" ht="45" customHeight="1">
+      <c r="A502" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="B502" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C502" s="5" t="inlineStr">
+        <is>
+          <t>New Functionality</t>
+        </is>
+      </c>
+      <c r="D502" s="6" t="inlineStr">
+        <is>
+          <t>when damage curse gengar is played, have the hp minus and plus and have the message say who the damage is moving from and to. Also the logic on this was incorrect, dugtrio used earthquake hurting 5 bench pokemon. Gengar then moved one single counter to dugtrio from 70hp to 60hp. He could have brought dugtrio down to 20hp</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>25/10: New shared move_damage_counter_animated (Powers): green '+10' on the source, red '-10' on the target, each HP row redrawn in its own slot, 0.35s apart. Player Curse message 'MOVED A DAMAGE COUNTER FROM X TO Y'; CPU 'CURSE: A DAMAGE COUNTER MOVES FROM X TO Y!'. NOTE on the logic: Curse's card text is 'Once during your turn ... move 1 damage counter', so one counter per Gengar per turn is correct -- it can't take Dugtrio 70 -&gt; 20 in one turn. See #503 for the target choice.</t>
+        </is>
+      </c>
+      <c r="G502" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="503" ht="45" customHeight="1">
+      <c r="A503" s="5" t="n">
+        <v>501</v>
+      </c>
+      <c r="B503" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C503" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D503" s="6" t="inlineStr">
+        <is>
+          <t>floating labels for bench damage are way off to the right a few hundred pixels. The label should be directly in the center of the pokemon card the HP is being removed from</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>25/10: show_floating_label centres its text in a 300px box placed at the given point, and bench damage passed the card's CENTRE as that box's left edge -&gt; ~150px right. card_ops.apply_bench_damage + the two Attack_Effects copies now use float_label_over, which for a benched Pokemon centres dead on the card (no outward nudge, measured off the real node). Poison/burn tick labels (hardcoded 530/1030) also moved onto the card.</t>
+        </is>
+      </c>
+      <c r="G503" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="504" ht="30" customHeight="1">
+      <c r="A504" s="5" t="n">
+        <v>502</v>
+      </c>
+      <c r="B504" s="5" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C504" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D504" s="6" t="inlineStr">
+        <is>
+          <t>On the next turn, gengar used damage curse to move one counter to rattata and kncok it out. This is a good idea great. But then the hp for rattata was shown as dugtrios so the active pokemon dugtrio had 0/30hp with the message rattata being knocked out</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>25/10: ROOT CAUSE: display_hp_circles_above_align() only draws the ACTIVE slot's HP row; Curse (and ~40 other power call sites) passed it a BENCHED Pokemon, so Rattata's 0/30 was painted over Dugtrio. The function now redirects any benched Pokemon to a redraw of its own bench slot -- fixes every caller at once.</t>
+        </is>
+      </c>
+      <c r="G504" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="505" ht="30" customHeight="1">
+      <c r="A505" s="5" t="n">
+        <v>503</v>
+      </c>
+      <c r="B505" s="5" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C505" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D505" s="6" t="inlineStr">
+        <is>
+          <t>Gengar then on the next turn moved one counter BACK to dugtrio. There were 4 bench pokemon all with 20 damage done (2 counters). 2 of those had 2ho left. Gengar could have won moving 4 counters from the higher HP mons to the near knockout mons and won the match entirely but instead did 1 counter to dugtrio. Are powers only considered once? it should be constantly reevaluated. It appears damage swap is conisdered a single time then used with no foresight into total damage spread or multiple uses. It then used dark mind to do 10 damage to the highest HP bench pokemon instead of the one that had 20hp left</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>25/10: CPU Curse rewritten as cpu_ai.cpu_pick_curse_move(): KO (ex first) &gt; bring the Defending Pokemon into this turn's attack range &gt; leave a Pokemon on 10 HP (one counter from a KO) &gt; chip; the counter comes off the Pokemon furthest from a KO, never off one this turn's attack is about to KO. Every Gengar with Curse now gets its go (the old code only checked the first). Re-evaluated on each of the 3 power passes per turn. Dark Mind / every bench snipe (cpu_rank_snipe_target) now strongly prefers leaving a Pokemon on 10-20 HP over chipping a healthy one. Curse is once per turn by card text, so 4 counters in one turn isn't legal.</t>
+        </is>
+      </c>
+      <c r="G505" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="506" ht="75" customHeight="1">
+      <c r="A506" s="5" t="n">
+        <v>504</v>
+      </c>
+      <c r="B506" s="5" t="inlineStr">
+        <is>
+          <t>Overworld</t>
+        </is>
+      </c>
+      <c r="C506" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D506" s="6" t="inlineStr">
+        <is>
+          <t>Player returned from battle into overworld, both player and opponent faced downwards. Oppoennt didn't return to correct position facing</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>25/10: Neither battle start saved the player's facing, so the battle return reused whatever a door last saved ('down'). Both MapManager battle starts now save it, and on return the opponent just fought is turned to face the player (_face_battled_opponent) whichever way its node was respawned.</t>
+        </is>
+      </c>
+      <c r="G506" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="5" t="n">
+        <v>505</v>
+      </c>
+      <c r="B507" s="5" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C507" s="5" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D507" s="6" t="inlineStr">
+        <is>
+          <t>The little icon that pops down to say the time of day should last at least twice as long. Multiply it's fly in and stay length by 2.5x</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>25/10: Time_Of_Day_Banner IN_TIME 0.35 -&gt; 0.875, HOLD_TIME 1.0 -&gt; 2.5 (x2.5).</t>
+        </is>
+      </c>
+      <c r="G507" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="5" t="n">
+        <v>506</v>
+      </c>
+      <c r="B508" s="5" t="inlineStr">
+        <is>
+          <t>Overworld</t>
+        </is>
+      </c>
+      <c r="C508" s="5" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D508" s="6" t="inlineStr">
+        <is>
+          <t>Decrease overworld darkness at normal night time by 10%, increase overoworld darkness during bedtime/midnight by 10%</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>25/10: Time_Of_Day_Grade BRIGHTNESS Night 0.85 -&gt; 0.935 (10% lighter), Bedtime 0.51 -&gt; 0.459 (10% darker).</t>
+        </is>
+      </c>
+      <c r="G508" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="5" t="n">
+        <v>507</v>
+      </c>
+      <c r="B509" s="5" t="inlineStr">
+        <is>
+          <t>Overworld</t>
+        </is>
+      </c>
+      <c r="C509" s="5" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D509" s="6" t="inlineStr">
+        <is>
+          <t>For midnight (bedtime) specifically, when the overworld is loaded, have the screen fade to black and back in and remove that last opponent the player battled so that they can't rematch the opponent during bedtime/midnight again. As soon as the game reloads, show teh opponent initially but don't give player control back until a quick fade in and out to remove it</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>25/10: MapManager._bedtime_dismiss_battled_opponent: back from a battle at Bedtime, the opponent shows, the player is locked, after 0.8s (and any message) a 0.35s fade to black, the opponent is removed, fade back in, control returned. Nobody is scheduled at Bedtime, so they don't come back.</t>
+        </is>
+      </c>
+      <c r="G509" s="6" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="510" ht="45" customHeight="1">
+      <c r="A510" s="5" t="n"/>
+      <c r="B510" s="5" t="n"/>
+      <c r="C510" s="5" t="n"/>
+      <c r="D510" s="6" t="n"/>
+      <c r="G510" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I79"/>
-  <conditionalFormatting sqref="A2:J999">
+  <conditionalFormatting sqref="A2:J998">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>OR($G2="New Issue",$G2="Fix Failed",$G2="Improve Further",$G2="New Functionality")</formula>
     </cfRule>

</xml_diff>